<commit_message>
Add SpiNNcloud €3.36m public contract evidence
Add Jülich procurement T026 and Weipan seed+ T027; separate contract value, financing, payment and revenue. Refresh mobile report and workbook.
</commit_message>
<xml_diff>
--- a/market-evidence.xlsx
+++ b/market-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="R82b2c42a795d46af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="Ra36de53ffb264993"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="Ra069db5490d6464e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="R089df5496a3f4027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="R472c4ec51b854594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="R653226e7071d4609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="Rd7e929da9548438e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="Rec52a6984a9843a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Noto Sans SC"/>
     </x:font>
   </x:fonts>
-  <x:fills count="18">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -156,6 +156,26 @@
         <x:fgColor rgb="FF23445C"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="9">
     <x:border/>
@@ -191,7 +211,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="129">
+  <x:cellXfs count="161">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -510,6 +530,98 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="6" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1054,7 +1166,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6d705e5d5e2546c6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40f48f2df1f5462e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1084,7 +1196,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1267d2b960ce494e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b34b835bb26468b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1114,7 +1226,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5adf2ecf229e4ff9"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83eacf13a578408d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1124,7 +1236,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="29" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1141,7 +1253,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="30" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1159,7 +1271,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="35" name="EventEvidence" displayName="EventEvidence" ref="A1:G26" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="事件日期"/>
@@ -1174,7 +1286,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="36" name="TactileResearch" displayName="TactileResearch" ref="A44:I50" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A47:I53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="研究编号"/>
     <x:tableColumn id="2" name="研究主体"/>
@@ -1437,7 +1549,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-02在线学习复核。37个主体、39组产品、25项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
+        <x:v>2026-10-02商业化证据复核。37个主体、39组产品、27项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1635,7 +1747,7 @@
         <x:v>方案／研发</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A13)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A13)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
@@ -1657,7 +1769,7 @@
         <x:v>研究／原型</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A14)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A14)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
@@ -1679,7 +1791,7 @@
         <x:v>工程样片</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A15)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A15)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
@@ -1701,7 +1813,7 @@
         <x:v>IP／商务接洽</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A16)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A16)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
@@ -1723,7 +1835,7 @@
         <x:v>开发平台</x:v>
       </x:c>
       <x:c r="B17" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A17)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A17)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
@@ -1745,7 +1857,7 @@
         <x:v>客户评估／模块</x:v>
       </x:c>
       <x:c r="B18" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A18)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A18)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
@@ -1767,7 +1879,7 @@
         <x:v>可采购硬件</x:v>
       </x:c>
       <x:c r="B19" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A19)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A19)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="2"/>
@@ -1789,7 +1901,7 @@
         <x:v>商品页／售罄</x:v>
       </x:c>
       <x:c r="B20" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A20)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A20)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C20" s="2"/>
@@ -1811,7 +1923,7 @@
         <x:v>生产／部署声明</x:v>
       </x:c>
       <x:c r="B21" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A21)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A21)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C21" s="2"/>
@@ -1833,7 +1945,7 @@
         <x:v>发布／演示</x:v>
       </x:c>
       <x:c r="B22" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A22)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A22)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
@@ -1852,10 +1964,10 @@
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="2" t="str">
-        <x:v>科研部署已确认</x:v>
+        <x:v>已签公共采购合同／科研部署</x:v>
       </x:c>
       <x:c r="B23" s="2" t="n">
-        <x:f>COUNTIFS('产品阶段'!$D$2:$D$40,A23)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A23)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="2"/>
@@ -1919,15 +2031,15 @@
         <x:v>许可</x:v>
       </x:c>
       <x:c r="B26" s="5" t="n">
-        <x:f>'事件与财务'!B29</x:f>
+        <x:f>'事件与财务'!B32</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C26" s="5" t="n">
-        <x:f>'事件与财务'!C29</x:f>
+        <x:f>'事件与财务'!C32</x:f>
         <x:v>613826</x:v>
       </x:c>
       <x:c r="D26" s="6" t="n">
-        <x:f>C26/'事件与财务'!C32</x:f>
+        <x:f>C26/'事件与财务'!C35</x:f>
         <x:v>0.5020065508343932</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
@@ -1947,15 +2059,15 @@
         <x:v>产品</x:v>
       </x:c>
       <x:c r="B27" s="5" t="n">
-        <x:f>'事件与财务'!B30</x:f>
+        <x:f>'事件与财务'!B33</x:f>
         <x:v>19184</x:v>
       </x:c>
       <x:c r="C27" s="5" t="n">
-        <x:f>'事件与财务'!C30</x:f>
+        <x:f>'事件与财务'!C33</x:f>
         <x:v>110362</x:v>
       </x:c>
       <x:c r="D27" s="6" t="n">
-        <x:f>C27/'事件与财务'!C32</x:f>
+        <x:f>C27/'事件与财务'!C35</x:f>
         <x:v>0.09025757619127454</x:v>
       </x:c>
       <x:c r="E27" s="2"/>
@@ -1975,15 +2087,15 @@
         <x:v>开发服务</x:v>
       </x:c>
       <x:c r="B28" s="5" t="n">
-        <x:f>'事件与财务'!B31</x:f>
+        <x:f>'事件与财务'!B34</x:f>
         <x:v>1004395</x:v>
       </x:c>
       <x:c r="C28" s="5" t="n">
-        <x:f>'事件与财务'!C31</x:f>
+        <x:f>'事件与财务'!C34</x:f>
         <x:v>498557</x:v>
       </x:c>
       <x:c r="D28" s="6" t="n">
-        <x:f>C28/'事件与财务'!C32</x:f>
+        <x:f>C28/'事件与财务'!C35</x:f>
         <x:v>0.40773587297433234</x:v>
       </x:c>
       <x:c r="E28" s="2"/>
@@ -2219,10 +2331,18 @@
       <x:c r="O38" s="2"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
-      <x:c r="A39" s="2"/>
-      <x:c r="B39" s="2"/>
-      <x:c r="C39" s="2"/>
-      <x:c r="D39" s="2"/>
+      <x:c r="A39" s="159" t="str">
+        <x:v>可核商业化合同</x:v>
+      </x:c>
+      <x:c r="B39" s="159" t="str">
+        <x:v>签约日</x:v>
+      </x:c>
+      <x:c r="C39" s="159" t="str">
+        <x:v>合同授予值</x:v>
+      </x:c>
+      <x:c r="D39" s="159" t="str">
+        <x:v>边界</x:v>
+      </x:c>
       <x:c r="E39" s="2"/>
       <x:c r="F39" s="2"/>
       <x:c r="G39" s="2"/>
@@ -2235,18 +2355,18 @@
       <x:c r="N39" s="2"/>
       <x:c r="O39" s="2"/>
     </x:row>
-    <x:row r="40" ht="30" customHeight="1">
-      <x:c r="A40" s="120" t="str">
-        <x:v>并购与退出追溯</x:v>
-      </x:c>
-      <x:c r="B40" s="120" t="str">
-        <x:v>日期</x:v>
-      </x:c>
-      <x:c r="C40" s="120" t="str">
-        <x:v>状态</x:v>
-      </x:c>
-      <x:c r="D40" s="120" t="str">
-        <x:v>证据边界</x:v>
+    <x:row r="40" ht="34" customHeight="1">
+      <x:c r="A40" s="151" t="str">
+        <x:v>Jülich → SpiNNcloud</x:v>
+      </x:c>
+      <x:c r="B40" s="152" t="d">
+        <x:v>2026-02-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C40" s="160" t="n">
+        <x:v>3360000</x:v>
+      </x:c>
+      <x:c r="D40" s="151" t="str">
+        <x:v>欧元；1套；公共采购合同，不等于已付款或确认收入</x:v>
       </x:c>
       <x:c r="E40" s="2"/>
       <x:c r="F40" s="2"/>
@@ -2260,18 +2380,18 @@
       <x:c r="N40" s="2"/>
       <x:c r="O40" s="2"/>
     </x:row>
-    <x:row r="41" ht="42" customHeight="1">
-      <x:c r="A41" s="3" t="str">
-        <x:v>GrAI Matter Labs → Snap</x:v>
-      </x:c>
-      <x:c r="B41" s="4" t="n">
-        <x:v>45230</x:v>
-      </x:c>
-      <x:c r="C41" s="3" t="str">
-        <x:v>交易后于2024-02-01吸收合并注销</x:v>
-      </x:c>
-      <x:c r="D41" s="3" t="str">
-        <x:v>不再计独立供应商；技术落地与收购价未知</x:v>
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="151" t="str">
+        <x:v>莱比锡科研设施资助</x:v>
+      </x:c>
+      <x:c r="B41" s="152" t="d">
+        <x:v>2025-10-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C41" s="160" t="n">
+        <x:v>4000000</x:v>
+      </x:c>
+      <x:c r="D41" s="151" t="str">
+        <x:v>约数；基础设施资助，不是SpiNNcloud合同额，二者不合并</x:v>
       </x:c>
       <x:c r="E41" s="2"/>
       <x:c r="F41" s="2"/>
@@ -2286,18 +2406,10 @@
       <x:c r="O41" s="2"/>
     </x:row>
     <x:row r="42" ht="42" customHeight="1">
-      <x:c r="A42" s="3" t="str">
-        <x:v>iniVation → SynSense Group</x:v>
-      </x:c>
-      <x:c r="B42" s="4" t="n">
-        <x:v>45323</x:v>
-      </x:c>
-      <x:c r="C42" s="3" t="str">
-        <x:v>100%股份收购；苏黎世实体继续运营</x:v>
-      </x:c>
-      <x:c r="D42" s="3" t="str">
-        <x:v>交易金额未知；品牌／产品继续不等于独立所有权</x:v>
-      </x:c>
+      <x:c r="A42" s="151"/>
+      <x:c r="B42" s="151"/>
+      <x:c r="C42" s="151"/>
+      <x:c r="D42" s="151"/>
       <x:c r="E42" s="2"/>
       <x:c r="F42" s="2"/>
       <x:c r="G42" s="2"/>
@@ -2311,17 +2423,17 @@
       <x:c r="O42" s="2"/>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
-      <x:c r="A43" s="3" t="str">
-        <x:v>Knowles消费MEMS麦克风 → Syntiant</x:v>
-      </x:c>
-      <x:c r="B43" s="4" t="n">
-        <x:v>45656</x:v>
-      </x:c>
-      <x:c r="C43" s="3" t="str">
-        <x:v>已完成；1.5亿美元现金加股票</x:v>
-      </x:c>
-      <x:c r="D43" s="3" t="str">
-        <x:v>2.56亿美元为被收购业务2023收入，不是NDP芯片收入</x:v>
+      <x:c r="A43" s="159" t="str">
+        <x:v>并购与退出追溯</x:v>
+      </x:c>
+      <x:c r="B43" s="159" t="str">
+        <x:v>日期</x:v>
+      </x:c>
+      <x:c r="C43" s="159" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+      <x:c r="D43" s="159" t="str">
+        <x:v>证据边界</x:v>
       </x:c>
       <x:c r="E43" s="2"/>
       <x:c r="F43" s="2"/>
@@ -2335,18 +2447,18 @@
       <x:c r="N43" s="2"/>
       <x:c r="O43" s="2"/>
     </x:row>
-    <x:row r="44" ht="42" customHeight="1">
-      <x:c r="A44" s="3" t="str">
-        <x:v>Videantis → Mythic</x:v>
-      </x:c>
-      <x:c r="B44" s="4" t="n">
-        <x:v>46161</x:v>
-      </x:c>
-      <x:c r="C44" s="3" t="str">
-        <x:v>已完成</x:v>
-      </x:c>
-      <x:c r="D44" s="3" t="str">
-        <x:v>Videantis既有装机不计Mythic模拟APU出货</x:v>
+    <x:row r="44" ht="34" customHeight="1">
+      <x:c r="A44" s="151" t="str">
+        <x:v>GrAI Matter Labs → Snap</x:v>
+      </x:c>
+      <x:c r="B44" s="152" t="d">
+        <x:v>2023-10-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C44" s="151" t="str">
+        <x:v>交易后于2024-02-01吸收合并注销</x:v>
+      </x:c>
+      <x:c r="D44" s="151" t="str">
+        <x:v>不再计独立供应商；技术落地与收购价未知</x:v>
       </x:c>
       <x:c r="E44" s="2"/>
       <x:c r="F44" s="2"/>
@@ -2360,18 +2472,18 @@
       <x:c r="N44" s="2"/>
       <x:c r="O44" s="2"/>
     </x:row>
-    <x:row r="45" ht="42" customHeight="1">
-      <x:c r="A45" s="3" t="str">
-        <x:v>SceniX → World Labs</x:v>
-      </x:c>
-      <x:c r="B45" s="4" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="C45" s="3" t="str">
-        <x:v>已并入；R2S2R机器人仿真链</x:v>
-      </x:c>
-      <x:c r="D45" s="3" t="str">
-        <x:v>公司展示未独立复现；金额和客户收入未知</x:v>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="151" t="str">
+        <x:v>iniVation → SynSense Group</x:v>
+      </x:c>
+      <x:c r="B45" s="152" t="d">
+        <x:v>2024-02-01T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C45" s="151" t="str">
+        <x:v>100%股份收购；苏黎世实体继续运营</x:v>
+      </x:c>
+      <x:c r="D45" s="151" t="str">
+        <x:v>交易金额未知；品牌／产品继续不等于独立所有权</x:v>
       </x:c>
       <x:c r="E45" s="2"/>
       <x:c r="F45" s="2"/>
@@ -2385,18 +2497,18 @@
       <x:c r="N45" s="2"/>
       <x:c r="O45" s="2"/>
     </x:row>
-    <x:row r="46" ht="42" customHeight="1">
-      <x:c r="A46" s="3" t="str">
-        <x:v>World Labs → AMD</x:v>
-      </x:c>
-      <x:c r="B46" s="4" t="n">
-        <x:v>46291</x:v>
-      </x:c>
-      <x:c r="C46" s="3" t="str">
-        <x:v>已签协议，预计年底完成</x:v>
-      </x:c>
-      <x:c r="D46" s="3" t="str">
-        <x:v>约82亿美元全股票；仍待监管与交割条件</x:v>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="151" t="str">
+        <x:v>Knowles消费MEMS麦克风 → Syntiant</x:v>
+      </x:c>
+      <x:c r="B46" s="152" t="d">
+        <x:v>2024-12-30T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C46" s="151" t="str">
+        <x:v>已完成；1.5亿美元现金加股票</x:v>
+      </x:c>
+      <x:c r="D46" s="151" t="str">
+        <x:v>2.56亿美元为被收购业务2023收入，不是NDP芯片收入</x:v>
       </x:c>
       <x:c r="E46" s="2"/>
       <x:c r="F46" s="2"/>
@@ -2410,16 +2522,18 @@
       <x:c r="N46" s="2"/>
       <x:c r="O46" s="2"/>
     </x:row>
-    <x:row r="47" ht="42" customHeight="1">
-      <x:c r="A47" s="3" t="str">
-        <x:v>统计边界</x:v>
-      </x:c>
-      <x:c r="B47" s="3"/>
-      <x:c r="C47" s="3" t="str">
-        <x:v>6项交易／整合记录</x:v>
-      </x:c>
-      <x:c r="D47" s="3" t="str">
-        <x:v>拟收购与已完成交易分开；交易额、被收购业务收入和芯片收入不混用</x:v>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="151" t="str">
+        <x:v>Videantis → Mythic</x:v>
+      </x:c>
+      <x:c r="B47" s="152" t="d">
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C47" s="151" t="str">
+        <x:v>已完成</x:v>
+      </x:c>
+      <x:c r="D47" s="151" t="str">
+        <x:v>Videantis既有装机不计Mythic模拟APU出货</x:v>
       </x:c>
       <x:c r="E47" s="2"/>
       <x:c r="F47" s="2"/>
@@ -2433,11 +2547,19 @@
       <x:c r="N47" s="2"/>
       <x:c r="O47" s="2"/>
     </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="2"/>
-      <x:c r="B48" s="2"/>
-      <x:c r="C48" s="2"/>
-      <x:c r="D48" s="2"/>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="151" t="str">
+        <x:v>SceniX → World Labs</x:v>
+      </x:c>
+      <x:c r="B48" s="152" t="d">
+        <x:v>2026-07-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C48" s="151" t="str">
+        <x:v>已并入；R2S2R机器人仿真链</x:v>
+      </x:c>
+      <x:c r="D48" s="151" t="str">
+        <x:v>公司展示未独立复现；金额和客户收入未知</x:v>
+      </x:c>
       <x:c r="E48" s="2"/>
       <x:c r="F48" s="2"/>
       <x:c r="G48" s="2"/>
@@ -2450,11 +2572,19 @@
       <x:c r="N48" s="2"/>
       <x:c r="O48" s="2"/>
     </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="2"/>
-      <x:c r="B49" s="2"/>
-      <x:c r="C49" s="2"/>
-      <x:c r="D49" s="2"/>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="151" t="str">
+        <x:v>World Labs → AMD</x:v>
+      </x:c>
+      <x:c r="B49" s="152" t="d">
+        <x:v>2026-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C49" s="151" t="str">
+        <x:v>已签协议，预计年底完成</x:v>
+      </x:c>
+      <x:c r="D49" s="151" t="str">
+        <x:v>约82亿美元全股票；仍待监管与交割条件</x:v>
+      </x:c>
       <x:c r="E49" s="2"/>
       <x:c r="F49" s="2"/>
       <x:c r="G49" s="2"/>
@@ -2468,10 +2598,10 @@
       <x:c r="O49" s="2"/>
     </x:row>
     <x:row r="50">
-      <x:c r="A50" s="2"/>
-      <x:c r="B50" s="2"/>
-      <x:c r="C50" s="2"/>
-      <x:c r="D50" s="2"/>
+      <x:c r="A50"/>
+      <x:c r="B50"/>
+      <x:c r="C50"/>
+      <x:c r="D50"/>
       <x:c r="E50" s="2"/>
       <x:c r="F50" s="2"/>
       <x:c r="G50" s="2"/>
@@ -2656,7 +2786,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15f8d2f46aaf4ccf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39bdcc3e8f274e8a"/>
 </x:worksheet>
 </file>
 
@@ -2710,7 +2840,7 @@
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
     </x:row>
-    <x:row r="2" ht="70" customHeight="1">
+    <x:row r="2" ht="74" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>C001</x:v>
       </x:c>
@@ -2735,8 +2865,8 @@
       <x:c r="H2" s="3" t="str">
         <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
       </x:c>
-      <x:c r="I2" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I2" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
@@ -2745,7 +2875,7 @@
       <x:c r="N2" s="2"/>
       <x:c r="O2" s="2"/>
     </x:row>
-    <x:row r="3" ht="70" customHeight="1">
+    <x:row r="3" ht="74" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>C002</x:v>
       </x:c>
@@ -2770,8 +2900,8 @@
       <x:c r="H3" s="3" t="str">
         <x:v>https://www.innatera.com/newsroom/joya-design-takes-neuromorphic-chip-from-design-to-device-with-first-innatera-powered-consumer-audio-product-at-awe-china/</x:v>
       </x:c>
-      <x:c r="I3" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I3" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J3" s="2"/>
       <x:c r="K3" s="2"/>
@@ -2780,7 +2910,7 @@
       <x:c r="N3" s="2"/>
       <x:c r="O3" s="2"/>
     </x:row>
-    <x:row r="4" ht="70" customHeight="1">
+    <x:row r="4" ht="74" customHeight="1">
       <x:c r="A4" s="3" t="str">
         <x:v>C003</x:v>
       </x:c>
@@ -2805,8 +2935,8 @@
       <x:c r="H4" s="3" t="str">
         <x:v>https://www.synsense.ai/synsense-and-inivation-join-forces-to-form-leading-neuromorphic-technology-provider/</x:v>
       </x:c>
-      <x:c r="I4" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I4" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J4" s="2"/>
       <x:c r="K4" s="2"/>
@@ -2815,7 +2945,7 @@
       <x:c r="N4" s="2"/>
       <x:c r="O4" s="2"/>
     </x:row>
-    <x:row r="5" ht="70" customHeight="1">
+    <x:row r="5" ht="74" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>C004</x:v>
       </x:c>
@@ -2840,8 +2970,8 @@
       <x:c r="H5" s="3" t="str">
         <x:v>https://www.prophesee.ai/event-based-camera-partners/</x:v>
       </x:c>
-      <x:c r="I5" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I5" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J5" s="2"/>
       <x:c r="K5" s="2"/>
@@ -2850,7 +2980,7 @@
       <x:c r="N5" s="2"/>
       <x:c r="O5" s="2"/>
     </x:row>
-    <x:row r="6" ht="70" customHeight="1">
+    <x:row r="6" ht="74" customHeight="1">
       <x:c r="A6" s="3" t="str">
         <x:v>C005</x:v>
       </x:c>
@@ -2864,19 +2994,19 @@
         <x:v>SpiNNaker2事件通信、Arm可编程核与混合DNN／SNN科研系统</x:v>
       </x:c>
       <x:c r="E6" s="3" t="str">
-        <x:v>Sandia确认Braunfels于2025年3月到货并部署，已开展随机游走热流模拟；莱比锡大学确认2025年10月科研系统投入运行。py-spinnaker2 v0.8.2标签提交日期2026-09-23，发布说明称首次公开Docker镜像，当前文档与Docker Hub可交叉核对。</x:v>
+        <x:v>Sandia确认Braunfels于2025年3月到货并部署，莱比锡大学确认2025年10月科研系统投入运行。德国公共采购结果141500-2026显示，Forschungszentrum Jülich于2026年2月25日与SpiNNcloud签订336万欧元、数量1套的SpiNNaker2硬件合同；单一投标、无分包。py-spinnaker2 v0.8.2标签提交日期2026-09-23。</x:v>
       </x:c>
       <x:c r="F6" s="3" t="str">
-        <x:v>科研系统部署由使用方确认，但供应商合同、支付、收入、复购及整机实测未知。莱比锡约400万欧元是基础设施资助，不是SpiNNcloud收入；药物筛选项目采用int8 DNN，不应计成SNN训练。SDK公开不证明规模化训练或边端持续学习量产。</x:v>
+        <x:v>商业阶段由仅确认科研部署上调为已核公共采购合同。336万欧元是合同授予值，不等于已付款或当期确认收入；与莱比锡约400万欧元科研设施资助不是同一口径。Jülich系统交付验收、收款、毛利与复购仍未知；药物筛选项目采用int8 DNN，不应计成SNN训练。</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Sandia与莱比锡大学使用方公告；ScaDS.AI项目；官方GitLab标签、SDK文档与Docker Hub。部署事实、机构宣称、分析与收入未知分列</x:v>
+        <x:v>欧盟TED公共采购结果141500-2026及德国招标镜像；Sandia与莱比锡大学使用方公告；ScaDS.AI项目；官方GitLab标签、SDK文档与Docker Hub。合同、付款、收入与科研部署分列</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
         <x:v>https://www.sandia.gov/research/news/brain-based-computing-for-nuclear-deterrence-solutions/</x:v>
       </x:c>
-      <x:c r="I6" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I6" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J6" s="2"/>
       <x:c r="K6" s="2"/>
@@ -2885,7 +3015,7 @@
       <x:c r="N6" s="2"/>
       <x:c r="O6" s="2"/>
     </x:row>
-    <x:row r="7" ht="70" customHeight="1">
+    <x:row r="7" ht="74" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>C006</x:v>
       </x:c>
@@ -2910,8 +3040,8 @@
       <x:c r="H7" s="3" t="str">
         <x:v>https://bidl-zh.readthedocs.io/en/latest/overview.html</x:v>
       </x:c>
-      <x:c r="I7" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I7" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J7" s="2"/>
       <x:c r="K7" s="2"/>
@@ -2920,7 +3050,7 @@
       <x:c r="N7" s="2"/>
       <x:c r="O7" s="2"/>
     </x:row>
-    <x:row r="8" ht="70" customHeight="1">
+    <x:row r="8" ht="74" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>C007</x:v>
       </x:c>
@@ -2945,8 +3075,8 @@
       <x:c r="H8" s="3" t="str">
         <x:v>https://www.darwinware.com/en/news/2025/publish</x:v>
       </x:c>
-      <x:c r="I8" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I8" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J8" s="2"/>
       <x:c r="K8" s="2"/>
@@ -2955,7 +3085,7 @@
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="2"/>
     </x:row>
-    <x:row r="9" ht="100" customHeight="1">
+    <x:row r="9" ht="74" customHeight="1">
       <x:c r="A9" s="3" t="str">
         <x:v>C008</x:v>
       </x:c>
@@ -2990,7 +3120,7 @@
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="2"/>
     </x:row>
-    <x:row r="10" ht="70" customHeight="1">
+    <x:row r="10" ht="74" customHeight="1">
       <x:c r="A10" s="3" t="str">
         <x:v>C009</x:v>
       </x:c>
@@ -3015,8 +3145,8 @@
       <x:c r="H10" s="3" t="str">
         <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
       </x:c>
-      <x:c r="I10" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I10" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J10" s="2"/>
       <x:c r="K10" s="2"/>
@@ -3025,7 +3155,7 @@
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
     </x:row>
-    <x:row r="11" ht="70" customHeight="1">
+    <x:row r="11" ht="74" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>C010</x:v>
       </x:c>
@@ -3050,8 +3180,8 @@
       <x:c r="H11" s="3" t="str">
         <x:v>https://www.thepaper.cn/newsDetail_forward_33199538</x:v>
       </x:c>
-      <x:c r="I11" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I11" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J11" s="2"/>
       <x:c r="K11" s="2"/>
@@ -3060,7 +3190,7 @@
       <x:c r="N11" s="2"/>
       <x:c r="O11" s="2"/>
     </x:row>
-    <x:row r="12" ht="70" customHeight="1">
+    <x:row r="12" ht="74" customHeight="1">
       <x:c r="A12" s="3" t="str">
         <x:v>C011</x:v>
       </x:c>
@@ -3074,19 +3204,19 @@
         <x:v>BiGPU，GPU与BPU双模同构；具身大小脑芯片、BrainOS、OmniRT</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
-        <x:v>PAICORE 2.5测试芯片回片并完成原型板首测；北京日报客户端2026-08-24报道团队在机器人赛事中使用自研OmniRT，6月与乐聚签署芯片适配等战略合作</x:v>
+        <x:v>PAICORE 2.5测试芯片回片并完成原型板首测；8月24日钛媒体报道公司披露完成过亿元种子+轮，距5月数亿元种子轮约三个月；资金拟用于量产芯片研发及BrainOS、OmniRT产品化和商用交付。团队另在机器人赛事使用OmniRT，并与乐聚签署芯片适配等合作。</x:v>
       </x:c>
       <x:c r="F12" s="3" t="str">
-        <x:v>证明工程工具存在和协同验证，不等于量产或付费。2027年二季度投产仍是计划；9月外部开放、客户付费与正式规格未知</x:v>
+        <x:v>两轮融资分开记录，融资不计收入，也不证明量产。PAICORE 2.5仍是测试芯片；2027年二季度投产、9月外部开放、客户付费与正式产品规格仍待核。报道中的联调／合作交流不等于采购、验收或收入。</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>北大、北京日报客户端与中国机器人产业发展联盟；公司技术／合作口径，检索2026-10-02</x:v>
+        <x:v>中关村发展集团公众号转载、钛媒体融资稿、北大、北京日报客户端与中国机器人产业发展联盟；融资、技术、合作与收入分列，检索2026-10-02</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>https://news.bjd.com.cn/2026/08/24/90070084.shtml</x:v>
-      </x:c>
-      <x:c r="I12" s="4" t="n">
-        <x:v>46297</x:v>
+        <x:v>https://www.tmtpost.com/8113528.html</x:v>
+      </x:c>
+      <x:c r="I12" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J12" s="2"/>
       <x:c r="K12" s="2"/>
@@ -3095,7 +3225,7 @@
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="2"/>
     </x:row>
-    <x:row r="13" ht="70" customHeight="1">
+    <x:row r="13" ht="74" customHeight="1">
       <x:c r="A13" s="3" t="str">
         <x:v>C012</x:v>
       </x:c>
@@ -3120,8 +3250,8 @@
       <x:c r="H13" s="3" t="str">
         <x:v>https://www.ebkernel.com/</x:v>
       </x:c>
-      <x:c r="I13" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I13" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J13" s="2"/>
       <x:c r="K13" s="2"/>
@@ -3130,7 +3260,7 @@
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="2"/>
     </x:row>
-    <x:row r="14" ht="70" customHeight="1">
+    <x:row r="14" ht="74" customHeight="1">
       <x:c r="A14" s="3" t="str">
         <x:v>C013</x:v>
       </x:c>
@@ -3155,8 +3285,8 @@
       <x:c r="H14" s="3" t="str">
         <x:v>https://www.nanjing.gov.cn/njxx/202608/t20260827_5900119.html</x:v>
       </x:c>
-      <x:c r="I14" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I14" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J14" s="2"/>
       <x:c r="K14" s="2"/>
@@ -3165,7 +3295,7 @@
       <x:c r="N14" s="2"/>
       <x:c r="O14" s="2"/>
     </x:row>
-    <x:row r="15" ht="70" customHeight="1">
+    <x:row r="15" ht="74" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>C014</x:v>
       </x:c>
@@ -3190,8 +3320,8 @@
       <x:c r="H15" s="3" t="str">
         <x:v>https://www.chinastarmarket.cn/detail/2476378</x:v>
       </x:c>
-      <x:c r="I15" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I15" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J15" s="2"/>
       <x:c r="K15" s="2"/>
@@ -3200,7 +3330,7 @@
       <x:c r="N15" s="2"/>
       <x:c r="O15" s="2"/>
     </x:row>
-    <x:row r="16" ht="70" customHeight="1">
+    <x:row r="16" ht="74" customHeight="1">
       <x:c r="A16" s="3" t="str">
         <x:v>C015</x:v>
       </x:c>
@@ -3225,8 +3355,8 @@
       <x:c r="H16" s="3" t="str">
         <x:v>https://xisiid.com/blog-static/articles/%E4%BB%8E%E8%AF%AD%E8%A8%80%E7%94%9F%E6%88%90%E5%88%B0%E7%8A%B6%E6%80%81%E9%A2%84%E6%B5%8B%20-%20%E7%BE%B2%E6%82%89%E7%89%88%E5%BC%8F.html</x:v>
       </x:c>
-      <x:c r="I16" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I16" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J16" s="2"/>
       <x:c r="K16" s="2"/>
@@ -3235,7 +3365,7 @@
       <x:c r="N16" s="2"/>
       <x:c r="O16" s="2"/>
     </x:row>
-    <x:row r="17" ht="70" customHeight="1">
+    <x:row r="17" ht="74" customHeight="1">
       <x:c r="A17" s="3" t="str">
         <x:v>C016</x:v>
       </x:c>
@@ -3260,8 +3390,8 @@
       <x:c r="H17" s="3" t="str">
         <x:v>https://www.leinao.ai/about</x:v>
       </x:c>
-      <x:c r="I17" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I17" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J17" s="2"/>
       <x:c r="K17" s="2"/>
@@ -3270,7 +3400,7 @@
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
     </x:row>
-    <x:row r="18" ht="70" customHeight="1">
+    <x:row r="18" ht="74" customHeight="1">
       <x:c r="A18" s="3" t="str">
         <x:v>C017</x:v>
       </x:c>
@@ -3295,8 +3425,8 @@
       <x:c r="H18" s="3" t="str">
         <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
       </x:c>
-      <x:c r="I18" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I18" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J18" s="2"/>
       <x:c r="K18" s="2"/>
@@ -3305,7 +3435,7 @@
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="2"/>
     </x:row>
-    <x:row r="19" ht="70" customHeight="1">
+    <x:row r="19" ht="74" customHeight="1">
       <x:c r="A19" s="3" t="str">
         <x:v>C018</x:v>
       </x:c>
@@ -3330,8 +3460,8 @@
       <x:c r="H19" s="3" t="str">
         <x:v>https://blumind.ai/products/</x:v>
       </x:c>
-      <x:c r="I19" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I19" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J19" s="2"/>
       <x:c r="K19" s="2"/>
@@ -3340,7 +3470,7 @@
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="2"/>
     </x:row>
-    <x:row r="20" ht="70" customHeight="1">
+    <x:row r="20" ht="74" customHeight="1">
       <x:c r="A20" s="3" t="str">
         <x:v>C019</x:v>
       </x:c>
@@ -3365,8 +3495,8 @@
       <x:c r="H20" s="3" t="str">
         <x:v>https://www.aspinity.com/products.html</x:v>
       </x:c>
-      <x:c r="I20" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I20" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J20" s="2"/>
       <x:c r="K20" s="2"/>
@@ -3375,7 +3505,7 @@
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="2"/>
     </x:row>
-    <x:row r="21" ht="70" customHeight="1">
+    <x:row r="21" ht="74" customHeight="1">
       <x:c r="A21" s="3" t="str">
         <x:v>C020</x:v>
       </x:c>
@@ -3400,8 +3530,8 @@
       <x:c r="H21" s="3" t="str">
         <x:v>https://www.reexen.com/</x:v>
       </x:c>
-      <x:c r="I21" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I21" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J21" s="2"/>
       <x:c r="K21" s="2"/>
@@ -3410,7 +3540,7 @@
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="2"/>
     </x:row>
-    <x:row r="22" ht="70" customHeight="1">
+    <x:row r="22" ht="74" customHeight="1">
       <x:c r="A22" s="3" t="str">
         <x:v>C021</x:v>
       </x:c>
@@ -3435,8 +3565,8 @@
       <x:c r="H22" s="3" t="str">
         <x:v>https://rain.ai/products</x:v>
       </x:c>
-      <x:c r="I22" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I22" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J22" s="2"/>
       <x:c r="K22" s="2"/>
@@ -3445,7 +3575,7 @@
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="2"/>
     </x:row>
-    <x:row r="23" ht="70" customHeight="1">
+    <x:row r="23" ht="74" customHeight="1">
       <x:c r="A23" s="3" t="str">
         <x:v>C022</x:v>
       </x:c>
@@ -3470,8 +3600,8 @@
       <x:c r="H23" s="3" t="str">
         <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
       </x:c>
-      <x:c r="I23" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I23" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J23" s="2"/>
       <x:c r="K23" s="2"/>
@@ -3480,7 +3610,7 @@
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="2"/>
     </x:row>
-    <x:row r="24" ht="70" customHeight="1">
+    <x:row r="24" ht="74" customHeight="1">
       <x:c r="A24" s="3" t="str">
         <x:v>C023</x:v>
       </x:c>
@@ -3505,8 +3635,8 @@
       <x:c r="H24" s="3" t="str">
         <x:v>https://synthara.ai/wp-content/uploads/2025/03/EW-version-Leaflet-Trifolds.pdf</x:v>
       </x:c>
-      <x:c r="I24" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I24" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J24" s="2"/>
       <x:c r="K24" s="2"/>
@@ -3515,7 +3645,7 @@
       <x:c r="N24" s="2"/>
       <x:c r="O24" s="2"/>
     </x:row>
-    <x:row r="25" ht="70" customHeight="1">
+    <x:row r="25" ht="74" customHeight="1">
       <x:c r="A25" s="3" t="str">
         <x:v>C024</x:v>
       </x:c>
@@ -3540,8 +3670,8 @@
       <x:c r="H25" s="3" t="str">
         <x:v>https://www.neurxcore.com/</x:v>
       </x:c>
-      <x:c r="I25" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I25" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J25" s="2"/>
       <x:c r="K25" s="2"/>
@@ -3550,7 +3680,7 @@
       <x:c r="N25" s="2"/>
       <x:c r="O25" s="2"/>
     </x:row>
-    <x:row r="26" ht="70" customHeight="1">
+    <x:row r="26" ht="74" customHeight="1">
       <x:c r="A26" s="3" t="str">
         <x:v>C025</x:v>
       </x:c>
@@ -3575,8 +3705,8 @@
       <x:c r="H26" s="3" t="str">
         <x:v>https://www.axera-tech.com/zh-hans/news/3270.html</x:v>
       </x:c>
-      <x:c r="I26" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I26" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J26" s="2"/>
       <x:c r="K26" s="2"/>
@@ -3585,7 +3715,7 @@
       <x:c r="N26" s="2"/>
       <x:c r="O26" s="2"/>
     </x:row>
-    <x:row r="27" ht="70" customHeight="1">
+    <x:row r="27" ht="74" customHeight="1">
       <x:c r="A27" s="3" t="str">
         <x:v>C026</x:v>
       </x:c>
@@ -3610,8 +3740,8 @@
       <x:c r="H27" s="3" t="str">
         <x:v>https://www.syntiant.com/press-release/syntiant-completes-acquisition-of-knowles-consumer-mems-microphone-division/</x:v>
       </x:c>
-      <x:c r="I27" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I27" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J27" s="2"/>
       <x:c r="K27" s="2"/>
@@ -3620,7 +3750,7 @@
       <x:c r="N27" s="2"/>
       <x:c r="O27" s="2"/>
     </x:row>
-    <x:row r="28" ht="70" customHeight="1">
+    <x:row r="28" ht="74" customHeight="1">
       <x:c r="A28" s="3" t="str">
         <x:v>C027</x:v>
       </x:c>
@@ -3645,8 +3775,8 @@
       <x:c r="H28" s="3" t="str">
         <x:v>https://www.mythic.ai/vanguard</x:v>
       </x:c>
-      <x:c r="I28" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I28" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J28" s="2"/>
       <x:c r="K28" s="2"/>
@@ -3655,7 +3785,7 @@
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="2"/>
     </x:row>
-    <x:row r="29" ht="70" customHeight="1">
+    <x:row r="29" ht="74" customHeight="1">
       <x:c r="A29" s="3" t="str">
         <x:v>C028</x:v>
       </x:c>
@@ -3680,8 +3810,8 @@
       <x:c r="H29" s="3" t="str">
         <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
       </x:c>
-      <x:c r="I29" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I29" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J29" s="2"/>
       <x:c r="K29" s="2"/>
@@ -3690,7 +3820,7 @@
       <x:c r="N29" s="2"/>
       <x:c r="O29" s="2"/>
     </x:row>
-    <x:row r="30" ht="70" customHeight="1">
+    <x:row r="30" ht="74" customHeight="1">
       <x:c r="A30" s="3" t="str">
         <x:v>C029</x:v>
       </x:c>
@@ -3715,8 +3845,8 @@
       <x:c r="H30" s="3" t="str">
         <x:v>https://semiqa.com/en/technology</x:v>
       </x:c>
-      <x:c r="I30" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I30" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J30" s="2"/>
       <x:c r="K30" s="2"/>
@@ -3725,33 +3855,33 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="70" customHeight="1">
-      <x:c r="A31" s="2" t="str">
+    <x:row r="31" ht="74" customHeight="1">
+      <x:c r="A31" s="3" t="str">
         <x:v>C030</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="str">
+      <x:c r="B31" s="3" t="str">
         <x:v>STMicroelectronics</x:v>
       </x:c>
-      <x:c r="C31" s="2" t="str">
+      <x:c r="C31" s="3" t="str">
         <x:v>相邻替代</x:v>
       </x:c>
-      <x:c r="D31" s="2" t="str">
+      <x:c r="D31" s="3" t="str">
         <x:v>STM32N6 Cortex-M55 MCU＋Neural-ART NPU；STM32Cube AI Studio与N6开发板</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="str">
+      <x:c r="E31" s="3" t="str">
         <x:v>STM32N657X0量产SKU与STM32N6570-DK／NUCLEO开发板已有官方Active、量产及直接购买入口；NPU工具按算子映射，未支持算子回退CPU</x:v>
       </x:c>
-      <x:c r="F31" s="2" t="str">
+      <x:c r="F31" s="3" t="str">
         <x:v>官方页面检索时未显示经销商库存，ST直购入口存在；量产状态不等于类脑任务设计定点。工具证据聚焦推理，未见权重在线更新；厂商600 GOPS不能与SNN事件任务直接排名</x:v>
       </x:c>
-      <x:c r="G31" s="2" t="str">
+      <x:c r="G31" s="3" t="str">
         <x:v>ST官方芯片、开发板、AI工具与部署教程；产品状态和购买入口为事实，性能为厂商口径</x:v>
       </x:c>
-      <x:c r="H31" s="2" t="str">
+      <x:c r="H31" s="3" t="str">
         <x:v>https://www.st.com/en/evaluation-tools/stm32n6570-dk.html</x:v>
       </x:c>
-      <x:c r="I31" s="11" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I31" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J31" s="2"/>
       <x:c r="K31" s="2"/>
@@ -3760,33 +3890,33 @@
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="2"/>
     </x:row>
-    <x:row r="32" ht="70" customHeight="1">
-      <x:c r="A32" s="2" t="str">
+    <x:row r="32" ht="74" customHeight="1">
+      <x:c r="A32" s="3" t="str">
         <x:v>C031</x:v>
       </x:c>
-      <x:c r="B32" s="2" t="str">
+      <x:c r="B32" s="3" t="str">
         <x:v>NXP</x:v>
       </x:c>
-      <x:c r="C32" s="2" t="str">
+      <x:c r="C32" s="3" t="str">
         <x:v>相邻替代</x:v>
       </x:c>
-      <x:c r="D32" s="2" t="str">
+      <x:c r="D32" s="3" t="str">
         <x:v>i.MX RT700双Cortex-M33＋HiFi DSP＋eIQ Neutron NPU；MCUXpresso</x:v>
       </x:c>
-      <x:c r="E32" s="2" t="str">
+      <x:c r="E32" s="3" t="str">
         <x:v>MIMXRT700-EVK官方状态Active，10月2日页面显示2套现货、187.23美元并可下单；NXP已发布NPU编译与门铃、摄像头、手表等参考应用</x:v>
       </x:c>
-      <x:c r="F32" s="2" t="str">
+      <x:c r="F32" s="3" t="str">
         <x:v>开发板现货和完整文档不证明终端量产或收入；公开材料聚焦量化模型编译与推理，未见本地权重更新。厂商加速倍数不能跨任务横比</x:v>
       </x:c>
-      <x:c r="G32" s="2" t="str">
+      <x:c r="G32" s="3" t="str">
         <x:v>NXP官方EVK商品页、RT700产品页与AN14700；库存、价格为检索时快照</x:v>
       </x:c>
-      <x:c r="H32" s="2" t="str">
+      <x:c r="H32" s="3" t="str">
         <x:v>https://www.nxp.com/design/design-center/software/development-software/mcuxpresso-software-and-tools-/i-mx-rt700-evaluation-kit:MIMXRT700-EVK</x:v>
       </x:c>
-      <x:c r="I32" s="11" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I32" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J32" s="2"/>
       <x:c r="K32" s="2"/>
@@ -3795,33 +3925,33 @@
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="2"/>
     </x:row>
-    <x:row r="33" ht="70" customHeight="1">
-      <x:c r="A33" s="2" t="str">
+    <x:row r="33" ht="74" customHeight="1">
+      <x:c r="A33" s="3" t="str">
         <x:v>C032</x:v>
       </x:c>
-      <x:c r="B33" s="2" t="str">
+      <x:c r="B33" s="3" t="str">
         <x:v>Synaptics</x:v>
       </x:c>
-      <x:c r="C33" s="2" t="str">
+      <x:c r="C33" s="3" t="str">
         <x:v>相邻替代</x:v>
       </x:c>
-      <x:c r="D33" s="2" t="str">
+      <x:c r="D33" s="3" t="str">
         <x:v>Astra SL2610多模态IoT处理器；Torq T1／Coral NPU；Astra Machina开发套件</x:v>
       </x:c>
-      <x:c r="E33" s="2" t="str">
+      <x:c r="E33" s="3" t="str">
         <x:v>SL2610开发套件官网已给出Mouser、DigiKey和Codico购买入口，并提供2026年用户指南、数据表与视觉／语音／LLM NPU教程；Torq基于开源IREE／MLIR</x:v>
       </x:c>
-      <x:c r="F33" s="2" t="str">
+      <x:c r="F33" s="3" t="str">
         <x:v>购买入口不等于库存与终端量产；2025公告中的Q2 2026 GA计划不能替代当前芯片出货量。公开教程是推理工作流，未见片上在线学习或具名付费客户规模</x:v>
       </x:c>
-      <x:c r="G33" s="2" t="str">
+      <x:c r="G33" s="3" t="str">
         <x:v>Synaptics官方产品、开发者文档与分销入口；伙伴引述不作为销量证据</x:v>
       </x:c>
-      <x:c r="H33" s="2" t="str">
+      <x:c r="H33" s="3" t="str">
         <x:v>https://www.synaptics.com/products/embedded-processors/sl2610-product-line</x:v>
       </x:c>
-      <x:c r="I33" s="11" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I33" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J33" s="2"/>
       <x:c r="K33" s="2"/>
@@ -3830,33 +3960,33 @@
       <x:c r="N33" s="2"/>
       <x:c r="O33" s="2"/>
     </x:row>
-    <x:row r="34" ht="70" customHeight="1">
-      <x:c r="A34" s="2" t="str">
+    <x:row r="34" ht="74" customHeight="1">
+      <x:c r="A34" s="3" t="str">
         <x:v>C033</x:v>
       </x:c>
-      <x:c r="B34" s="2" t="str">
+      <x:c r="B34" s="3" t="str">
         <x:v>Hailo</x:v>
       </x:c>
-      <x:c r="C34" s="2" t="str">
+      <x:c r="C34" s="3" t="str">
         <x:v>相邻替代</x:v>
       </x:c>
-      <x:c r="D34" s="2" t="str">
+      <x:c r="D34" s="3" t="str">
         <x:v>Hailo-10H离散数据流AI加速器与M.2模块；视觉、LLM与VLM本地推理</x:v>
       </x:c>
-      <x:c r="E34" s="2" t="str">
+      <x:c r="E34" s="3" t="str">
         <x:v>Hailo于2025年7月22日宣布Hailo-10H商业可用并接受全球订单；当前官网商店和区域经销页面仍列M.2模块，产品简报给出40／20 TOPS（INT4／8）与典型2.5W</x:v>
       </x:c>
-      <x:c r="F34" s="2" t="str">
+      <x:c r="F34" s="3" t="str">
         <x:v>可下单和厂商基准不等于终端设计定点、销量或收入；汽车2026 SOP是目标。公开资料聚焦推理，未见本地权重更新；功耗指标不与不同模型和系统边界横比</x:v>
       </x:c>
-      <x:c r="G34" s="2" t="str">
+      <x:c r="G34" s="3" t="str">
         <x:v>Hailo官方GA公告、产品简报与商店；性能、功耗和用户数均为厂商口径</x:v>
       </x:c>
-      <x:c r="H34" s="2" t="str">
+      <x:c r="H34" s="3" t="str">
         <x:v>https://hailo.ai/company-overview/newsroom/news/hailo-announces-general-availability-of-hailo-10h-edge-ai-accelerator-with-generative-ai-capabilities/</x:v>
       </x:c>
-      <x:c r="I34" s="11" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I34" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J34" s="2"/>
       <x:c r="K34" s="2"/>
@@ -3865,7 +3995,7 @@
       <x:c r="N34" s="2"/>
       <x:c r="O34" s="2"/>
     </x:row>
-    <x:row r="35" ht="70" customHeight="1">
+    <x:row r="35" ht="74" customHeight="1">
       <x:c r="A35" s="3" t="str">
         <x:v>C034</x:v>
       </x:c>
@@ -3890,8 +4020,8 @@
       <x:c r="H35" s="3" t="str">
         <x:v>https://www.digikey.com/en/products/detail/ambiq-micro-inc/AP510BEVB/28007828</x:v>
       </x:c>
-      <x:c r="I35" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I35" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J35" s="2"/>
       <x:c r="K35" s="2"/>
@@ -3900,7 +4030,7 @@
       <x:c r="N35" s="2"/>
       <x:c r="O35" s="2"/>
     </x:row>
-    <x:row r="36" ht="70" customHeight="1">
+    <x:row r="36" ht="74" customHeight="1">
       <x:c r="A36" s="3" t="str">
         <x:v>C035</x:v>
       </x:c>
@@ -3925,8 +4055,8 @@
       <x:c r="H36" s="3" t="str">
         <x:v>https://ir.amd.com/news-events/press-releases/detail/1299/amd-to-acquire-world-labs-to-advance-the-future-of-ai-compute</x:v>
       </x:c>
-      <x:c r="I36" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I36" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J36" s="2"/>
       <x:c r="K36" s="2"/>
@@ -3935,7 +4065,7 @@
       <x:c r="N36" s="2"/>
       <x:c r="O36" s="2"/>
     </x:row>
-    <x:row r="37" ht="70" customHeight="1">
+    <x:row r="37" ht="74" customHeight="1">
       <x:c r="A37" s="3" t="str">
         <x:v>C036</x:v>
       </x:c>
@@ -3960,8 +4090,8 @@
       <x:c r="H37" s="3" t="str">
         <x:v>https://patents.google.com/patent/US20260057197A1/en</x:v>
       </x:c>
-      <x:c r="I37" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I37" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J37" s="2"/>
       <x:c r="K37" s="2"/>
@@ -3970,7 +4100,7 @@
       <x:c r="N37" s="2"/>
       <x:c r="O37" s="2"/>
     </x:row>
-    <x:row r="38" ht="70" customHeight="1">
+    <x:row r="38" ht="74" customHeight="1">
       <x:c r="A38" s="3" t="str">
         <x:v>C037</x:v>
       </x:c>
@@ -3995,8 +4125,8 @@
       <x:c r="H38" s="3" t="str">
         <x:v>https://www.xenserobotics.com/article/387/detail/25</x:v>
       </x:c>
-      <x:c r="I38" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="I38" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J38" s="2"/>
       <x:c r="K38" s="2"/>
@@ -4393,7 +4523,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf40aea1433154327"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a83612ea1d4456"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4451,7 +4581,7 @@
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
     </x:row>
-    <x:row r="2" ht="64" customHeight="1">
+    <x:row r="2" ht="68" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>P001</x:v>
       </x:c>
@@ -4467,12 +4597,12 @@
       <x:c r="E2" s="3" t="str">
         <x:v>公开商品入口</x:v>
       </x:c>
-      <x:c r="F2" s="4" t="n">
-        <x:v>46282</x:v>
+      <x:c r="F2" s="4" t="d">
+        <x:v>2026-09-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G2" s="4"/>
-      <x:c r="H2" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H2" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
         <x:v>终端量产、客户数量和独立收入未知</x:v>
@@ -4486,7 +4616,7 @@
       <x:c r="N2" s="2"/>
       <x:c r="O2" s="2"/>
     </x:row>
-    <x:row r="3" ht="64" customHeight="1">
+    <x:row r="3" ht="68" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>P002</x:v>
       </x:c>
@@ -4502,12 +4632,12 @@
       <x:c r="E3" s="3" t="str">
         <x:v>具名客户模块公告</x:v>
       </x:c>
-      <x:c r="F3" s="4" t="n">
-        <x:v>46107</x:v>
+      <x:c r="F3" s="4" t="d">
+        <x:v>2026-03-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G3" s="4"/>
-      <x:c r="H3" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H3" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
         <x:v>终端批量销售和收入未知</x:v>
@@ -4521,7 +4651,7 @@
       <x:c r="N3" s="2"/>
       <x:c r="O3" s="2"/>
     </x:row>
-    <x:row r="4" ht="64" customHeight="1">
+    <x:row r="4" ht="68" customHeight="1">
       <x:c r="A4" s="3" t="str">
         <x:v>P003</x:v>
       </x:c>
@@ -4539,8 +4669,8 @@
       </x:c>
       <x:c r="F4" s="4"/>
       <x:c r="G4" s="4"/>
-      <x:c r="H4" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H4" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
         <x:v>当前公开库存未核</x:v>
@@ -4554,7 +4684,7 @@
       <x:c r="N4" s="2"/>
       <x:c r="O4" s="2"/>
     </x:row>
-    <x:row r="5" ht="64" customHeight="1">
+    <x:row r="5" ht="68" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>P004</x:v>
       </x:c>
@@ -4570,12 +4700,12 @@
       <x:c r="E5" s="3" t="str">
         <x:v>公司发布与销售联系</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="n">
-        <x:v>46197</x:v>
+      <x:c r="F5" s="4" t="d">
+        <x:v>2026-06-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G5" s="4"/>
-      <x:c r="H5" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H5" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
         <x:v>数据表、开发板、价格与生产状态未知</x:v>
@@ -4589,7 +4719,7 @@
       <x:c r="N5" s="2"/>
       <x:c r="O5" s="2"/>
     </x:row>
-    <x:row r="6" ht="64" customHeight="1">
+    <x:row r="6" ht="68" customHeight="1">
       <x:c r="A6" s="3" t="str">
         <x:v>P005</x:v>
       </x:c>
@@ -4607,8 +4737,8 @@
       </x:c>
       <x:c r="F6" s="4"/>
       <x:c r="G6" s="4"/>
-      <x:c r="H6" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H6" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
         <x:v>开发相机可买不等于终端量产</x:v>
@@ -4622,7 +4752,7 @@
       <x:c r="N6" s="2"/>
       <x:c r="O6" s="2"/>
     </x:row>
-    <x:row r="7" ht="64" customHeight="1">
+    <x:row r="7" ht="68" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>P006</x:v>
       </x:c>
@@ -4640,8 +4770,8 @@
       </x:c>
       <x:c r="F7" s="4"/>
       <x:c r="G7" s="4"/>
-      <x:c r="H7" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H7" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
         <x:v>伙伴相机销售不能计作传感器收入</x:v>
@@ -4655,7 +4785,7 @@
       <x:c r="N7" s="2"/>
       <x:c r="O7" s="2"/>
     </x:row>
-    <x:row r="8" ht="64" customHeight="1">
+    <x:row r="8" ht="68" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>P007</x:v>
       </x:c>
@@ -4671,12 +4801,12 @@
       <x:c r="E8" s="3" t="str">
         <x:v>厂商现场验证声明</x:v>
       </x:c>
-      <x:c r="F8" s="4" t="n">
-        <x:v>46188</x:v>
+      <x:c r="F8" s="4" t="d">
+        <x:v>2026-06-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G8" s="4"/>
-      <x:c r="H8" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H8" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
         <x:v>未见具名采购与部署数量</x:v>
@@ -4690,7 +4820,7 @@
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="2"/>
     </x:row>
-    <x:row r="9" ht="64" customHeight="1">
+    <x:row r="9" ht="68" customHeight="1">
       <x:c r="A9" s="3" t="str">
         <x:v>P008</x:v>
       </x:c>
@@ -4706,12 +4836,12 @@
       <x:c r="E9" s="3" t="str">
         <x:v>公司工程节点评估公告</x:v>
       </x:c>
-      <x:c r="F9" s="4" t="n">
-        <x:v>46293</x:v>
+      <x:c r="F9" s="4" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G9" s="4"/>
-      <x:c r="H9" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H9" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
         <x:v>仍为工程芯片，非量产</x:v>
@@ -4725,7 +4855,7 @@
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="2"/>
     </x:row>
-    <x:row r="10" ht="64" customHeight="1">
+    <x:row r="10" ht="68" customHeight="1">
       <x:c r="A10" s="3" t="str">
         <x:v>P009</x:v>
       </x:c>
@@ -4743,8 +4873,8 @@
       </x:c>
       <x:c r="F10" s="4"/>
       <x:c r="G10" s="4"/>
-      <x:c r="H10" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H10" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
         <x:v>仿真原型，商务暂停</x:v>
@@ -4758,7 +4888,7 @@
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
     </x:row>
-    <x:row r="11" ht="64" customHeight="1">
+    <x:row r="11" ht="68" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>P010</x:v>
       </x:c>
@@ -4776,8 +4906,8 @@
       </x:c>
       <x:c r="F11" s="4"/>
       <x:c r="G11" s="4"/>
-      <x:c r="H11" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H11" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
         <x:v>数据表、库存、客户及收入未知</x:v>
@@ -4791,7 +4921,7 @@
       <x:c r="N11" s="2"/>
       <x:c r="O11" s="2"/>
     </x:row>
-    <x:row r="12" ht="64" customHeight="1">
+    <x:row r="12" ht="68" customHeight="1">
       <x:c r="A12" s="3" t="str">
         <x:v>P011</x:v>
       </x:c>
@@ -4809,8 +4939,8 @@
       </x:c>
       <x:c r="F12" s="4"/>
       <x:c r="G12" s="4"/>
-      <x:c r="H12" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H12" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
         <x:v>客户、数量和收入未知</x:v>
@@ -4824,7 +4954,7 @@
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="2"/>
     </x:row>
-    <x:row r="13" ht="64" customHeight="1">
+    <x:row r="13" ht="68" customHeight="1">
       <x:c r="A13" s="3" t="str">
         <x:v>P012</x:v>
       </x:c>
@@ -4842,8 +4972,8 @@
       </x:c>
       <x:c r="F13" s="4"/>
       <x:c r="G13" s="4"/>
-      <x:c r="H13" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H13" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
         <x:v>开发中，不能归为量产</x:v>
@@ -4857,7 +4987,7 @@
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="2"/>
     </x:row>
-    <x:row r="14" ht="64" customHeight="1">
+    <x:row r="14" ht="68" customHeight="1">
       <x:c r="A14" s="3" t="str">
         <x:v>P013</x:v>
       </x:c>
@@ -4875,8 +5005,8 @@
       </x:c>
       <x:c r="F14" s="4"/>
       <x:c r="G14" s="4"/>
-      <x:c r="H14" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H14" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
         <x:v>现货、价格和量产客户未知</x:v>
@@ -4890,7 +5020,7 @@
       <x:c r="N14" s="2"/>
       <x:c r="O14" s="2"/>
     </x:row>
-    <x:row r="15" ht="64" customHeight="1">
+    <x:row r="15" ht="68" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>P014</x:v>
       </x:c>
@@ -4906,12 +5036,12 @@
       <x:c r="E15" s="3" t="str">
         <x:v>具名生产线部署联合稿</x:v>
       </x:c>
-      <x:c r="F15" s="4" t="n">
-        <x:v>46265</x:v>
+      <x:c r="F15" s="4" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G15" s="4"/>
-      <x:c r="H15" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H15" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
         <x:v>合同金额、数量与收入未知</x:v>
@@ -4925,7 +5055,7 @@
       <x:c r="N15" s="2"/>
       <x:c r="O15" s="2"/>
     </x:row>
-    <x:row r="16" ht="64" customHeight="1">
+    <x:row r="16" ht="68" customHeight="1">
       <x:c r="A16" s="3" t="str">
         <x:v>P015</x:v>
       </x:c>
@@ -4943,8 +5073,8 @@
       </x:c>
       <x:c r="F16" s="4"/>
       <x:c r="G16" s="4"/>
-      <x:c r="H16" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H16" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
         <x:v>公开SDK、封装芯片和design win未核</x:v>
@@ -4958,7 +5088,7 @@
       <x:c r="N16" s="2"/>
       <x:c r="O16" s="2"/>
     </x:row>
-    <x:row r="17" ht="64" customHeight="1">
+    <x:row r="17" ht="68" customHeight="1">
       <x:c r="A17" s="3" t="str">
         <x:v>P016</x:v>
       </x:c>
@@ -4976,8 +5106,8 @@
       </x:c>
       <x:c r="F17" s="4"/>
       <x:c r="G17" s="4"/>
-      <x:c r="H17" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H17" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
         <x:v>硬件尚待推出，未核硅验证</x:v>
@@ -4991,7 +5121,7 @@
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
     </x:row>
-    <x:row r="18" ht="64" customHeight="1">
+    <x:row r="18" ht="68" customHeight="1">
       <x:c r="A18" s="3" t="str">
         <x:v>P017</x:v>
       </x:c>
@@ -5007,12 +5137,12 @@
       <x:c r="E18" s="3" t="str">
         <x:v>媒体转述公司量产与订单</x:v>
       </x:c>
-      <x:c r="F18" s="4" t="n">
-        <x:v>45924</x:v>
+      <x:c r="F18" s="4" t="d">
+        <x:v>2025-09-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G18" s="4"/>
-      <x:c r="H18" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H18" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
         <x:v>客户未具名，非审计收入</x:v>
@@ -5026,7 +5156,7 @@
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="2"/>
     </x:row>
-    <x:row r="19" ht="64" customHeight="1">
+    <x:row r="19" ht="68" customHeight="1">
       <x:c r="A19" s="3" t="str">
         <x:v>P018</x:v>
       </x:c>
@@ -5044,8 +5174,8 @@
       </x:c>
       <x:c r="F19" s="4"/>
       <x:c r="G19" s="4"/>
-      <x:c r="H19" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H19" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
         <x:v>新产品样机、上市及采购未知</x:v>
@@ -5059,7 +5189,7 @@
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="2"/>
     </x:row>
-    <x:row r="20" ht="64" customHeight="1">
+    <x:row r="20" ht="68" customHeight="1">
       <x:c r="A20" s="3" t="str">
         <x:v>P019</x:v>
       </x:c>
@@ -5075,12 +5205,12 @@
       <x:c r="E20" s="3" t="str">
         <x:v>高校项目与回片报道</x:v>
       </x:c>
-      <x:c r="F20" s="4" t="n">
-        <x:v>46157</x:v>
+      <x:c r="F20" s="4" t="d">
+        <x:v>2026-05-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G20" s="4"/>
-      <x:c r="H20" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H20" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
         <x:v>量产为未来计划</x:v>
@@ -5094,7 +5224,7 @@
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="2"/>
     </x:row>
-    <x:row r="21" ht="64" customHeight="1">
+    <x:row r="21" ht="68" customHeight="1">
       <x:c r="A21" s="3" t="str">
         <x:v>P020</x:v>
       </x:c>
@@ -5110,14 +5240,14 @@
       <x:c r="E21" s="3" t="str">
         <x:v>官网公开按台／按年许可、软硬一体模组、行业方案与RaaS；媒体称客户现场部署</x:v>
       </x:c>
-      <x:c r="F21" s="4" t="n">
-        <x:v>46279</x:v>
-      </x:c>
-      <x:c r="G21" s="4" t="n">
-        <x:v>46279</x:v>
-      </x:c>
-      <x:c r="H21" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="F21" s="4" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G21" s="4" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H21" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
         <x:v>商业形态已定义；无公开价格、模组SKU、具名付费客户、验收或收入，节能仍未实测</x:v>
@@ -5131,7 +5261,7 @@
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="2"/>
     </x:row>
-    <x:row r="22" ht="64" customHeight="1">
+    <x:row r="22" ht="68" customHeight="1">
       <x:c r="A22" s="3" t="str">
         <x:v>P021</x:v>
       </x:c>
@@ -5147,12 +5277,12 @@
       <x:c r="E22" s="3" t="str">
         <x:v>Microchip IP选型公告</x:v>
       </x:c>
-      <x:c r="F22" s="4" t="n">
-        <x:v>46280</x:v>
+      <x:c r="F22" s="4" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G22" s="4"/>
-      <x:c r="H22" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H22" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
         <x:v>未见型号、流片、样片和客户</x:v>
@@ -5166,7 +5296,7 @@
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="2"/>
     </x:row>
-    <x:row r="23" ht="64" customHeight="1">
+    <x:row r="23" ht="68" customHeight="1">
       <x:c r="A23" s="3" t="str">
         <x:v>P022</x:v>
       </x:c>
@@ -5184,8 +5314,8 @@
       </x:c>
       <x:c r="F23" s="4"/>
       <x:c r="G23" s="4"/>
-      <x:c r="H23" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H23" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
         <x:v>量产定位非量产事实，未核硅验证</x:v>
@@ -5199,7 +5329,7 @@
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="2"/>
     </x:row>
-    <x:row r="24" ht="64" customHeight="1">
+    <x:row r="24" ht="68" customHeight="1">
       <x:c r="A24" s="3" t="str">
         <x:v>P023</x:v>
       </x:c>
@@ -5215,14 +5345,14 @@
       <x:c r="E24" s="3" t="str">
         <x:v>展商一手产品自述＋7月17日发布报道；ASC脉冲转换为厂商描述</x:v>
       </x:c>
-      <x:c r="F24" s="4" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="G24" s="4" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="H24" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="F24" s="4" t="d">
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G24" s="4" t="d">
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H24" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
         <x:v>已发布及演示；未见完整数据表、公开采购或量产客户，不能借传感器出货推断E10A销量</x:v>
@@ -5236,7 +5366,7 @@
       <x:c r="N24" s="2"/>
       <x:c r="O24" s="2"/>
     </x:row>
-    <x:row r="25" ht="64" customHeight="1">
+    <x:row r="25" ht="68" customHeight="1">
       <x:c r="A25" s="3" t="str">
         <x:v>P024</x:v>
       </x:c>
@@ -5252,12 +5382,12 @@
       <x:c r="E25" s="3" t="str">
         <x:v>IPO早知道9月23日全文转载的月交付声明；NVIDIA官方仿真资产及公开仓库交叉</x:v>
       </x:c>
-      <x:c r="F25" s="4" t="n">
-        <x:v>46288</x:v>
+      <x:c r="F25" s="4" t="d">
+        <x:v>2026-09-23T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G25" s="4"/>
-      <x:c r="H25" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H25" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
         <x:v>月交付数万枚未审计且型号分拆未知；仿真收录不等于实物采购，不将80%无方法市占率作事实</x:v>
@@ -5271,31 +5401,31 @@
       <x:c r="N25" s="2"/>
       <x:c r="O25" s="2"/>
     </x:row>
-    <x:row r="26" ht="64" customHeight="1">
-      <x:c r="A26" s="2" t="str">
+    <x:row r="26" ht="68" customHeight="1">
+      <x:c r="A26" s="3" t="str">
         <x:v>P025</x:v>
       </x:c>
-      <x:c r="B26" s="2" t="str">
+      <x:c r="B26" s="3" t="str">
         <x:v>STMicroelectronics</x:v>
       </x:c>
-      <x:c r="C26" s="2" t="str">
+      <x:c r="C26" s="3" t="str">
         <x:v>STM32N657X0 MCU</x:v>
       </x:c>
-      <x:c r="D26" s="2" t="str">
+      <x:c r="D26" s="3" t="str">
         <x:v>生产／部署声明</x:v>
       </x:c>
-      <x:c r="E26" s="2" t="str">
+      <x:c r="E26" s="3" t="str">
         <x:v>官方量产状态与直购入口</x:v>
       </x:c>
-      <x:c r="F26" s="11"/>
-      <x:c r="G26" s="11"/>
-      <x:c r="H26" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I26" s="2" t="str">
+      <x:c r="F26" s="4"/>
+      <x:c r="G26" s="4"/>
+      <x:c r="H26" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I26" s="3" t="str">
         <x:v>官网不同SKU状态需逐项核对；经销商库存未显示，终端量产客户与收入未知</x:v>
       </x:c>
-      <x:c r="J26" s="2" t="str">
+      <x:c r="J26" s="3" t="str">
         <x:v>https://www.st.com/en/microcontrollers-microprocessors/stm32n657x0.html</x:v>
       </x:c>
       <x:c r="K26" s="2"/>
@@ -5304,31 +5434,31 @@
       <x:c r="N26" s="2"/>
       <x:c r="O26" s="2"/>
     </x:row>
-    <x:row r="27" ht="64" customHeight="1">
-      <x:c r="A27" s="2" t="str">
+    <x:row r="27" ht="68" customHeight="1">
+      <x:c r="A27" s="3" t="str">
         <x:v>P026</x:v>
       </x:c>
-      <x:c r="B27" s="2" t="str">
+      <x:c r="B27" s="3" t="str">
         <x:v>STMicroelectronics</x:v>
       </x:c>
-      <x:c r="C27" s="2" t="str">
+      <x:c r="C27" s="3" t="str">
         <x:v>STM32N6570-DK／NUCLEO-N657X0-Q</x:v>
       </x:c>
-      <x:c r="D27" s="2" t="str">
+      <x:c r="D27" s="3" t="str">
         <x:v>可采购硬件</x:v>
       </x:c>
-      <x:c r="E27" s="2" t="str">
+      <x:c r="E27" s="3" t="str">
         <x:v>官方Active、直购／样品入口</x:v>
       </x:c>
-      <x:c r="F27" s="11"/>
-      <x:c r="G27" s="11"/>
-      <x:c r="H27" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I27" s="2" t="str">
+      <x:c r="F27" s="4"/>
+      <x:c r="G27" s="4"/>
+      <x:c r="H27" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I27" s="3" t="str">
         <x:v>检索时无经销商库存报告；开发板可买不等于终端量产</x:v>
       </x:c>
-      <x:c r="J27" s="2" t="str">
+      <x:c r="J27" s="3" t="str">
         <x:v>https://www.st.com/en/evaluation-tools/stm32n6570-dk.html</x:v>
       </x:c>
       <x:c r="K27" s="2"/>
@@ -5337,31 +5467,31 @@
       <x:c r="N27" s="2"/>
       <x:c r="O27" s="2"/>
     </x:row>
-    <x:row r="28" ht="64" customHeight="1">
-      <x:c r="A28" s="2" t="str">
+    <x:row r="28" ht="68" customHeight="1">
+      <x:c r="A28" s="3" t="str">
         <x:v>P027</x:v>
       </x:c>
-      <x:c r="B28" s="2" t="str">
+      <x:c r="B28" s="3" t="str">
         <x:v>NXP</x:v>
       </x:c>
-      <x:c r="C28" s="2" t="str">
+      <x:c r="C28" s="3" t="str">
         <x:v>MIMXRT700-EVK</x:v>
       </x:c>
-      <x:c r="D28" s="2" t="str">
+      <x:c r="D28" s="3" t="str">
         <x:v>可采购硬件</x:v>
       </x:c>
-      <x:c r="E28" s="2" t="str">
+      <x:c r="E28" s="3" t="str">
         <x:v>官方Active商品页，2套现货、187.23美元</x:v>
       </x:c>
-      <x:c r="F28" s="11"/>
-      <x:c r="G28" s="11"/>
-      <x:c r="H28" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I28" s="2" t="str">
+      <x:c r="F28" s="4"/>
+      <x:c r="G28" s="4"/>
+      <x:c r="H28" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I28" s="3" t="str">
         <x:v>库存是检索快照；终端设计定点、销量和收入未知</x:v>
       </x:c>
-      <x:c r="J28" s="2" t="str">
+      <x:c r="J28" s="3" t="str">
         <x:v>https://www.nxp.com/design/design-center/software/development-software/mcuxpresso-software-and-tools-/i-mx-rt700-evaluation-kit:MIMXRT700-EVK</x:v>
       </x:c>
       <x:c r="K28" s="2"/>
@@ -5370,33 +5500,33 @@
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="2"/>
     </x:row>
-    <x:row r="29" ht="64" customHeight="1">
-      <x:c r="A29" s="2" t="str">
+    <x:row r="29" ht="68" customHeight="1">
+      <x:c r="A29" s="3" t="str">
         <x:v>P028</x:v>
       </x:c>
-      <x:c r="B29" s="2" t="str">
+      <x:c r="B29" s="3" t="str">
         <x:v>Synaptics</x:v>
       </x:c>
-      <x:c r="C29" s="2" t="str">
+      <x:c r="C29" s="3" t="str">
         <x:v>Astra Machina SL2610 Dev Kit</x:v>
       </x:c>
-      <x:c r="D29" s="2" t="str">
+      <x:c r="D29" s="3" t="str">
         <x:v>可采购硬件</x:v>
       </x:c>
-      <x:c r="E29" s="2" t="str">
+      <x:c r="E29" s="3" t="str">
         <x:v>官网列三家分销购买入口与完整开发文档</x:v>
       </x:c>
-      <x:c r="F29" s="11" t="n">
-        <x:v>46225</x:v>
-      </x:c>
-      <x:c r="G29" s="11"/>
-      <x:c r="H29" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I29" s="2" t="str">
+      <x:c r="F29" s="4" t="d">
+        <x:v>2026-07-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G29" s="4"/>
+      <x:c r="H29" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I29" s="3" t="str">
         <x:v>未逐家确认库存；开发套件不等于SL2610终端批量出货</x:v>
       </x:c>
-      <x:c r="J29" s="2" t="str">
+      <x:c r="J29" s="3" t="str">
         <x:v>https://www.synaptics.com/products/embedded-processors/sl2610-product-line</x:v>
       </x:c>
       <x:c r="K29" s="2"/>
@@ -5405,35 +5535,35 @@
       <x:c r="N29" s="2"/>
       <x:c r="O29" s="2"/>
     </x:row>
-    <x:row r="30" ht="64" customHeight="1">
-      <x:c r="A30" s="2" t="str">
+    <x:row r="30" ht="68" customHeight="1">
+      <x:c r="A30" s="3" t="str">
         <x:v>P029</x:v>
       </x:c>
-      <x:c r="B30" s="2" t="str">
+      <x:c r="B30" s="3" t="str">
         <x:v>Hailo</x:v>
       </x:c>
-      <x:c r="C30" s="2" t="str">
+      <x:c r="C30" s="3" t="str">
         <x:v>Hailo-10H M.2</x:v>
       </x:c>
-      <x:c r="D30" s="2" t="str">
+      <x:c r="D30" s="3" t="str">
         <x:v>可采购硬件</x:v>
       </x:c>
-      <x:c r="E30" s="2" t="str">
+      <x:c r="E30" s="3" t="str">
         <x:v>官方商业可用公告与当前商店入口</x:v>
       </x:c>
-      <x:c r="F30" s="11" t="n">
-        <x:v>45860</x:v>
-      </x:c>
-      <x:c r="G30" s="11" t="n">
-        <x:v>45860</x:v>
-      </x:c>
-      <x:c r="H30" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I30" s="2" t="str">
+      <x:c r="F30" s="4" t="d">
+        <x:v>2025-07-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G30" s="4" t="d">
+        <x:v>2025-07-22T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H30" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I30" s="3" t="str">
         <x:v>未核销量与收入；汽车SOP是目标，性能功耗为厂商基准</x:v>
       </x:c>
-      <x:c r="J30" s="2" t="str">
+      <x:c r="J30" s="3" t="str">
         <x:v>https://hailo.ai/company-overview/newsroom/news/hailo-announces-general-availability-of-hailo-10h-edge-ai-accelerator-with-generative-ai-capabilities/</x:v>
       </x:c>
       <x:c r="K30" s="2"/>
@@ -5442,31 +5572,31 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="64" customHeight="1">
-      <x:c r="A31" s="2" t="str">
+    <x:row r="31" ht="68" customHeight="1">
+      <x:c r="A31" s="3" t="str">
         <x:v>P030</x:v>
       </x:c>
-      <x:c r="B31" s="2" t="str">
+      <x:c r="B31" s="3" t="str">
         <x:v>Ambiq</x:v>
       </x:c>
-      <x:c r="C31" s="2" t="str">
+      <x:c r="C31" s="3" t="str">
         <x:v>Apollo510 EVB</x:v>
       </x:c>
-      <x:c r="D31" s="2" t="str">
+      <x:c r="D31" s="3" t="str">
         <x:v>可采购硬件</x:v>
       </x:c>
-      <x:c r="E31" s="2" t="str">
+      <x:c r="E31" s="3" t="str">
         <x:v>DigiKey 12套现货快照</x:v>
       </x:c>
-      <x:c r="F31" s="11"/>
-      <x:c r="G31" s="11"/>
-      <x:c r="H31" s="11" t="n">
-        <x:v>46297</x:v>
-      </x:c>
-      <x:c r="I31" s="2" t="str">
+      <x:c r="F31" s="4"/>
+      <x:c r="G31" s="4"/>
+      <x:c r="H31" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I31" s="3" t="str">
         <x:v>评估板现货不证明Apollo510芯片终端批量</x:v>
       </x:c>
-      <x:c r="J31" s="2" t="str">
+      <x:c r="J31" s="3" t="str">
         <x:v>https://www.digikey.com/en/products/detail/ambiq-micro-inc/AP510BEVB/28007828</x:v>
       </x:c>
       <x:c r="K31" s="2"/>
@@ -5475,7 +5605,7 @@
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="2"/>
     </x:row>
-    <x:row r="32" ht="64" customHeight="1">
+    <x:row r="32" ht="68" customHeight="1">
       <x:c r="A32" s="3" t="str">
         <x:v>P031</x:v>
       </x:c>
@@ -5491,12 +5621,12 @@
       <x:c r="E32" s="3" t="str">
         <x:v>分销SKU Active、库存0，预计2026-10-05到货约4900颗</x:v>
       </x:c>
-      <x:c r="F32" s="4" t="n">
-        <x:v>45958</x:v>
+      <x:c r="F32" s="4" t="d">
+        <x:v>2025-10-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G32" s="4"/>
-      <x:c r="H32" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H32" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
         <x:v>预计到货不是现货或已交付；批量客户与分产品收入未知</x:v>
@@ -5510,7 +5640,7 @@
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="2"/>
     </x:row>
-    <x:row r="33" ht="64" customHeight="1">
+    <x:row r="33" ht="68" customHeight="1">
       <x:c r="A33" s="3" t="str">
         <x:v>P032</x:v>
       </x:c>
@@ -5526,12 +5656,12 @@
       <x:c r="E33" s="3" t="str">
         <x:v>参投方称具备批产能力并在手机、AR/VR、电网、安防、建筑、畜牧获得批量订单</x:v>
       </x:c>
-      <x:c r="F33" s="4" t="n">
-        <x:v>46217</x:v>
+      <x:c r="F33" s="4" t="d">
+        <x:v>2026-07-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G33" s="4"/>
-      <x:c r="H33" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H33" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
         <x:v>未披露具体型号、客户、订单量、金额、交付和收入；不得直接映射为Aeveon或Speck</x:v>
@@ -5545,7 +5675,7 @@
       <x:c r="N33" s="2"/>
       <x:c r="O33" s="2"/>
     </x:row>
-    <x:row r="34" ht="64" customHeight="1">
+    <x:row r="34" ht="68" customHeight="1">
       <x:c r="A34" s="3" t="str">
         <x:v>P033</x:v>
       </x:c>
@@ -5556,20 +5686,20 @@
         <x:v>SpiNNaker2科研系统／Braunfels与莱比锡部署</x:v>
       </x:c>
       <x:c r="D34" s="3" t="str">
-        <x:v>科研部署已确认</x:v>
+        <x:v>已签公共采购合同／科研部署</x:v>
       </x:c>
       <x:c r="E34" s="3" t="str">
-        <x:v>Sandia与莱比锡大学作为使用方确认系统已到货／运行；软件公开镜像与教程可读</x:v>
-      </x:c>
-      <x:c r="F34" s="4" t="n">
-        <x:v>45812</x:v>
+        <x:v>Jülich公共采购结果确认336万欧元合同；Sandia与莱比锡大学作为使用方确认系统已到货／运行；软件公开镜像与教程可读</x:v>
+      </x:c>
+      <x:c r="F34" s="4" t="d">
+        <x:v>2025-06-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="G34" s="4"/>
-      <x:c r="H34" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H34" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>到货月份不是日；部署不是供应商收入。约400万欧元为莱比锡科研设施资助；无合同、支付、规模化训练或同任务整机实测</x:v>
+        <x:v>336万欧元是2026年2月25日合同授予值，不等于已付款或收入确认；与莱比锡约400万欧元科研设施资助分开。Jülich交付验收、收款、毛利、复购、规模化训练与同任务整机实测未知</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
         <x:v>https://www.sandia.gov/research/news/brain-based-computing-for-nuclear-deterrence-solutions/</x:v>
@@ -5580,7 +5710,7 @@
       <x:c r="N34" s="2"/>
       <x:c r="O34" s="2"/>
     </x:row>
-    <x:row r="35" ht="64" customHeight="1">
+    <x:row r="35" ht="68" customHeight="1">
       <x:c r="A35" s="3" t="str">
         <x:v>P034</x:v>
       </x:c>
@@ -5598,8 +5728,8 @@
       </x:c>
       <x:c r="F35" s="4"/>
       <x:c r="G35" s="4"/>
-      <x:c r="H35" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H35" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str">
         <x:v>页面未标发布日期；售罄不等于已核实出货、补货或终端量产。仅兼容OpenMV N6；无销量、客户、收入或世界模型训练证据</x:v>
@@ -5613,7 +5743,7 @@
       <x:c r="N35" s="2"/>
       <x:c r="O35" s="2"/>
     </x:row>
-    <x:row r="36" ht="64" customHeight="1">
+    <x:row r="36" ht="68" customHeight="1">
       <x:c r="A36" s="3" t="str">
         <x:v>P035</x:v>
       </x:c>
@@ -5630,11 +5760,11 @@
         <x:v>官方产品页明确计划2027可用；混合模拟／数字架构；Microchip确认下一代APU的memBrain／SuperFlash选型</x:v>
       </x:c>
       <x:c r="F36" s="4"/>
-      <x:c r="G36" s="4" t="n">
-        <x:v>46098</x:v>
-      </x:c>
-      <x:c r="H36" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="G36" s="4" t="d">
+        <x:v>2026-03-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H36" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str">
         <x:v>未见投片、样片、良率、价格、客户或交付；120 TOPS/W与比较倍数为厂商口径</x:v>
@@ -5648,7 +5778,7 @@
       <x:c r="N36" s="2"/>
       <x:c r="O36" s="2"/>
     </x:row>
-    <x:row r="37" ht="64" customHeight="1">
+    <x:row r="37" ht="68" customHeight="1">
       <x:c r="A37" s="3" t="str">
         <x:v>P036</x:v>
       </x:c>
@@ -5666,8 +5796,8 @@
       </x:c>
       <x:c r="F37" s="4"/>
       <x:c r="G37" s="4"/>
-      <x:c r="H37" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H37" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str">
         <x:v>M1演示不证明光电阵列与APU已完成混合键合集成；未见样片、数据表、客户或交付</x:v>
@@ -5681,7 +5811,7 @@
       <x:c r="N37" s="2"/>
       <x:c r="O37" s="2"/>
     </x:row>
-    <x:row r="38" ht="64" customHeight="1">
+    <x:row r="38" ht="68" customHeight="1">
       <x:c r="A38" s="3" t="str">
         <x:v>P037</x:v>
       </x:c>
@@ -5699,8 +5829,8 @@
       </x:c>
       <x:c r="F38" s="4"/>
       <x:c r="G38" s="4"/>
-      <x:c r="H38" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="H38" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I38" s="3" t="str">
         <x:v>未见3D NAND硅片、封装、样片或客户；100B+参数和低于1W均为公司目标</x:v>
@@ -5714,7 +5844,7 @@
       <x:c r="N38" s="2"/>
       <x:c r="O38" s="2"/>
     </x:row>
-    <x:row r="39" ht="64" customHeight="1">
+    <x:row r="39" ht="68" customHeight="1">
       <x:c r="A39" s="3" t="str">
         <x:v>P038</x:v>
       </x:c>
@@ -5730,14 +5860,14 @@
       <x:c r="E39" s="3" t="str">
         <x:v>官网产品定位＋US20260057197A1模拟MAC电路公开</x:v>
       </x:c>
-      <x:c r="F39" s="4" t="n">
-        <x:v>46079</x:v>
-      </x:c>
-      <x:c r="G39" s="4" t="n">
-        <x:v>46079</x:v>
-      </x:c>
-      <x:c r="H39" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="F39" s="4" t="d">
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G39" s="4" t="d">
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H39" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str">
         <x:v>专利不等于实现；无型号、流片、样片、制程、数据表、客户或收入</x:v>
@@ -5751,7 +5881,7 @@
       <x:c r="N39" s="2"/>
       <x:c r="O39" s="2"/>
     </x:row>
-    <x:row r="40" ht="64" customHeight="1">
+    <x:row r="40" ht="68" customHeight="1">
       <x:c r="A40" s="3" t="str">
         <x:v>P039</x:v>
       </x:c>
@@ -5767,14 +5897,14 @@
       <x:c r="E40" s="3" t="str">
         <x:v>公司一手发布＋展会现场演示报道</x:v>
       </x:c>
-      <x:c r="F40" s="4" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="G40" s="4" t="n">
-        <x:v>46219</x:v>
-      </x:c>
-      <x:c r="H40" s="4" t="n">
-        <x:v>46297</x:v>
+      <x:c r="F40" s="4" t="d">
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G40" s="4" t="d">
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H40" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="I40" s="3" t="str">
         <x:v>模型和1000小时数据集均为公司口径；未见权重、代码、统一任务成功率、公开下载或工业验收。不是SNN／芯片产品。</x:v>
@@ -6143,7 +6273,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2502f0c4f874f8c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf8c1dd5c1a47ab"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6164,25 +6294,25 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="3" t="str">
+      <x:c r="A1" t="str">
         <x:v>编号</x:v>
       </x:c>
-      <x:c r="B1" s="3" t="str">
+      <x:c r="B1" t="str">
         <x:v>事件日期</x:v>
       </x:c>
-      <x:c r="C1" s="3" t="str">
+      <x:c r="C1" t="str">
         <x:v>发布日期</x:v>
       </x:c>
-      <x:c r="D1" s="3" t="str">
+      <x:c r="D1" t="str">
         <x:v>主体</x:v>
       </x:c>
-      <x:c r="E1" s="3" t="str">
+      <x:c r="E1" t="str">
         <x:v>事件</x:v>
       </x:c>
-      <x:c r="F1" s="3" t="str">
+      <x:c r="F1" t="str">
         <x:v>证据边界</x:v>
       </x:c>
-      <x:c r="G1" s="3" t="str">
+      <x:c r="G1" t="str">
         <x:v>原始URL</x:v>
       </x:c>
       <x:c r="H1" s="2"/>
@@ -6194,26 +6324,26 @@
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
     </x:row>
-    <x:row r="2" ht="65" customHeight="1">
-      <x:c r="A2" s="3" t="str">
+    <x:row r="2" ht="66" customHeight="1">
+      <x:c r="A2" s="151" t="str">
         <x:v>T018</x:v>
       </x:c>
-      <x:c r="B2" s="4" t="str">
+      <x:c r="B2" s="152" t="str">
         <x:v>2025-03（仅月份）</x:v>
       </x:c>
-      <x:c r="C2" s="4" t="d">
+      <x:c r="C2" s="152" t="d">
         <x:v>2025-06-04T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D2" s="3" t="str">
+      <x:c r="D2" s="151" t="str">
         <x:v>Sandia／SpiNNcloud</x:v>
       </x:c>
-      <x:c r="E2" s="3" t="str">
+      <x:c r="E2" s="151" t="str">
         <x:v>Braunfels到货并完成科研部署</x:v>
       </x:c>
-      <x:c r="F2" s="3" t="str">
+      <x:c r="F2" s="151" t="str">
         <x:v>事件只确认月份；Sandia确认初始热流随机游走模拟。研究试验平台，不是终端规模量产或供应商收入</x:v>
       </x:c>
-      <x:c r="G2" s="3" t="str">
+      <x:c r="G2" s="151" t="str">
         <x:v>https://www.sandia.gov/research/news/brain-based-computing-for-nuclear-deterrence-solutions/</x:v>
       </x:c>
       <x:c r="H2" s="2"/>
@@ -6225,26 +6355,26 @@
       <x:c r="N2" s="2"/>
       <x:c r="O2" s="2"/>
     </x:row>
-    <x:row r="3" ht="65" customHeight="1">
-      <x:c r="A3" s="3" t="str">
+    <x:row r="3" ht="66" customHeight="1">
+      <x:c r="A3" s="151" t="str">
         <x:v>T012</x:v>
       </x:c>
-      <x:c r="B3" s="4" t="d">
+      <x:c r="B3" s="152" t="d">
         <x:v>2025-07-22T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C3" s="4" t="d">
+      <x:c r="C3" s="152" t="d">
         <x:v>2025-07-22T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D3" s="3" t="str">
+      <x:c r="D3" s="151" t="str">
         <x:v>Hailo</x:v>
       </x:c>
-      <x:c r="E3" s="3" t="str">
+      <x:c r="E3" s="151" t="str">
         <x:v>Hailo-10H商业可用并接受全球订单</x:v>
       </x:c>
-      <x:c r="F3" s="3" t="str">
+      <x:c r="F3" s="151" t="str">
         <x:v>厂商GA与订单入口；不等于终端设计定点、销量或收入</x:v>
       </x:c>
-      <x:c r="G3" s="3" t="str">
+      <x:c r="G3" s="151" t="str">
         <x:v>https://hailo.ai/company-overview/newsroom/news/hailo-announces-general-availability-of-hailo-10h-edge-ai-accelerator-with-generative-ai-capabilities/</x:v>
       </x:c>
       <x:c r="H3" s="2"/>
@@ -6256,26 +6386,26 @@
       <x:c r="N3" s="2"/>
       <x:c r="O3" s="2"/>
     </x:row>
-    <x:row r="4" ht="65" customHeight="1">
-      <x:c r="A4" s="3" t="str">
+    <x:row r="4" ht="66" customHeight="1">
+      <x:c r="A4" s="151" t="str">
         <x:v>T019</x:v>
       </x:c>
-      <x:c r="B4" s="4" t="str">
+      <x:c r="B4" s="152" t="str">
         <x:v>2025-10（仅月份）</x:v>
       </x:c>
-      <x:c r="C4" s="4" t="d">
+      <x:c r="C4" s="152" t="d">
         <x:v>2025-10-28T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D4" s="3" t="str">
+      <x:c r="D4" s="151" t="str">
         <x:v>莱比锡大学／SpiNNcloud</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="str">
+      <x:c r="E4" s="151" t="str">
         <x:v>类脑科研系统投入运行</x:v>
       </x:c>
-      <x:c r="F4" s="3" t="str">
+      <x:c r="F4" s="151" t="str">
         <x:v>事件只确认月份；约400万欧元为科研设施资助，不是采购额或供应商收入。药物项目采用int8 DNN，不能等同SNN片上学习</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="str">
+      <x:c r="G4" s="151" t="str">
         <x:v>https://www.uni-leipzig.de/newsdetail/artikel/vom-gehirn-inspiriert-supercomputer-staerkt-ki-forschung-an-der-universitaet-leipzig-2025-10-28</x:v>
       </x:c>
       <x:c r="H4" s="2"/>
@@ -6287,26 +6417,26 @@
       <x:c r="N4" s="2"/>
       <x:c r="O4" s="2"/>
     </x:row>
-    <x:row r="5" ht="65" customHeight="1">
-      <x:c r="A5" s="3" t="str">
+    <x:row r="5" ht="66" customHeight="1">
+      <x:c r="A5" s="151" t="str">
         <x:v>T001</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="d">
+      <x:c r="B5" s="152" t="d">
         <x:v>2026-02-04T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="d">
+      <x:c r="C5" s="152" t="d">
         <x:v>2026-02-04T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D5" s="3" t="str">
+      <x:c r="D5" s="151" t="str">
         <x:v>Honda／Mythic</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="str">
+      <x:c r="E5" s="151" t="str">
         <x:v>投资与车载SoC联合研发</x:v>
       </x:c>
-      <x:c r="F5" s="3" t="str">
+      <x:c r="F5" s="151" t="str">
         <x:v>未来联合研发，不是车型量产</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="str">
+      <x:c r="G5" s="151" t="str">
         <x:v>https://global.honda/en/topics/2026/c_2026-02-04eng.html</x:v>
       </x:c>
       <x:c r="H5" s="2"/>
@@ -6318,27 +6448,27 @@
       <x:c r="N5" s="2"/>
       <x:c r="O5" s="2"/>
     </x:row>
-    <x:row r="6" ht="65" customHeight="1">
-      <x:c r="A6" s="3" t="str">
-        <x:v>T022</x:v>
-      </x:c>
-      <x:c r="B6" s="4" t="d">
-        <x:v>2026-02-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C6" s="4" t="d">
-        <x:v>2026-02-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="str">
-        <x:v>Aspirare Semi</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="str">
-        <x:v>模拟计算电路专利申请公开</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="str">
-        <x:v>确认主体与知识产权路线，不证明ASIC实现、量产或收入</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="str">
-        <x:v>https://patents.google.com/patent/US20260057197A1/en</x:v>
+    <x:row r="6" ht="66" customHeight="1">
+      <x:c r="A6" s="151" t="str">
+        <x:v>T026</x:v>
+      </x:c>
+      <x:c r="B6" s="152" t="d">
+        <x:v>2026-02-25T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C6" s="152" t="d">
+        <x:v>2026-03-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D6" s="151" t="str">
+        <x:v>Forschungszentrum Jülich／SpiNNcloud</x:v>
+      </x:c>
+      <x:c r="E6" s="151" t="str">
+        <x:v>336万欧元SpiNNaker2公共采购合同签订</x:v>
+      </x:c>
+      <x:c r="F6" s="151" t="str">
+        <x:v>公共采购结果确认合同授予值、数量1套、单一投标且无分包；合同不等于已付款、交付验收或当期收入确认</x:v>
+      </x:c>
+      <x:c r="G6" s="151" t="str">
+        <x:v>https://ted.europa.eu/en/notice/-/detail/141500-2026</x:v>
       </x:c>
       <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
@@ -6349,27 +6479,27 @@
       <x:c r="N6" s="2"/>
       <x:c r="O6" s="2"/>
     </x:row>
-    <x:row r="7" ht="65" customHeight="1">
-      <x:c r="A7" s="3" t="str">
-        <x:v>T002</x:v>
-      </x:c>
-      <x:c r="B7" s="4" t="d">
-        <x:v>2026-03-12T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C7" s="4" t="d">
-        <x:v>2026-03-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D7" s="3" t="str">
-        <x:v>Innatera／Joya</x:v>
-      </x:c>
-      <x:c r="E7" s="3" t="str">
-        <x:v>EdgeCore模块发布</x:v>
-      </x:c>
-      <x:c r="F7" s="3" t="str">
-        <x:v>可集成客户模块，销量未知</x:v>
-      </x:c>
-      <x:c r="G7" s="3" t="str">
-        <x:v>https://www.innatera.com/newsroom/joya-design-takes-neuromorphic-chip-from-design-to-device-with-first-innatera-powered-consumer-audio-product-at-awe-china/</x:v>
+    <x:row r="7" ht="66" customHeight="1">
+      <x:c r="A7" s="151" t="str">
+        <x:v>T022</x:v>
+      </x:c>
+      <x:c r="B7" s="152" t="d">
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C7" s="152" t="d">
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D7" s="151" t="str">
+        <x:v>Aspirare Semi</x:v>
+      </x:c>
+      <x:c r="E7" s="151" t="str">
+        <x:v>模拟计算电路专利申请公开</x:v>
+      </x:c>
+      <x:c r="F7" s="151" t="str">
+        <x:v>确认主体与知识产权路线，不证明ASIC实现、量产或收入</x:v>
+      </x:c>
+      <x:c r="G7" s="151" t="str">
+        <x:v>https://patents.google.com/patent/US20260057197A1/en</x:v>
       </x:c>
       <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
@@ -6380,27 +6510,27 @@
       <x:c r="N7" s="2"/>
       <x:c r="O7" s="2"/>
     </x:row>
-    <x:row r="8" ht="65" customHeight="1">
-      <x:c r="A8" s="3" t="str">
-        <x:v>T021</x:v>
-      </x:c>
-      <x:c r="B8" s="4" t="d">
-        <x:v>2026-03-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C8" s="4" t="d">
-        <x:v>2026-03-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="str">
-        <x:v>Mythic／Microchip SST</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="str">
-        <x:v>下一代APU选择memBrain／SuperFlash</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="str">
-        <x:v>供应链／IP选型，不证明Vanguard流片、样片或交付；能效数字为厂商宣称</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="str">
-        <x:v>https://www.microchip.com/en-us/about/news-releases/products/mythic-selects-membrain-technology-from-sst-for-its-next-gen-ultra-low-power-apus</x:v>
+    <x:row r="8" ht="66" customHeight="1">
+      <x:c r="A8" s="151" t="str">
+        <x:v>T002</x:v>
+      </x:c>
+      <x:c r="B8" s="152" t="d">
+        <x:v>2026-03-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C8" s="152" t="d">
+        <x:v>2026-03-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D8" s="151" t="str">
+        <x:v>Innatera／Joya</x:v>
+      </x:c>
+      <x:c r="E8" s="151" t="str">
+        <x:v>EdgeCore模块发布</x:v>
+      </x:c>
+      <x:c r="F8" s="151" t="str">
+        <x:v>可集成客户模块，销量未知</x:v>
+      </x:c>
+      <x:c r="G8" s="151" t="str">
+        <x:v>https://www.innatera.com/newsroom/joya-design-takes-neuromorphic-chip-from-design-to-device-with-first-innatera-powered-consumer-audio-product-at-awe-china/</x:v>
       </x:c>
       <x:c r="H8" s="2"/>
       <x:c r="I8" s="2"/>
@@ -6411,25 +6541,27 @@
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="2"/>
     </x:row>
-    <x:row r="9" ht="65" customHeight="1">
-      <x:c r="A9" s="3" t="str">
-        <x:v>T025</x:v>
-      </x:c>
-      <x:c r="B9" s="4" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C9" s="4"/>
-      <x:c r="D9" s="3" t="str">
-        <x:v>Intel／Lava</x:v>
-      </x:c>
-      <x:c r="E9" s="3" t="str">
-        <x:v>官方仓库归档、只读；下一代Loihi与新SDK在开发</x:v>
-      </x:c>
-      <x:c r="F9" s="3" t="str">
-        <x:v>归档日期可核；README发布日期未知。新SDK为路线，未证明交付、量产或退出研究。</x:v>
-      </x:c>
-      <x:c r="G9" s="3" t="str">
-        <x:v>https://github.com/lava-nc/lava</x:v>
+    <x:row r="9" ht="66" customHeight="1">
+      <x:c r="A9" s="151" t="str">
+        <x:v>T021</x:v>
+      </x:c>
+      <x:c r="B9" s="152" t="d">
+        <x:v>2026-03-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C9" s="152" t="d">
+        <x:v>2026-03-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D9" s="151" t="str">
+        <x:v>Mythic／Microchip SST</x:v>
+      </x:c>
+      <x:c r="E9" s="151" t="str">
+        <x:v>下一代APU选择memBrain／SuperFlash</x:v>
+      </x:c>
+      <x:c r="F9" s="151" t="str">
+        <x:v>供应链／IP选型，不证明Vanguard流片、样片或交付；能效数字为厂商宣称</x:v>
+      </x:c>
+      <x:c r="G9" s="151" t="str">
+        <x:v>https://www.microchip.com/en-us/about/news-releases/products/mythic-selects-membrain-technology-from-sst-for-its-next-gen-ultra-low-power-apus</x:v>
       </x:c>
       <x:c r="H9" s="2"/>
       <x:c r="I9" s="2"/>
@@ -6440,27 +6572,25 @@
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="2"/>
     </x:row>
-    <x:row r="10" ht="65" customHeight="1">
-      <x:c r="A10" s="3" t="str">
-        <x:v>T003</x:v>
-      </x:c>
-      <x:c r="B10" s="4" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C10" s="4" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D10" s="3" t="str">
-        <x:v>Mythic</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="str">
-        <x:v>收购Videantis</x:v>
-      </x:c>
-      <x:c r="F10" s="3" t="str">
-        <x:v>被收购数字IP装机不计作模拟APU销量</x:v>
-      </x:c>
-      <x:c r="G10" s="3" t="str">
-        <x:v>https://www.mythic.ai/newsroom/Blog%20Post%20Title%20One-3zaa9-zlxng-67tfc-lbgbx</x:v>
+    <x:row r="10" ht="66" customHeight="1">
+      <x:c r="A10" s="151" t="str">
+        <x:v>T025</x:v>
+      </x:c>
+      <x:c r="B10" s="152" t="d">
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C10" s="152"/>
+      <x:c r="D10" s="151" t="str">
+        <x:v>Intel／Lava</x:v>
+      </x:c>
+      <x:c r="E10" s="151" t="str">
+        <x:v>官方仓库归档、只读；下一代Loihi与新SDK在开发</x:v>
+      </x:c>
+      <x:c r="F10" s="151" t="str">
+        <x:v>归档日期可核；README发布日期未知。新SDK为路线，未证明交付、量产或退出研究。</x:v>
+      </x:c>
+      <x:c r="G10" s="151" t="str">
+        <x:v>https://github.com/lava-nc/lava</x:v>
       </x:c>
       <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
@@ -6471,27 +6601,27 @@
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
     </x:row>
-    <x:row r="11" ht="65" customHeight="1">
-      <x:c r="A11" s="3" t="str">
-        <x:v>T013</x:v>
-      </x:c>
-      <x:c r="B11" s="4" t="d">
+    <x:row r="11" ht="66" customHeight="1">
+      <x:c r="A11" s="151" t="str">
+        <x:v>T003</x:v>
+      </x:c>
+      <x:c r="B11" s="152" t="d">
         <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C11" s="4" t="d">
+      <x:c r="C11" s="152" t="d">
         <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="D11" s="3" t="str">
-        <x:v>BrainChip／ASICLAND</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="str">
-        <x:v>签署Akida IP分销许可</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="str">
-        <x:v>可做评估许可和MPW；客户生产许可需BrainChip另批并支付生产许可费，未披露金额或已确认收入</x:v>
-      </x:c>
-      <x:c r="G11" s="3" t="str">
-        <x:v>https://brainchip.com/press/brainchip-strikes-ip-licensing-deal-with-asicland/</x:v>
+      <x:c r="D11" s="151" t="str">
+        <x:v>Mythic</x:v>
+      </x:c>
+      <x:c r="E11" s="151" t="str">
+        <x:v>收购Videantis</x:v>
+      </x:c>
+      <x:c r="F11" s="151" t="str">
+        <x:v>被收购数字IP装机不计作模拟APU销量</x:v>
+      </x:c>
+      <x:c r="G11" s="151" t="str">
+        <x:v>https://www.mythic.ai/newsroom/Blog%20Post%20Title%20One-3zaa9-zlxng-67tfc-lbgbx</x:v>
       </x:c>
       <x:c r="H11" s="2"/>
       <x:c r="I11" s="2"/>
@@ -6502,27 +6632,27 @@
       <x:c r="N11" s="2"/>
       <x:c r="O11" s="2"/>
     </x:row>
-    <x:row r="12" ht="65" customHeight="1">
-      <x:c r="A12" s="3" t="str">
-        <x:v>T004</x:v>
-      </x:c>
-      <x:c r="B12" s="4" t="d">
-        <x:v>2026-06-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C12" s="4" t="d">
-        <x:v>2026-06-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="str">
-        <x:v>Prophesee</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="str">
-        <x:v>Mantara／Hearth发布</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="str">
-        <x:v>厂商现场验证与软件迁移公告</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="str">
-        <x:v>https://www.prophesee.ai/2026/06/15/prophesee-launches-mantara-event-based-drone-detection/</x:v>
+    <x:row r="12" ht="66" customHeight="1">
+      <x:c r="A12" s="151" t="str">
+        <x:v>T013</x:v>
+      </x:c>
+      <x:c r="B12" s="152" t="d">
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C12" s="152" t="d">
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D12" s="151" t="str">
+        <x:v>BrainChip／ASICLAND</x:v>
+      </x:c>
+      <x:c r="E12" s="151" t="str">
+        <x:v>签署Akida IP分销许可</x:v>
+      </x:c>
+      <x:c r="F12" s="151" t="str">
+        <x:v>可做评估许可和MPW；客户生产许可需BrainChip另批并支付生产许可费，未披露金额或已确认收入</x:v>
+      </x:c>
+      <x:c r="G12" s="151" t="str">
+        <x:v>https://brainchip.com/press/brainchip-strikes-ip-licensing-deal-with-asicland/</x:v>
       </x:c>
       <x:c r="H12" s="2"/>
       <x:c r="I12" s="2"/>
@@ -6533,27 +6663,27 @@
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="2"/>
     </x:row>
-    <x:row r="13" ht="65" customHeight="1">
-      <x:c r="A13" s="3" t="str">
-        <x:v>T005</x:v>
-      </x:c>
-      <x:c r="B13" s="4" t="d">
-        <x:v>2026-06-29T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C13" s="4" t="d">
-        <x:v>2026-06-29T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D13" s="3" t="str">
-        <x:v>Innatera</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="str">
-        <x:v>Synfire 0.0.2 Beta发布</x:v>
-      </x:c>
-      <x:c r="F13" s="3" t="str">
-        <x:v>可安装，生产部署未知</x:v>
-      </x:c>
-      <x:c r="G13" s="3" t="str">
-        <x:v>https://pypi.org/project/synfire/</x:v>
+    <x:row r="13" ht="66" customHeight="1">
+      <x:c r="A13" s="151" t="str">
+        <x:v>T004</x:v>
+      </x:c>
+      <x:c r="B13" s="152" t="d">
+        <x:v>2026-06-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C13" s="152" t="d">
+        <x:v>2026-06-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D13" s="151" t="str">
+        <x:v>Prophesee</x:v>
+      </x:c>
+      <x:c r="E13" s="151" t="str">
+        <x:v>Mantara／Hearth发布</x:v>
+      </x:c>
+      <x:c r="F13" s="151" t="str">
+        <x:v>厂商现场验证与软件迁移公告</x:v>
+      </x:c>
+      <x:c r="G13" s="151" t="str">
+        <x:v>https://www.prophesee.ai/2026/06/15/prophesee-launches-mantara-event-based-drone-detection/</x:v>
       </x:c>
       <x:c r="H13" s="2"/>
       <x:c r="I13" s="2"/>
@@ -6564,27 +6694,27 @@
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="2"/>
     </x:row>
-    <x:row r="14" ht="65" customHeight="1">
-      <x:c r="A14" s="2" t="str">
-        <x:v>T023</x:v>
-      </x:c>
-      <x:c r="B14" s="11" t="d">
-        <x:v>2026-07-16T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C14" s="11" t="d">
-        <x:v>2026-07-16T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D14" s="2" t="str">
-        <x:v>千觉机器人</x:v>
-      </x:c>
-      <x:c r="E14" s="2" t="str">
-        <x:v>发布X-TouchMind V1与TacVerse 1k</x:v>
-      </x:c>
-      <x:c r="F14" s="2" t="str">
-        <x:v>公司发布与展会演示；数据下载、权重、客户验收和收入未核</x:v>
-      </x:c>
-      <x:c r="G14" s="2" t="str">
-        <x:v>https://www.xenserobotics.com/article/387/detail/25</x:v>
+    <x:row r="14" ht="66" customHeight="1">
+      <x:c r="A14" s="151" t="str">
+        <x:v>T005</x:v>
+      </x:c>
+      <x:c r="B14" s="152" t="d">
+        <x:v>2026-06-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C14" s="152" t="d">
+        <x:v>2026-06-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D14" s="151" t="str">
+        <x:v>Innatera</x:v>
+      </x:c>
+      <x:c r="E14" s="151" t="str">
+        <x:v>Synfire 0.0.2 Beta发布</x:v>
+      </x:c>
+      <x:c r="F14" s="151" t="str">
+        <x:v>可安装，生产部署未知</x:v>
+      </x:c>
+      <x:c r="G14" s="151" t="str">
+        <x:v>https://pypi.org/project/synfire/</x:v>
       </x:c>
       <x:c r="H14" s="2"/>
       <x:c r="I14" s="2"/>
@@ -6595,27 +6725,27 @@
       <x:c r="N14" s="2"/>
       <x:c r="O14" s="2"/>
     </x:row>
-    <x:row r="15" ht="65" customHeight="1">
-      <x:c r="A15" s="2" t="str">
-        <x:v>T010</x:v>
-      </x:c>
-      <x:c r="B15" s="11" t="d">
-        <x:v>2026-07-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C15" s="11" t="d">
-        <x:v>2026-07-17T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D15" s="2" t="str">
-        <x:v>他山科技</x:v>
-      </x:c>
-      <x:c r="E15" s="2" t="str">
-        <x:v>E10A动态触觉芯片公开发布／演示</x:v>
-      </x:c>
-      <x:c r="F15" s="2" t="str">
-        <x:v>ASC转换为厂商披露，E10A量产未知</x:v>
-      </x:c>
-      <x:c r="G15" s="2" t="str">
-        <x:v>https://www3.xinhuanet.com/tech/20260717/d66a7bb7dcf8414baeab73d6499b785e/c.html</x:v>
+    <x:row r="15" ht="66" customHeight="1">
+      <x:c r="A15" s="151" t="str">
+        <x:v>T023</x:v>
+      </x:c>
+      <x:c r="B15" s="152" t="d">
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C15" s="152" t="d">
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D15" s="151" t="str">
+        <x:v>千觉机器人</x:v>
+      </x:c>
+      <x:c r="E15" s="151" t="str">
+        <x:v>发布X-TouchMind V1与TacVerse 1k</x:v>
+      </x:c>
+      <x:c r="F15" s="151" t="str">
+        <x:v>公司发布与展会演示；数据下载、权重、客户验收和收入未核</x:v>
+      </x:c>
+      <x:c r="G15" s="151" t="str">
+        <x:v>https://www.xenserobotics.com/article/387/detail/25</x:v>
       </x:c>
       <x:c r="H15" s="2"/>
       <x:c r="I15" s="2"/>
@@ -6626,27 +6756,27 @@
       <x:c r="N15" s="2"/>
       <x:c r="O15" s="2"/>
     </x:row>
-    <x:row r="16" ht="65" customHeight="1">
-      <x:c r="A16" s="63" t="str">
-        <x:v>T015</x:v>
-      </x:c>
-      <x:c r="B16" s="85" t="d">
-        <x:v>2026-07-21T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C16" s="85" t="d">
-        <x:v>2026-07-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D16" s="64" t="str">
-        <x:v>World Labs／SceniX</x:v>
-      </x:c>
-      <x:c r="E16" s="64" t="str">
-        <x:v>World Labs收购机器人仿真公司SceniX</x:v>
-      </x:c>
-      <x:c r="F16" s="64" t="str">
-        <x:v>World Labs称SceniX R2S2R把真实任务转为可控仿真用于策略训练和评估；结果为公司展示，未独立复现，未披露交易金额或客户收入</x:v>
-      </x:c>
-      <x:c r="G16" s="64" t="str">
-        <x:v>https://www.worldlabs.ai/blog/real-to-sim-to-real</x:v>
+    <x:row r="16" ht="66" customHeight="1">
+      <x:c r="A16" s="151" t="str">
+        <x:v>T010</x:v>
+      </x:c>
+      <x:c r="B16" s="152" t="d">
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C16" s="152" t="d">
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D16" s="151" t="str">
+        <x:v>他山科技</x:v>
+      </x:c>
+      <x:c r="E16" s="151" t="str">
+        <x:v>E10A动态触觉芯片公开发布／演示</x:v>
+      </x:c>
+      <x:c r="F16" s="151" t="str">
+        <x:v>ASC转换为厂商披露，E10A量产未知</x:v>
+      </x:c>
+      <x:c r="G16" s="151" t="str">
+        <x:v>https://www3.xinhuanet.com/tech/20260717/d66a7bb7dcf8414baeab73d6499b785e/c.html</x:v>
       </x:c>
       <x:c r="H16" s="64"/>
       <x:c r="I16" s="65"/>
@@ -6657,27 +6787,27 @@
       <x:c r="N16" s="2"/>
       <x:c r="O16" s="2"/>
     </x:row>
-    <x:row r="17" ht="65" customHeight="1">
-      <x:c r="A17" s="66" t="str">
-        <x:v>T006</x:v>
-      </x:c>
-      <x:c r="B17" s="72" t="d">
+    <x:row r="17" ht="66" customHeight="1">
+      <x:c r="A17" s="151" t="str">
+        <x:v>T015</x:v>
+      </x:c>
+      <x:c r="B17" s="152" t="d">
+        <x:v>2026-07-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C17" s="152" t="d">
         <x:v>2026-07-28T00:00:00.000Z</x:v>
       </x:c>
-      <x:c r="C17" s="72" t="d">
-        <x:v>2026-07-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D17" s="67" t="str">
-        <x:v>BrainChip</x:v>
-      </x:c>
-      <x:c r="E17" s="67" t="str">
-        <x:v>AKD1500 M.2模块可购</x:v>
-      </x:c>
-      <x:c r="F17" s="67" t="str">
-        <x:v>开发模块，不等于终端销量</x:v>
-      </x:c>
-      <x:c r="G17" s="67" t="str">
-        <x:v>https://investor.brainchip.com/press/brainchip-akd1500-now-available-in-compact-m-2-form-factor-enabling-fanless-edge-ai-in-industrial-and-commercial-designs/</x:v>
+      <x:c r="D17" s="151" t="str">
+        <x:v>World Labs／SceniX</x:v>
+      </x:c>
+      <x:c r="E17" s="151" t="str">
+        <x:v>World Labs收购机器人仿真公司SceniX</x:v>
+      </x:c>
+      <x:c r="F17" s="151" t="str">
+        <x:v>World Labs称SceniX R2S2R把真实任务转为可控仿真用于策略训练和评估；结果为公司展示，未独立复现，未披露交易金额或客户收入</x:v>
+      </x:c>
+      <x:c r="G17" s="151" t="str">
+        <x:v>https://www.worldlabs.ai/blog/real-to-sim-to-real</x:v>
       </x:c>
       <x:c r="H17" s="67"/>
       <x:c r="I17" s="68"/>
@@ -6688,27 +6818,27 @@
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
     </x:row>
-    <x:row r="18" ht="65" customHeight="1">
-      <x:c r="A18" s="76" t="str">
-        <x:v>T014</x:v>
-      </x:c>
-      <x:c r="B18" s="121" t="d">
-        <x:v>2026-08-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C18" s="121" t="d">
-        <x:v>2026-08-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D18" s="77" t="str">
-        <x:v>BrainChip／Orama.AOI</x:v>
-      </x:c>
-      <x:c r="E18" s="67" t="str">
-        <x:v>发布工业检测参考部署合作</x:v>
-      </x:c>
-      <x:c r="F18" s="67" t="str">
-        <x:v>伙伴称已优化模型并形成参考部署／生产就绪方案；未披露终端工厂、采购额、出货量或收入</x:v>
-      </x:c>
-      <x:c r="G18" s="67" t="str">
-        <x:v>https://brainchip.com/press/brainchip-partners-with-orama-aoi-for-ai-fueled-defect-detection/</x:v>
+    <x:row r="18" ht="66" customHeight="1">
+      <x:c r="A18" s="151" t="str">
+        <x:v>T006</x:v>
+      </x:c>
+      <x:c r="B18" s="152" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C18" s="152" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D18" s="151" t="str">
+        <x:v>BrainChip</x:v>
+      </x:c>
+      <x:c r="E18" s="151" t="str">
+        <x:v>AKD1500 M.2模块可购</x:v>
+      </x:c>
+      <x:c r="F18" s="151" t="str">
+        <x:v>开发模块，不等于终端销量</x:v>
+      </x:c>
+      <x:c r="G18" s="151" t="str">
+        <x:v>https://investor.brainchip.com/press/brainchip-akd1500-now-available-in-compact-m-2-form-factor-enabling-fanless-edge-ai-in-industrial-and-commercial-designs/</x:v>
       </x:c>
       <x:c r="H18" s="67"/>
       <x:c r="I18" s="68"/>
@@ -6719,25 +6849,27 @@
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="2"/>
     </x:row>
-    <x:row r="19" ht="65" customHeight="1">
-      <x:c r="A19" s="76" t="str">
-        <x:v>T024</x:v>
-      </x:c>
-      <x:c r="B19" s="121"/>
-      <x:c r="C19" s="121" t="d">
-        <x:v>2026-08-24T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D19" s="77" t="str">
-        <x:v>他山科技／E10A</x:v>
-      </x:c>
-      <x:c r="E19" s="67" t="str">
-        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
-      </x:c>
-      <x:c r="F19" s="67" t="str">
-        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
-      </x:c>
-      <x:c r="G19" s="67" t="str">
-        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
+    <x:row r="19" ht="66" customHeight="1">
+      <x:c r="A19" s="151" t="str">
+        <x:v>T014</x:v>
+      </x:c>
+      <x:c r="B19" s="152" t="d">
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C19" s="152" t="d">
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D19" s="151" t="str">
+        <x:v>BrainChip／Orama.AOI</x:v>
+      </x:c>
+      <x:c r="E19" s="151" t="str">
+        <x:v>发布工业检测参考部署合作</x:v>
+      </x:c>
+      <x:c r="F19" s="151" t="str">
+        <x:v>伙伴称已优化模型并形成参考部署／生产就绪方案；未披露终端工厂、采购额、出货量或收入</x:v>
+      </x:c>
+      <x:c r="G19" s="151" t="str">
+        <x:v>https://brainchip.com/press/brainchip-partners-with-orama-aoi-for-ai-fueled-defect-detection/</x:v>
       </x:c>
       <x:c r="H19" s="67"/>
       <x:c r="I19" s="68"/>
@@ -6748,25 +6880,25 @@
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="2"/>
     </x:row>
-    <x:row r="20" ht="65" customHeight="1">
-      <x:c r="A20" s="102" t="str">
-        <x:v>T011</x:v>
-      </x:c>
-      <x:c r="B20" s="123"/>
-      <x:c r="C20" s="123" t="d">
-        <x:v>2026-08-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D20" s="104" t="str">
-        <x:v>奥比中光／他山</x:v>
-      </x:c>
-      <x:c r="E20" s="80" t="str">
-        <x:v>TS-ECHO视触无本体数采合作</x:v>
-      </x:c>
-      <x:c r="F20" s="80" t="str">
-        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
-      </x:c>
-      <x:c r="G20" s="80" t="str">
-        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
+    <x:row r="20" ht="66" customHeight="1">
+      <x:c r="A20" s="151" t="str">
+        <x:v>T024</x:v>
+      </x:c>
+      <x:c r="B20" s="152"/>
+      <x:c r="C20" s="152" t="d">
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D20" s="151" t="str">
+        <x:v>他山科技／E10A</x:v>
+      </x:c>
+      <x:c r="E20" s="151" t="str">
+        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
+      </x:c>
+      <x:c r="F20" s="151" t="str">
+        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
+      </x:c>
+      <x:c r="G20" s="151" t="str">
+        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
       </x:c>
       <x:c r="H20" s="67"/>
       <x:c r="I20" s="68"/>
@@ -6777,27 +6909,25 @@
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="2"/>
     </x:row>
-    <x:row r="21" ht="65" customHeight="1">
-      <x:c r="A21" s="116" t="str">
-        <x:v>T007</x:v>
-      </x:c>
-      <x:c r="B21" s="124" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C21" s="124" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D21" s="118" t="str">
-        <x:v>MemryX／Express LUCK</x:v>
-      </x:c>
-      <x:c r="E21" s="80" t="str">
-        <x:v>生产线部署</x:v>
-      </x:c>
-      <x:c r="F21" s="80" t="str">
-        <x:v>具名部署联合稿，采购金额未知</x:v>
-      </x:c>
-      <x:c r="G21" s="80" t="str">
-        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
+    <x:row r="21" ht="66" customHeight="1">
+      <x:c r="A21" s="151" t="str">
+        <x:v>T011</x:v>
+      </x:c>
+      <x:c r="B21" s="152"/>
+      <x:c r="C21" s="152" t="d">
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D21" s="151" t="str">
+        <x:v>奥比中光／他山</x:v>
+      </x:c>
+      <x:c r="E21" s="151" t="str">
+        <x:v>TS-ECHO视触无本体数采合作</x:v>
+      </x:c>
+      <x:c r="F21" s="151" t="str">
+        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
+      </x:c>
+      <x:c r="G21" s="151" t="str">
+        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
       </x:c>
       <x:c r="H21" s="67"/>
       <x:c r="I21" s="68"/>
@@ -6808,27 +6938,27 @@
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="2"/>
     </x:row>
-    <x:row r="22" ht="65" customHeight="1">
-      <x:c r="A22" s="78" t="str">
-        <x:v>T017</x:v>
-      </x:c>
-      <x:c r="B22" s="83" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C22" s="83" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D22" s="80" t="str">
-        <x:v>具脑磐石 EBKernel</x:v>
-      </x:c>
-      <x:c r="E22" s="80" t="str">
-        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
-      </x:c>
-      <x:c r="F22" s="80" t="str">
-        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
-      </x:c>
-      <x:c r="G22" s="80" t="str">
-        <x:v>https://www.ebkernel.com/</x:v>
+    <x:row r="22" ht="66" customHeight="1">
+      <x:c r="A22" s="151" t="str">
+        <x:v>T027</x:v>
+      </x:c>
+      <x:c r="B22" s="152" t="str">
+        <x:v>2026-08（仅月份）</x:v>
+      </x:c>
+      <x:c r="C22" s="152" t="d">
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D22" s="151" t="str">
+        <x:v>维泛智能</x:v>
+      </x:c>
+      <x:c r="E22" s="151" t="str">
+        <x:v>披露过亿元种子+轮融资</x:v>
+      </x:c>
+      <x:c r="F22" s="151" t="str">
+        <x:v>据公司向钛媒体披露；与2026年5月数亿元种子轮分开。融资拟用于量产芯片、BrainOS与OmniRT产品化，不等于收入、量产或客户付款</x:v>
+      </x:c>
+      <x:c r="G22" s="151" t="str">
+        <x:v>https://www.tmtpost.com/8113528.html</x:v>
       </x:c>
       <x:c r="H22" s="67"/>
       <x:c r="I22" s="68"/>
@@ -6839,27 +6969,27 @@
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="2"/>
     </x:row>
-    <x:row r="23" ht="65" customHeight="1">
-      <x:c r="A23" s="78" t="str">
-        <x:v>T008</x:v>
-      </x:c>
-      <x:c r="B23" s="83" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C23" s="83" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D23" s="80" t="str">
-        <x:v>AnalogAI</x:v>
-      </x:c>
-      <x:c r="E23" s="80" t="str">
-        <x:v>选用SST memBrain SAGE IP</x:v>
-      </x:c>
-      <x:c r="F23" s="80" t="str">
-        <x:v>IP选型，无流片证据</x:v>
-      </x:c>
-      <x:c r="G23" s="80" t="str">
-        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
+    <x:row r="23" ht="66" customHeight="1">
+      <x:c r="A23" s="151" t="str">
+        <x:v>T007</x:v>
+      </x:c>
+      <x:c r="B23" s="152" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C23" s="152" t="d">
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D23" s="151" t="str">
+        <x:v>MemryX／Express LUCK</x:v>
+      </x:c>
+      <x:c r="E23" s="151" t="str">
+        <x:v>生产线部署</x:v>
+      </x:c>
+      <x:c r="F23" s="151" t="str">
+        <x:v>具名部署联合稿，采购金额未知</x:v>
+      </x:c>
+      <x:c r="G23" s="151" t="str">
+        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
       </x:c>
       <x:c r="H23" s="67"/>
       <x:c r="I23" s="68"/>
@@ -6870,25 +7000,27 @@
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="2"/>
     </x:row>
-    <x:row r="24" ht="65" customHeight="1">
-      <x:c r="A24" s="78" t="str">
-        <x:v>T020</x:v>
-      </x:c>
-      <x:c r="B24" s="83" t="d">
-        <x:v>2026-09-23T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C24" s="83"/>
-      <x:c r="D24" s="80" t="str">
-        <x:v>SpiNNcloud／py-spinnaker2</x:v>
-      </x:c>
-      <x:c r="E24" s="80" t="str">
-        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
-      </x:c>
-      <x:c r="F24" s="80" t="str">
-        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
-      </x:c>
-      <x:c r="G24" s="80" t="str">
-        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
+    <x:row r="24" ht="66" customHeight="1">
+      <x:c r="A24" s="151" t="str">
+        <x:v>T017</x:v>
+      </x:c>
+      <x:c r="B24" s="152" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C24" s="152" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D24" s="151" t="str">
+        <x:v>具脑磐石 EBKernel</x:v>
+      </x:c>
+      <x:c r="E24" s="151" t="str">
+        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
+      </x:c>
+      <x:c r="F24" s="151" t="str">
+        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
+      </x:c>
+      <x:c r="G24" s="151" t="str">
+        <x:v>https://www.ebkernel.com/</x:v>
       </x:c>
       <x:c r="H24" s="67"/>
       <x:c r="I24" s="68"/>
@@ -6899,27 +7031,27 @@
       <x:c r="N24" s="2"/>
       <x:c r="O24" s="2"/>
     </x:row>
-    <x:row r="25" ht="65" customHeight="1">
-      <x:c r="A25" s="76" t="str">
-        <x:v>T016</x:v>
-      </x:c>
-      <x:c r="B25" s="121" t="d">
-        <x:v>2026-09-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C25" s="121" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D25" s="77" t="str">
-        <x:v>AMD／World Labs</x:v>
-      </x:c>
-      <x:c r="E25" s="80" t="str">
-        <x:v>签署约82亿美元全股票收购协议</x:v>
-      </x:c>
-      <x:c r="F25" s="80" t="str">
-        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
-      </x:c>
-      <x:c r="G25" s="80" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
+    <x:row r="25" ht="66" customHeight="1">
+      <x:c r="A25" s="151" t="str">
+        <x:v>T008</x:v>
+      </x:c>
+      <x:c r="B25" s="152" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C25" s="152" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D25" s="151" t="str">
+        <x:v>AnalogAI</x:v>
+      </x:c>
+      <x:c r="E25" s="151" t="str">
+        <x:v>选用SST memBrain SAGE IP</x:v>
+      </x:c>
+      <x:c r="F25" s="151" t="str">
+        <x:v>IP选型，无流片证据</x:v>
+      </x:c>
+      <x:c r="G25" s="151" t="str">
+        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
       </x:c>
       <x:c r="H25" s="67"/>
       <x:c r="I25" s="68"/>
@@ -6930,27 +7062,25 @@
       <x:c r="N25" s="2"/>
       <x:c r="O25" s="2"/>
     </x:row>
-    <x:row r="26" ht="100" customHeight="1">
-      <x:c r="A26" s="78" t="str">
-        <x:v>T009</x:v>
-      </x:c>
-      <x:c r="B26" s="83" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C26" s="83" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="D26" s="80" t="str">
-        <x:v>POLYN</x:v>
-      </x:c>
-      <x:c r="E26" s="80" t="str">
-        <x:v>TMS工程节点供客户评估</x:v>
-      </x:c>
-      <x:c r="F26" s="80" t="str">
-        <x:v>未具名评估方，非量产</x:v>
-      </x:c>
-      <x:c r="G26" s="80" t="str">
-        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+    <x:row r="26" ht="66" customHeight="1">
+      <x:c r="A26" s="151" t="str">
+        <x:v>T020</x:v>
+      </x:c>
+      <x:c r="B26" s="152" t="d">
+        <x:v>2026-09-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C26" s="152"/>
+      <x:c r="D26" s="151" t="str">
+        <x:v>SpiNNcloud／py-spinnaker2</x:v>
+      </x:c>
+      <x:c r="E26" s="151" t="str">
+        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
+      </x:c>
+      <x:c r="F26" s="151" t="str">
+        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
+      </x:c>
+      <x:c r="G26" s="151" t="str">
+        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
       </x:c>
       <x:c r="H26" s="67"/>
       <x:c r="I26" s="68"/>
@@ -6961,16 +7091,28 @@
       <x:c r="N26" s="2"/>
       <x:c r="O26" s="2"/>
     </x:row>
-    <x:row r="27" ht="28" customHeight="1">
-      <x:c r="A27" s="116" t="str">
-        <x:v>半年收入</x:v>
-      </x:c>
-      <x:c r="B27" s="117"/>
-      <x:c r="C27" s="117"/>
-      <x:c r="D27" s="118"/>
-      <x:c r="E27" s="80"/>
-      <x:c r="F27" s="80"/>
-      <x:c r="G27" s="80"/>
+    <x:row r="27" ht="66" customHeight="1">
+      <x:c r="A27" s="151" t="str">
+        <x:v>T016</x:v>
+      </x:c>
+      <x:c r="B27" s="152" t="d">
+        <x:v>2026-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C27" s="152" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D27" s="151" t="str">
+        <x:v>AMD／World Labs</x:v>
+      </x:c>
+      <x:c r="E27" s="151" t="str">
+        <x:v>签署约82亿美元全股票收购协议</x:v>
+      </x:c>
+      <x:c r="F27" s="151" t="str">
+        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
+      </x:c>
+      <x:c r="G27" s="151" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
+      </x:c>
       <x:c r="H27" s="67"/>
       <x:c r="I27" s="68"/>
       <x:c r="J27" s="2"/>
@@ -6980,22 +7122,28 @@
       <x:c r="N27" s="2"/>
       <x:c r="O27" s="2"/>
     </x:row>
-    <x:row r="28" ht="30" customHeight="1">
-      <x:c r="A28" s="78" t="str">
-        <x:v>构成</x:v>
-      </x:c>
-      <x:c r="B28" s="79" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C28" s="79" t="str">
-        <x:v>2026 H1</x:v>
-      </x:c>
-      <x:c r="D28" s="80" t="str">
-        <x:v>来源</x:v>
-      </x:c>
-      <x:c r="E28" s="80"/>
-      <x:c r="F28" s="80"/>
-      <x:c r="G28" s="80"/>
+    <x:row r="28" ht="66" customHeight="1">
+      <x:c r="A28" s="151" t="str">
+        <x:v>T009</x:v>
+      </x:c>
+      <x:c r="B28" s="152" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C28" s="152" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D28" s="151" t="str">
+        <x:v>POLYN</x:v>
+      </x:c>
+      <x:c r="E28" s="151" t="str">
+        <x:v>TMS工程节点供客户评估</x:v>
+      </x:c>
+      <x:c r="F28" s="151" t="str">
+        <x:v>未具名评估方，非量产</x:v>
+      </x:c>
+      <x:c r="G28" s="151" t="str">
+        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+      </x:c>
       <x:c r="H28" s="67"/>
       <x:c r="I28" s="68"/>
       <x:c r="J28" s="2"/>
@@ -7006,18 +7154,10 @@
       <x:c r="O28" s="2"/>
     </x:row>
     <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="78" t="str">
-        <x:v>许可</x:v>
-      </x:c>
-      <x:c r="B29" s="79" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C29" s="79" t="n">
-        <x:v>613826</x:v>
-      </x:c>
-      <x:c r="D29" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
-      </x:c>
+      <x:c r="A29" s="78"/>
+      <x:c r="B29" s="79"/>
+      <x:c r="C29" s="79"/>
+      <x:c r="D29" s="80"/>
       <x:c r="E29" s="80"/>
       <x:c r="F29" s="80"/>
       <x:c r="G29" s="80"/>
@@ -7031,18 +7171,12 @@
       <x:c r="O29" s="2"/>
     </x:row>
     <x:row r="30" ht="30" customHeight="1">
-      <x:c r="A30" s="78" t="str">
-        <x:v>产品</x:v>
-      </x:c>
-      <x:c r="B30" s="79" t="n">
-        <x:v>19184</x:v>
-      </x:c>
-      <x:c r="C30" s="79" t="n">
-        <x:v>110362</x:v>
-      </x:c>
-      <x:c r="D30" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
-      </x:c>
+      <x:c r="A30" s="102" t="str">
+        <x:v>半年收入</x:v>
+      </x:c>
+      <x:c r="B30" s="103"/>
+      <x:c r="C30" s="103"/>
+      <x:c r="D30" s="104"/>
       <x:c r="E30" s="80"/>
       <x:c r="F30" s="80"/>
       <x:c r="G30" s="80"/>
@@ -7055,18 +7189,18 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="30" customHeight="1">
-      <x:c r="A31" s="78" t="str">
-        <x:v>开发服务</x:v>
-      </x:c>
-      <x:c r="B31" s="79" t="n">
-        <x:v>1004395</x:v>
-      </x:c>
-      <x:c r="C31" s="79" t="n">
-        <x:v>498557</x:v>
-      </x:c>
-      <x:c r="D31" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
+    <x:row r="31" ht="28" customHeight="1">
+      <x:c r="A31" s="153" t="str">
+        <x:v>构成</x:v>
+      </x:c>
+      <x:c r="B31" s="154" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C31" s="154" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D31" s="155" t="str">
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="E31" s="80"/>
       <x:c r="F31" s="80"/>
@@ -7080,20 +7214,18 @@
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="2"/>
     </x:row>
-    <x:row r="32" ht="30" customHeight="1">
+    <x:row r="32" ht="26" customHeight="1">
       <x:c r="A32" s="78" t="str">
-        <x:v>合计</x:v>
+        <x:v>许可</x:v>
       </x:c>
       <x:c r="B32" s="79" t="n">
-        <x:f>SUM(B29:B31)</x:f>
-        <x:v>1023579</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C32" s="79" t="n">
-        <x:f>SUM(C29:C31)</x:f>
-        <x:v>1222745</x:v>
+        <x:v>613826</x:v>
       </x:c>
       <x:c r="D32" s="80" t="str">
-        <x:v>监管半年报</x:v>
+        <x:v>半年报Note 3</x:v>
       </x:c>
       <x:c r="E32" s="80"/>
       <x:c r="F32" s="80"/>
@@ -7107,11 +7239,19 @@
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="2"/>
     </x:row>
-    <x:row r="33" ht="24" customHeight="1">
-      <x:c r="A33" s="78"/>
-      <x:c r="B33" s="80"/>
-      <x:c r="C33" s="80"/>
-      <x:c r="D33" s="80"/>
+    <x:row r="33" ht="26" customHeight="1">
+      <x:c r="A33" s="78" t="str">
+        <x:v>产品</x:v>
+      </x:c>
+      <x:c r="B33" s="79" t="n">
+        <x:v>19184</x:v>
+      </x:c>
+      <x:c r="C33" s="79" t="n">
+        <x:v>110362</x:v>
+      </x:c>
+      <x:c r="D33" s="80" t="str">
+        <x:v>半年报Note 3</x:v>
+      </x:c>
       <x:c r="E33" s="80"/>
       <x:c r="F33" s="80"/>
       <x:c r="G33" s="80"/>
@@ -7124,18 +7264,18 @@
       <x:c r="N33" s="2"/>
       <x:c r="O33" s="2"/>
     </x:row>
-    <x:row r="34" ht="24" customHeight="1">
+    <x:row r="34" ht="26" customHeight="1">
       <x:c r="A34" s="78" t="str">
-        <x:v>现金与客户指标</x:v>
-      </x:c>
-      <x:c r="B34" s="80" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C34" s="80" t="str">
-        <x:v>2026 H1</x:v>
+        <x:v>开发服务</x:v>
+      </x:c>
+      <x:c r="B34" s="79" t="n">
+        <x:v>1004395</x:v>
+      </x:c>
+      <x:c r="C34" s="79" t="n">
+        <x:v>498557</x:v>
       </x:c>
       <x:c r="D34" s="80" t="str">
-        <x:v>边界</x:v>
+        <x:v>半年报Note 3</x:v>
       </x:c>
       <x:c r="E34" s="80"/>
       <x:c r="F34" s="80"/>
@@ -7149,18 +7289,20 @@
       <x:c r="N34" s="2"/>
       <x:c r="O34" s="2"/>
     </x:row>
-    <x:row r="35" ht="24" customHeight="1">
+    <x:row r="35" ht="26" customHeight="1">
       <x:c r="A35" s="76" t="str">
-        <x:v>客户收款</x:v>
-      </x:c>
-      <x:c r="B35" s="77" t="n">
-        <x:v>1522026</x:v>
-      </x:c>
-      <x:c r="C35" s="77" t="n">
-        <x:v>813247</x:v>
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B35" s="86" t="n">
+        <x:f>SUM(B32:B34)</x:f>
+        <x:v>1023579</x:v>
+      </x:c>
+      <x:c r="C35" s="86" t="n">
+        <x:f>SUM(C32:C34)</x:f>
+        <x:v>1222745</x:v>
       </x:c>
       <x:c r="D35" s="77" t="str">
-        <x:v>现金流，不等于收入</x:v>
+        <x:v>监管半年报</x:v>
       </x:c>
       <x:c r="E35" s="77"/>
       <x:c r="F35" s="77"/>
@@ -7175,18 +7317,10 @@
       <x:c r="O35" s="2"/>
     </x:row>
     <x:row r="36" ht="72" customHeight="1">
-      <x:c r="A36" s="78" t="str">
-        <x:v>经营现金净流出</x:v>
-      </x:c>
-      <x:c r="B36" s="80" t="n">
-        <x:v>6990176</x:v>
-      </x:c>
-      <x:c r="C36" s="80" t="n">
-        <x:v>11253495</x:v>
-      </x:c>
-      <x:c r="D36" s="83" t="str">
-        <x:v>按流出绝对值展示</x:v>
-      </x:c>
+      <x:c r="A36" s="78"/>
+      <x:c r="B36" s="80"/>
+      <x:c r="C36" s="80"/>
+      <x:c r="D36" s="83"/>
       <x:c r="E36" s="80"/>
       <x:c r="F36" s="80"/>
       <x:c r="G36" s="80"/>
@@ -7200,17 +7334,17 @@
       <x:c r="O36" s="2"/>
     </x:row>
     <x:row r="37" ht="28" customHeight="1">
-      <x:c r="A37" s="116" t="str">
-        <x:v>期末现金及现金等价物</x:v>
-      </x:c>
-      <x:c r="B37" s="118" t="n">
-        <x:v>13458121</x:v>
-      </x:c>
-      <x:c r="C37" s="118" t="n">
-        <x:v>20304971</x:v>
-      </x:c>
-      <x:c r="D37" s="119" t="str">
-        <x:v>各年6月30日</x:v>
+      <x:c r="A37" s="153" t="str">
+        <x:v>现金与客户指标</x:v>
+      </x:c>
+      <x:c r="B37" s="155" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C37" s="155" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D37" s="156" t="str">
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="E37" s="118"/>
       <x:c r="F37" s="118"/>
@@ -7224,18 +7358,18 @@
       <x:c r="N37" s="2"/>
       <x:c r="O37" s="2"/>
     </x:row>
-    <x:row r="38" ht="72" customHeight="1">
+    <x:row r="38" ht="30" customHeight="1">
       <x:c r="A38" s="78" t="str">
-        <x:v>&gt;10%客户收入合计</x:v>
-      </x:c>
-      <x:c r="B38" s="80" t="n">
-        <x:v>809706</x:v>
-      </x:c>
-      <x:c r="C38" s="80" t="n">
-        <x:v>983780</x:v>
+        <x:v>客户收款</x:v>
+      </x:c>
+      <x:c r="B38" s="79" t="n">
+        <x:v>1522026</x:v>
+      </x:c>
+      <x:c r="C38" s="79" t="n">
+        <x:v>813247</x:v>
       </x:c>
       <x:c r="D38" s="83" t="str">
-        <x:v>2026约占H1收入80.5%</x:v>
+        <x:v>现金流，不等于收入</x:v>
       </x:c>
       <x:c r="E38" s="80"/>
       <x:c r="F38" s="80"/>
@@ -7249,16 +7383,18 @@
       <x:c r="N38" s="2"/>
       <x:c r="O38" s="2"/>
     </x:row>
-    <x:row r="39" ht="72" customHeight="1">
+    <x:row r="39" ht="30" customHeight="1">
       <x:c r="A39" s="78" t="str">
-        <x:v>首批AKD1500生产批次</x:v>
-      </x:c>
-      <x:c r="B39" s="80"/>
-      <x:c r="C39" s="80" t="n">
-        <x:v>2000</x:v>
+        <x:v>经营现金净流出</x:v>
+      </x:c>
+      <x:c r="B39" s="79" t="n">
+        <x:v>6990176</x:v>
+      </x:c>
+      <x:c r="C39" s="79" t="n">
+        <x:v>11253495</x:v>
       </x:c>
       <x:c r="D39" s="83" t="str">
-        <x:v>颗；公司收到，不是客户出货</x:v>
+        <x:v>按流出绝对值展示</x:v>
       </x:c>
       <x:c r="E39" s="80"/>
       <x:c r="F39" s="80"/>
@@ -7272,11 +7408,19 @@
       <x:c r="N39" s="2"/>
       <x:c r="O39" s="2"/>
     </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="78"/>
-      <x:c r="B40" s="80"/>
-      <x:c r="C40" s="80"/>
-      <x:c r="D40" s="80"/>
+    <x:row r="40" ht="30" customHeight="1">
+      <x:c r="A40" s="78" t="str">
+        <x:v>期末现金及现金等价物</x:v>
+      </x:c>
+      <x:c r="B40" s="79" t="n">
+        <x:v>13458121</x:v>
+      </x:c>
+      <x:c r="C40" s="79" t="n">
+        <x:v>20304971</x:v>
+      </x:c>
+      <x:c r="D40" s="80" t="str">
+        <x:v>各年6月30日</x:v>
+      </x:c>
       <x:c r="E40" s="80"/>
       <x:c r="F40" s="80"/>
       <x:c r="G40" s="80"/>
@@ -7289,15 +7433,19 @@
       <x:c r="N40" s="2"/>
       <x:c r="O40" s="2"/>
     </x:row>
-    <x:row r="41" ht="28" customHeight="1">
-      <x:c r="A41" s="116" t="str">
-        <x:v>来源</x:v>
-      </x:c>
-      <x:c r="B41" s="118" t="str">
-        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
-      </x:c>
-      <x:c r="C41" s="118"/>
-      <x:c r="D41" s="118"/>
+    <x:row r="41" ht="30" customHeight="1">
+      <x:c r="A41" s="132" t="str">
+        <x:v>&gt;10%客户收入合计</x:v>
+      </x:c>
+      <x:c r="B41" s="134" t="n">
+        <x:v>809706</x:v>
+      </x:c>
+      <x:c r="C41" s="134" t="n">
+        <x:v>983780</x:v>
+      </x:c>
+      <x:c r="D41" s="133" t="str">
+        <x:v>2026约占H1收入80.5%</x:v>
+      </x:c>
       <x:c r="E41" s="80"/>
       <x:c r="F41" s="80"/>
       <x:c r="G41" s="80"/>
@@ -7310,15 +7458,17 @@
       <x:c r="N41" s="2"/>
       <x:c r="O41" s="2"/>
     </x:row>
-    <x:row r="42" ht="44" customHeight="1">
+    <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="105" t="str">
-        <x:v>边界</x:v>
-      </x:c>
-      <x:c r="B42" s="80" t="str">
-        <x:v>监管文件披露首批2,000颗生产批次及良率低于预期；未披露客户出货、单品收入或版税。</x:v>
-      </x:c>
-      <x:c r="C42" s="80"/>
-      <x:c r="D42" s="80"/>
+        <x:v>首批AKD1500生产批次</x:v>
+      </x:c>
+      <x:c r="B42" s="79"/>
+      <x:c r="C42" s="79" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D42" s="80" t="str">
+        <x:v>颗；公司收到，不是客户出货</x:v>
+      </x:c>
       <x:c r="E42" s="80"/>
       <x:c r="F42" s="80"/>
       <x:c r="G42" s="80"/>
@@ -7348,34 +7498,20 @@
       <x:c r="N43" s="2"/>
       <x:c r="O43" s="2"/>
     </x:row>
-    <x:row r="44" ht="44" customHeight="1">
+    <x:row r="44" ht="34" customHeight="1">
       <x:c r="A44" s="105" t="str">
-        <x:v>研究编号</x:v>
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="B44" s="80" t="str">
-        <x:v>研究主体</x:v>
-      </x:c>
-      <x:c r="C44" s="80" t="str">
-        <x:v>路线</x:v>
-      </x:c>
-      <x:c r="D44" s="83" t="str">
-        <x:v>发布日期</x:v>
-      </x:c>
-      <x:c r="E44" s="80" t="str">
-        <x:v>证据类型</x:v>
-      </x:c>
-      <x:c r="F44" s="80" t="str">
-        <x:v>作者报告指标</x:v>
-      </x:c>
-      <x:c r="G44" s="80" t="str">
-        <x:v>边界</x:v>
-      </x:c>
-      <x:c r="H44" s="80" t="str">
-        <x:v>原始URL</x:v>
-      </x:c>
-      <x:c r="I44" s="127" t="str">
-        <x:v>检索日期</x:v>
-      </x:c>
+        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
+      </x:c>
+      <x:c r="C44" s="80"/>
+      <x:c r="D44" s="83"/>
+      <x:c r="E44" s="80"/>
+      <x:c r="F44" s="80"/>
+      <x:c r="G44" s="80"/>
+      <x:c r="H44" s="80"/>
+      <x:c r="I44" s="127"/>
       <x:c r="J44" s="2"/>
       <x:c r="K44" s="2"/>
       <x:c r="L44" s="2"/>
@@ -7383,34 +7519,20 @@
       <x:c r="N44" s="2"/>
       <x:c r="O44" s="2"/>
     </x:row>
-    <x:row r="45" ht="64" customHeight="1">
+    <x:row r="45" ht="34" customHeight="1">
       <x:c r="A45" s="106" t="str">
-        <x:v>R001</x:v>
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="B45" s="107" t="str">
-        <x:v>GelNeuro／中科院自动化所</x:v>
-      </x:c>
-      <x:c r="C45" s="107" t="str">
-        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
-      </x:c>
-      <x:c r="D45" s="125" t="d">
-        <x:v>2026-07-06T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E45" s="107" t="str">
-        <x:v>作者预印本实机研究结果，未独立复现</x:v>
-      </x:c>
-      <x:c r="F45" s="107" t="str">
-        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
-      </x:c>
-      <x:c r="G45" s="107" t="str">
-        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
-      </x:c>
-      <x:c r="H45" s="107" t="str">
-        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
-      </x:c>
-      <x:c r="I45" s="128" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>BrainChip财务数据来自监管半年报；SpiNNcloud 336万欧元为公共采购合同授予值，不计入BrainChip收入图，也不等于SpiNNcloud已付款或确认收入。</x:v>
+      </x:c>
+      <x:c r="C45" s="107"/>
+      <x:c r="D45" s="125"/>
+      <x:c r="E45" s="107"/>
+      <x:c r="F45" s="107"/>
+      <x:c r="G45" s="107"/>
+      <x:c r="H45" s="107"/>
+      <x:c r="I45" s="128"/>
       <x:c r="J45" s="2"/>
       <x:c r="K45" s="2"/>
       <x:c r="L45" s="2"/>
@@ -7419,33 +7541,15 @@
       <x:c r="O45" s="2"/>
     </x:row>
     <x:row r="46" ht="64" customHeight="1">
-      <x:c r="A46" s="4" t="str">
-        <x:v>R002</x:v>
-      </x:c>
-      <x:c r="B46" s="3" t="str">
-        <x:v>SpikingTac／中科院自动化所</x:v>
-      </x:c>
-      <x:c r="C46" s="3" t="str">
-        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
-      </x:c>
-      <x:c r="D46" s="4" t="d">
-        <x:v>2026-02-27T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E46" s="3" t="str">
-        <x:v>作者预印本研究样机，未独立复现</x:v>
-      </x:c>
-      <x:c r="F46" s="3" t="str">
-        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
-      </x:c>
-      <x:c r="G46" s="3" t="str">
-        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
-      </x:c>
-      <x:c r="H46" s="3" t="str">
-        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
-      </x:c>
-      <x:c r="I46" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
-      </x:c>
+      <x:c r="A46" s="4"/>
+      <x:c r="B46" s="3"/>
+      <x:c r="C46" s="3"/>
+      <x:c r="D46" s="4"/>
+      <x:c r="E46" s="3"/>
+      <x:c r="F46" s="3"/>
+      <x:c r="G46" s="3"/>
+      <x:c r="H46" s="3"/>
+      <x:c r="I46" s="4"/>
       <x:c r="J46" s="2"/>
       <x:c r="K46" s="2"/>
       <x:c r="L46" s="2"/>
@@ -7455,31 +7559,31 @@
     </x:row>
     <x:row r="47" ht="64" customHeight="1">
       <x:c r="A47" s="4" t="str">
-        <x:v>R003</x:v>
+        <x:v>研究编号</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>OmniVTA／NUS、CASIA等</x:v>
+        <x:v>研究主体</x:v>
       </x:c>
       <x:c r="C47" s="3" t="str">
-        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
-      </x:c>
-      <x:c r="D47" s="4" t="d">
-        <x:v>2026-03-19T00:00:00.000Z</x:v>
+        <x:v>路线</x:v>
+      </x:c>
+      <x:c r="D47" s="4" t="str">
+        <x:v>发布日期</x:v>
       </x:c>
       <x:c r="E47" s="3" t="str">
-        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
+        <x:v>证据类型</x:v>
       </x:c>
       <x:c r="F47" s="3" t="str">
-        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
+        <x:v>作者报告指标</x:v>
       </x:c>
       <x:c r="G47" s="3" t="str">
-        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="H47" s="3" t="str">
-        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
-      </x:c>
-      <x:c r="I47" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>原始URL</x:v>
+      </x:c>
+      <x:c r="I47" s="4" t="str">
+        <x:v>检索日期</x:v>
       </x:c>
       <x:c r="J47" s="2"/>
       <x:c r="K47" s="2"/>
@@ -7488,30 +7592,30 @@
       <x:c r="N47" s="2"/>
       <x:c r="O47" s="2"/>
     </x:row>
-    <x:row r="48" ht="64" customHeight="1">
+    <x:row r="48" ht="82" customHeight="1">
       <x:c r="A48" s="3" t="str">
-        <x:v>R004</x:v>
+        <x:v>R001</x:v>
       </x:c>
       <x:c r="B48" s="3" t="str">
-        <x:v>Event-VLA／上海科技大学等</x:v>
+        <x:v>GelNeuro／中科院自动化所</x:v>
       </x:c>
       <x:c r="C48" s="3" t="str">
-        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
+        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
       </x:c>
       <x:c r="D48" s="4" t="d">
-        <x:v>2026-06-28T00:00:00.000Z</x:v>
+        <x:v>2026-07-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E48" s="3" t="str">
-        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
+        <x:v>作者预印本实机研究结果，未独立复现</x:v>
       </x:c>
       <x:c r="F48" s="3" t="str">
-        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
+        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
-        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
+        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
       </x:c>
       <x:c r="H48" s="3" t="str">
-        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
+        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
       </x:c>
       <x:c r="I48" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7523,30 +7627,30 @@
       <x:c r="N48" s="2"/>
       <x:c r="O48" s="2"/>
     </x:row>
-    <x:row r="49" ht="64" customHeight="1">
+    <x:row r="49" ht="82" customHeight="1">
       <x:c r="A49" s="3" t="str">
-        <x:v>R005</x:v>
+        <x:v>R002</x:v>
       </x:c>
       <x:c r="B49" s="3" t="str">
-        <x:v>TouchWorld／研究团队</x:v>
+        <x:v>SpikingTac／中科院自动化所</x:v>
       </x:c>
       <x:c r="C49" s="3" t="str">
-        <x:v>预测式＋反应式触觉基础模型</x:v>
+        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
       </x:c>
       <x:c r="D49" s="4" t="d">
-        <x:v>2026-07-08T00:00:00.000Z</x:v>
+        <x:v>2026-02-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E49" s="3" t="str">
-        <x:v>作者预印本研究；未独立复现</x:v>
+        <x:v>作者预印本研究样机，未独立复现</x:v>
       </x:c>
       <x:c r="F49" s="3" t="str">
-        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
+        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
       </x:c>
       <x:c r="G49" s="3" t="str">
-        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
+        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
       </x:c>
       <x:c r="H49" s="3" t="str">
-        <x:v>https://arxiv.org/abs/2607.07287</x:v>
+        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
       </x:c>
       <x:c r="I49" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7558,30 +7662,30 @@
       <x:c r="N49" s="2"/>
       <x:c r="O49" s="2"/>
     </x:row>
-    <x:row r="50" ht="180" customHeight="1">
+    <x:row r="50" ht="82" customHeight="1">
       <x:c r="A50" s="3" t="str">
-        <x:v>R006</x:v>
+        <x:v>R003</x:v>
       </x:c>
       <x:c r="B50" s="3" t="str">
-        <x:v>CLP-SNN／LMU、Intel等</x:v>
+        <x:v>OmniVTA／NUS、CASIA等</x:v>
       </x:c>
       <x:c r="C50" s="3" t="str">
-        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
       </x:c>
       <x:c r="D50" s="4" t="d">
-        <x:v>2026-05-05T00:00:00.000Z</x:v>
+        <x:v>2026-03-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E50" s="3" t="str">
-        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
       </x:c>
       <x:c r="F50" s="3" t="str">
-        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
       </x:c>
       <x:c r="G50" s="3" t="str">
-        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
       </x:c>
       <x:c r="H50" s="3" t="str">
-        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
       </x:c>
       <x:c r="I50" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7593,24 +7697,34 @@
       <x:c r="N50" s="2"/>
       <x:c r="O50" s="2"/>
     </x:row>
-    <x:row r="51" ht="24" customHeight="1">
-      <x:c r="A51" s="2" t="str">
-        <x:v>并购与退出日期</x:v>
-      </x:c>
-      <x:c r="B51" s="2" t="str">
-        <x:v>交易／整合</x:v>
-      </x:c>
-      <x:c r="C51" s="2" t="str">
-        <x:v>状态</x:v>
-      </x:c>
-      <x:c r="D51" s="2" t="str">
-        <x:v>证据边界</x:v>
-      </x:c>
-      <x:c r="E51" s="2"/>
-      <x:c r="F51" s="2"/>
-      <x:c r="G51" s="2"/>
-      <x:c r="H51" s="2"/>
-      <x:c r="I51" s="2"/>
+    <x:row r="51" ht="82" customHeight="1">
+      <x:c r="A51" s="3" t="str">
+        <x:v>R004</x:v>
+      </x:c>
+      <x:c r="B51" s="3" t="str">
+        <x:v>Event-VLA／上海科技大学等</x:v>
+      </x:c>
+      <x:c r="C51" s="3" t="str">
+        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
+      </x:c>
+      <x:c r="D51" s="4" t="d">
+        <x:v>2026-06-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E51" s="3" t="str">
+        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
+      </x:c>
+      <x:c r="F51" s="3" t="str">
+        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
+      </x:c>
+      <x:c r="G51" s="3" t="str">
+        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
+      </x:c>
+      <x:c r="H51" s="3" t="str">
+        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
+      </x:c>
+      <x:c r="I51" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J51" s="2"/>
       <x:c r="K51" s="2"/>
       <x:c r="L51" s="2"/>
@@ -7618,24 +7732,34 @@
       <x:c r="N51" s="2"/>
       <x:c r="O51" s="2"/>
     </x:row>
-    <x:row r="52" ht="50" customHeight="1">
-      <x:c r="A52" s="11" t="n">
-        <x:v>45230</x:v>
-      </x:c>
-      <x:c r="B52" s="2" t="str">
-        <x:v>GrAI Matter Labs → Snap</x:v>
-      </x:c>
-      <x:c r="C52" s="2" t="str">
-        <x:v>交易后于2024-02-01吸收合并注销</x:v>
-      </x:c>
-      <x:c r="D52" s="2" t="str">
-        <x:v>不再计独立供应商；技术落地与收购价未知</x:v>
-      </x:c>
-      <x:c r="E52" s="2"/>
-      <x:c r="F52" s="2"/>
-      <x:c r="G52" s="2"/>
-      <x:c r="H52" s="2"/>
-      <x:c r="I52" s="2"/>
+    <x:row r="52" ht="82" customHeight="1">
+      <x:c r="A52" s="4" t="str">
+        <x:v>R005</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="str">
+        <x:v>TouchWorld／研究团队</x:v>
+      </x:c>
+      <x:c r="C52" s="3" t="str">
+        <x:v>预测式＋反应式触觉基础模型</x:v>
+      </x:c>
+      <x:c r="D52" s="4" t="d">
+        <x:v>2026-07-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E52" s="3" t="str">
+        <x:v>作者预印本研究；未独立复现</x:v>
+      </x:c>
+      <x:c r="F52" s="3" t="str">
+        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
+      </x:c>
+      <x:c r="G52" s="3" t="str">
+        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="str">
+        <x:v>https://arxiv.org/abs/2607.07287</x:v>
+      </x:c>
+      <x:c r="I52" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J52" s="2"/>
       <x:c r="K52" s="2"/>
       <x:c r="L52" s="2"/>
@@ -7643,24 +7767,34 @@
       <x:c r="N52" s="2"/>
       <x:c r="O52" s="2"/>
     </x:row>
-    <x:row r="53" ht="50" customHeight="1">
-      <x:c r="A53" s="11" t="n">
-        <x:v>45323</x:v>
-      </x:c>
-      <x:c r="B53" s="2" t="str">
-        <x:v>iniVation → SynSense Group</x:v>
-      </x:c>
-      <x:c r="C53" s="2" t="str">
-        <x:v>100%股份收购；苏黎世实体继续运营</x:v>
-      </x:c>
-      <x:c r="D53" s="2" t="str">
-        <x:v>交易金额未知；品牌／产品继续不等于独立所有权</x:v>
-      </x:c>
-      <x:c r="E53" s="2"/>
-      <x:c r="F53" s="2"/>
-      <x:c r="G53" s="2"/>
-      <x:c r="H53" s="2"/>
-      <x:c r="I53" s="2"/>
+    <x:row r="53" ht="82" customHeight="1">
+      <x:c r="A53" s="4" t="str">
+        <x:v>R006</x:v>
+      </x:c>
+      <x:c r="B53" s="3" t="str">
+        <x:v>CLP-SNN／LMU、Intel等</x:v>
+      </x:c>
+      <x:c r="C53" s="3" t="str">
+        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+      </x:c>
+      <x:c r="D53" s="4" t="d">
+        <x:v>2026-05-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E53" s="3" t="str">
+        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+      </x:c>
+      <x:c r="F53" s="3" t="str">
+        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+      </x:c>
+      <x:c r="G53" s="3" t="str">
+        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+      </x:c>
+      <x:c r="H53" s="3" t="str">
+        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+      </x:c>
+      <x:c r="I53" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J53" s="2"/>
       <x:c r="K53" s="2"/>
       <x:c r="L53" s="2"/>
@@ -7669,18 +7803,10 @@
       <x:c r="O53" s="2"/>
     </x:row>
     <x:row r="54" ht="50" customHeight="1">
-      <x:c r="A54" s="11" t="n">
-        <x:v>45656</x:v>
-      </x:c>
-      <x:c r="B54" s="2" t="str">
-        <x:v>Knowles消费MEMS麦克风 → Syntiant</x:v>
-      </x:c>
-      <x:c r="C54" s="2" t="str">
-        <x:v>已完成；1.5亿美元现金加股票</x:v>
-      </x:c>
-      <x:c r="D54" s="2" t="str">
-        <x:v>2.56亿美元为被收购业务2023收入，不是NDP芯片收入</x:v>
-      </x:c>
+      <x:c r="A54" s="11"/>
+      <x:c r="B54" s="2"/>
+      <x:c r="C54" s="2"/>
+      <x:c r="D54" s="2"/>
       <x:c r="E54" s="2"/>
       <x:c r="F54" s="2"/>
       <x:c r="G54" s="2"/>
@@ -7694,18 +7820,10 @@
       <x:c r="O54" s="2"/>
     </x:row>
     <x:row r="55" ht="50" customHeight="1">
-      <x:c r="A55" s="11" t="n">
-        <x:v>46161</x:v>
-      </x:c>
-      <x:c r="B55" s="2" t="str">
-        <x:v>Videantis → Mythic</x:v>
-      </x:c>
-      <x:c r="C55" s="2" t="str">
-        <x:v>已完成</x:v>
-      </x:c>
-      <x:c r="D55" s="2" t="str">
-        <x:v>Videantis既有装机不计Mythic模拟APU出货</x:v>
-      </x:c>
+      <x:c r="A55" s="11"/>
+      <x:c r="B55" s="2"/>
+      <x:c r="C55" s="2"/>
+      <x:c r="D55" s="2"/>
       <x:c r="E55" s="2"/>
       <x:c r="F55" s="2"/>
       <x:c r="G55" s="2"/>
@@ -7719,18 +7837,10 @@
       <x:c r="O55" s="2"/>
     </x:row>
     <x:row r="56" ht="50" customHeight="1">
-      <x:c r="A56" s="11" t="n">
-        <x:v>46224</x:v>
-      </x:c>
-      <x:c r="B56" s="2" t="str">
-        <x:v>SceniX → World Labs</x:v>
-      </x:c>
-      <x:c r="C56" s="2" t="str">
-        <x:v>已并入；R2S2R机器人仿真链</x:v>
-      </x:c>
-      <x:c r="D56" s="2" t="str">
-        <x:v>公司展示未独立复现；金额和客户收入未知</x:v>
-      </x:c>
+      <x:c r="A56" s="11"/>
+      <x:c r="B56" s="2"/>
+      <x:c r="C56" s="2"/>
+      <x:c r="D56" s="2"/>
       <x:c r="E56" s="2"/>
       <x:c r="F56" s="2"/>
       <x:c r="G56" s="2"/>
@@ -7744,18 +7854,10 @@
       <x:c r="O56" s="2"/>
     </x:row>
     <x:row r="57" ht="50" customHeight="1">
-      <x:c r="A57" s="11" t="n">
-        <x:v>46291</x:v>
-      </x:c>
-      <x:c r="B57" s="2" t="str">
-        <x:v>World Labs → AMD</x:v>
-      </x:c>
-      <x:c r="C57" s="2" t="str">
-        <x:v>已签协议，预计年底完成</x:v>
-      </x:c>
-      <x:c r="D57" s="2" t="str">
-        <x:v>约82亿美元全股票；仍待监管与交割条件</x:v>
-      </x:c>
+      <x:c r="A57" s="11"/>
+      <x:c r="B57" s="2"/>
+      <x:c r="C57" s="2"/>
+      <x:c r="D57" s="2"/>
       <x:c r="E57" s="2"/>
       <x:c r="F57" s="2"/>
       <x:c r="G57" s="2"/>
@@ -7822,8 +7924,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d3df74c6dde4e36"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3ce6845916b4d7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra950f82ed62346bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c7a631d9754f9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Track Prophesee restructuring and ModelCat pivot
Refresh the mobile report, evidence data, charts and workbook to 38 companies, 40 product records and 29 events.
</commit_message>
<xml_diff>
--- a/market-evidence.xlsx
+++ b/market-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="R472c4ec51b854594"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="R653226e7071d4609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="Rd7e929da9548438e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="Rec52a6984a9843a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="R537b605574be4760"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="Raff751be60c14ce2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="R7a810256b33f471f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="R7bedf60f1bec451f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,7 +69,7 @@
       <x:name val="Noto Sans SC"/>
     </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="28">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -176,6 +176,36 @@
         <x:fgColor rgb="FF23445C"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="9">
     <x:border/>
@@ -211,7 +241,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="161">
+  <x:cellXfs count="186">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -621,6 +651,69 @@
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="26" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="6" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="3" fillId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1166,7 +1259,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R40f48f2df1f5462e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3bba0f9f16954405"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1196,7 +1289,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b34b835bb26468b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b7f94dbe09b4ab0"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1226,7 +1319,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83eacf13a578408d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3549f9c9096d4b63"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1236,7 +1329,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I38" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1253,7 +1346,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1271,7 +1364,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="事件日期"/>
@@ -1286,7 +1379,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A47:I53" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A49:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="研究编号"/>
     <x:tableColumn id="2" name="研究主体"/>
@@ -1500,7 +1593,7 @@
     <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
@@ -1549,7 +1642,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-02商业化证据复核。37个主体、39组产品、27项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
+        <x:v>2026-10-02小公司、退出收购与路线转向复核。38个主体、40组产品、29项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1609,7 +1702,6 @@
         <x:v>硬件与平台</x:v>
       </x:c>
       <x:c r="B6" s="2" t="n">
-        <x:f>COUNTIF('主体证据'!$C$2:$C$38,A6)</x:f>
         <x:v>11</x:v>
       </x:c>
       <x:c r="C6" s="2"/>
@@ -1631,7 +1723,6 @@
         <x:v>模型与系统</x:v>
       </x:c>
       <x:c r="B7" s="2" t="n">
-        <x:f>COUNTIF('主体证据'!$C$2:$C$38,A7)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C7" s="2"/>
@@ -1653,8 +1744,7 @@
         <x:v>相邻替代</x:v>
       </x:c>
       <x:c r="B8" s="2" t="n">
-        <x:f>COUNTIF('主体证据'!$C$2:$C$38,A8)</x:f>
-        <x:v>19</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C8" s="2"/>
       <x:c r="D8" s="2"/>
@@ -1747,7 +1837,7 @@
         <x:v>方案／研发</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A13)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A13)</x:f>
         <x:v>7</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
@@ -1769,7 +1859,7 @@
         <x:v>研究／原型</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A14)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A14)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
@@ -1791,7 +1881,7 @@
         <x:v>工程样片</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A15)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A15)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
@@ -1813,7 +1903,7 @@
         <x:v>IP／商务接洽</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A16)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A16)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
@@ -1835,8 +1925,8 @@
         <x:v>开发平台</x:v>
       </x:c>
       <x:c r="B17" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A17)</x:f>
-        <x:v>1</x:v>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A17)</x:f>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="2"/>
@@ -1857,7 +1947,7 @@
         <x:v>客户评估／模块</x:v>
       </x:c>
       <x:c r="B18" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A18)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A18)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
@@ -1879,7 +1969,7 @@
         <x:v>可采购硬件</x:v>
       </x:c>
       <x:c r="B19" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A19)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A19)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="2"/>
@@ -1901,7 +1991,7 @@
         <x:v>商品页／售罄</x:v>
       </x:c>
       <x:c r="B20" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A20)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A20)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C20" s="2"/>
@@ -1923,7 +2013,7 @@
         <x:v>生产／部署声明</x:v>
       </x:c>
       <x:c r="B21" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A21)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A21)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C21" s="2"/>
@@ -1945,7 +2035,7 @@
         <x:v>发布／演示</x:v>
       </x:c>
       <x:c r="B22" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A22)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A22)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
@@ -1967,7 +2057,7 @@
         <x:v>已签公共采购合同／科研部署</x:v>
       </x:c>
       <x:c r="B23" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$40,A23)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A23)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="2"/>
@@ -2031,15 +2121,15 @@
         <x:v>许可</x:v>
       </x:c>
       <x:c r="B26" s="5" t="n">
-        <x:f>'事件与财务'!B32</x:f>
+        <x:f>'事件与财务'!B34</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C26" s="5" t="n">
-        <x:f>'事件与财务'!C32</x:f>
+        <x:f>'事件与财务'!C34</x:f>
         <x:v>613826</x:v>
       </x:c>
       <x:c r="D26" s="6" t="n">
-        <x:f>C26/'事件与财务'!C35</x:f>
+        <x:f>C26/'事件与财务'!C37</x:f>
         <x:v>0.5020065508343932</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
@@ -2059,15 +2149,15 @@
         <x:v>产品</x:v>
       </x:c>
       <x:c r="B27" s="5" t="n">
-        <x:f>'事件与财务'!B33</x:f>
+        <x:f>'事件与财务'!B35</x:f>
         <x:v>19184</x:v>
       </x:c>
       <x:c r="C27" s="5" t="n">
-        <x:f>'事件与财务'!C33</x:f>
+        <x:f>'事件与财务'!C35</x:f>
         <x:v>110362</x:v>
       </x:c>
       <x:c r="D27" s="6" t="n">
-        <x:f>C27/'事件与财务'!C35</x:f>
+        <x:f>C27/'事件与财务'!C37</x:f>
         <x:v>0.09025757619127454</x:v>
       </x:c>
       <x:c r="E27" s="2"/>
@@ -2087,15 +2177,15 @@
         <x:v>开发服务</x:v>
       </x:c>
       <x:c r="B28" s="5" t="n">
-        <x:f>'事件与财务'!B34</x:f>
+        <x:f>'事件与财务'!B36</x:f>
         <x:v>1004395</x:v>
       </x:c>
       <x:c r="C28" s="5" t="n">
-        <x:f>'事件与财务'!C34</x:f>
+        <x:f>'事件与财务'!C36</x:f>
         <x:v>498557</x:v>
       </x:c>
       <x:c r="D28" s="6" t="n">
-        <x:f>C28/'事件与财务'!C35</x:f>
+        <x:f>C28/'事件与财务'!C37</x:f>
         <x:v>0.40773587297433234</x:v>
       </x:c>
       <x:c r="E28" s="2"/>
@@ -2331,16 +2421,16 @@
       <x:c r="O38" s="2"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
-      <x:c r="A39" s="159" t="str">
+      <x:c r="A39" s="185" t="str">
         <x:v>可核商业化合同</x:v>
       </x:c>
-      <x:c r="B39" s="159" t="str">
+      <x:c r="B39" s="185" t="str">
         <x:v>签约日</x:v>
       </x:c>
-      <x:c r="C39" s="159" t="str">
+      <x:c r="C39" s="185" t="str">
         <x:v>合同授予值</x:v>
       </x:c>
-      <x:c r="D39" s="159" t="str">
+      <x:c r="D39" s="185" t="str">
         <x:v>边界</x:v>
       </x:c>
       <x:c r="E39" s="2"/>
@@ -2355,7 +2445,7 @@
       <x:c r="N39" s="2"/>
       <x:c r="O39" s="2"/>
     </x:row>
-    <x:row r="40" ht="34" customHeight="1">
+    <x:row r="40" ht="48" customHeight="1">
       <x:c r="A40" s="151" t="str">
         <x:v>Jülich → SpiNNcloud</x:v>
       </x:c>
@@ -2380,7 +2470,7 @@
       <x:c r="N40" s="2"/>
       <x:c r="O40" s="2"/>
     </x:row>
-    <x:row r="41" ht="34" customHeight="1">
+    <x:row r="41" ht="48" customHeight="1">
       <x:c r="A41" s="151" t="str">
         <x:v>莱比锡科研设施资助</x:v>
       </x:c>
@@ -2423,16 +2513,16 @@
       <x:c r="O42" s="2"/>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
-      <x:c r="A43" s="159" t="str">
+      <x:c r="A43" s="185" t="str">
         <x:v>并购与退出追溯</x:v>
       </x:c>
-      <x:c r="B43" s="159" t="str">
+      <x:c r="B43" s="185" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="C43" s="159" t="str">
+      <x:c r="C43" s="185" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="D43" s="159" t="str">
+      <x:c r="D43" s="185" t="str">
         <x:v>证据边界</x:v>
       </x:c>
       <x:c r="E43" s="2"/>
@@ -2447,7 +2537,7 @@
       <x:c r="N43" s="2"/>
       <x:c r="O43" s="2"/>
     </x:row>
-    <x:row r="44" ht="34" customHeight="1">
+    <x:row r="44" ht="82" customHeight="1">
       <x:c r="A44" s="151" t="str">
         <x:v>GrAI Matter Labs → Snap</x:v>
       </x:c>
@@ -2472,7 +2562,7 @@
       <x:c r="N44" s="2"/>
       <x:c r="O44" s="2"/>
     </x:row>
-    <x:row r="45" ht="34" customHeight="1">
+    <x:row r="45" ht="82" customHeight="1">
       <x:c r="A45" s="151" t="str">
         <x:v>iniVation → SynSense Group</x:v>
       </x:c>
@@ -2497,18 +2587,18 @@
       <x:c r="N45" s="2"/>
       <x:c r="O45" s="2"/>
     </x:row>
-    <x:row r="46" ht="34" customHeight="1">
+    <x:row r="46" ht="82" customHeight="1">
       <x:c r="A46" s="151" t="str">
-        <x:v>Knowles消费MEMS麦克风 → Syntiant</x:v>
-      </x:c>
-      <x:c r="B46" s="152" t="d">
-        <x:v>2024-12-30T00:00:00.000Z</x:v>
+        <x:v>Prophesee司法重整 → 持续经营与全栈转向</x:v>
+      </x:c>
+      <x:c r="B46" s="152" t="str">
+        <x:v>2024-10-15／2026-05-05</x:v>
       </x:c>
       <x:c r="C46" s="151" t="str">
-        <x:v>已完成；1.5亿美元现金加股票</x:v>
+        <x:v>2024年启动司法重整；2026年5月法院批准重整计划，6月公司宣布2000万欧元融资</x:v>
       </x:c>
       <x:c r="D46" s="151" t="str">
-        <x:v>2.56亿美元为被收购业务2023收入，不是NDP芯片收入</x:v>
+        <x:v>不是收购或清算；融资不计收入。经营恢复、Mantara商业化和长期偿付情况仍需持续跟踪</x:v>
       </x:c>
       <x:c r="E46" s="2"/>
       <x:c r="F46" s="2"/>
@@ -2522,18 +2612,18 @@
       <x:c r="N46" s="2"/>
       <x:c r="O46" s="2"/>
     </x:row>
-    <x:row r="47" ht="34" customHeight="1">
+    <x:row r="47" ht="82" customHeight="1">
       <x:c r="A47" s="151" t="str">
-        <x:v>Videantis → Mythic</x:v>
+        <x:v>Knowles消费MEMS麦克风 → Syntiant</x:v>
       </x:c>
       <x:c r="B47" s="152" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
+        <x:v>2024-12-30T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C47" s="151" t="str">
-        <x:v>已完成</x:v>
+        <x:v>已完成；1.5亿美元现金加股票</x:v>
       </x:c>
       <x:c r="D47" s="151" t="str">
-        <x:v>Videantis既有装机不计Mythic模拟APU出货</x:v>
+        <x:v>2.56亿美元为被收购业务2023收入，不是NDP芯片收入</x:v>
       </x:c>
       <x:c r="E47" s="2"/>
       <x:c r="F47" s="2"/>
@@ -2547,18 +2637,18 @@
       <x:c r="N47" s="2"/>
       <x:c r="O47" s="2"/>
     </x:row>
-    <x:row r="48" ht="34" customHeight="1">
+    <x:row r="48" ht="82" customHeight="1">
       <x:c r="A48" s="151" t="str">
-        <x:v>SceniX → World Labs</x:v>
+        <x:v>Eta Compute → ModelCat路线转向</x:v>
       </x:c>
       <x:c r="B48" s="152" t="d">
-        <x:v>2026-07-21T00:00:00.000Z</x:v>
+        <x:v>2025-08-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C48" s="151" t="str">
-        <x:v>已并入；R2S2R机器人仿真链</x:v>
+        <x:v>更名并把核心产品转为硬件感知的模型构建软件；NXP eIQ Model Creator采用订阅收费</x:v>
       </x:c>
       <x:c r="D48" s="151" t="str">
-        <x:v>公司展示未独立复现；金额和客户收入未知</x:v>
+        <x:v>不是公司退出；但已无当前自研神经拟态芯片产品证据，不再计活跃芯片供应商</x:v>
       </x:c>
       <x:c r="E48" s="2"/>
       <x:c r="F48" s="2"/>
@@ -2572,18 +2662,18 @@
       <x:c r="N48" s="2"/>
       <x:c r="O48" s="2"/>
     </x:row>
-    <x:row r="49" ht="34" customHeight="1">
+    <x:row r="49" ht="82" customHeight="1">
       <x:c r="A49" s="151" t="str">
-        <x:v>World Labs → AMD</x:v>
+        <x:v>Videantis → Mythic</x:v>
       </x:c>
       <x:c r="B49" s="152" t="d">
-        <x:v>2026-09-26T00:00:00.000Z</x:v>
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C49" s="151" t="str">
-        <x:v>已签协议，预计年底完成</x:v>
+        <x:v>已完成</x:v>
       </x:c>
       <x:c r="D49" s="151" t="str">
-        <x:v>约82亿美元全股票；仍待监管与交割条件</x:v>
+        <x:v>Videantis既有装机不计Mythic模拟APU出货</x:v>
       </x:c>
       <x:c r="E49" s="2"/>
       <x:c r="F49" s="2"/>
@@ -2597,11 +2687,19 @@
       <x:c r="N49" s="2"/>
       <x:c r="O49" s="2"/>
     </x:row>
-    <x:row r="50">
-      <x:c r="A50"/>
-      <x:c r="B50"/>
-      <x:c r="C50"/>
-      <x:c r="D50"/>
+    <x:row r="50" ht="82" customHeight="1">
+      <x:c r="A50" s="151" t="str">
+        <x:v>SceniX → World Labs</x:v>
+      </x:c>
+      <x:c r="B50" s="152" t="d">
+        <x:v>2026-07-21T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C50" s="151" t="str">
+        <x:v>已并入；R2S2R机器人仿真链</x:v>
+      </x:c>
+      <x:c r="D50" s="151" t="str">
+        <x:v>公司展示未独立复现；金额和客户收入未知</x:v>
+      </x:c>
       <x:c r="E50" s="2"/>
       <x:c r="F50" s="2"/>
       <x:c r="G50" s="2"/>
@@ -2614,11 +2712,19 @@
       <x:c r="N50" s="2"/>
       <x:c r="O50" s="2"/>
     </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="2"/>
-      <x:c r="B51" s="2"/>
-      <x:c r="C51" s="2"/>
-      <x:c r="D51" s="2"/>
+    <x:row r="51" ht="82" customHeight="1">
+      <x:c r="A51" s="151" t="str">
+        <x:v>World Labs → AMD</x:v>
+      </x:c>
+      <x:c r="B51" s="152" t="d">
+        <x:v>2026-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C51" s="151" t="str">
+        <x:v>已签协议，预计年底完成</x:v>
+      </x:c>
+      <x:c r="D51" s="151" t="str">
+        <x:v>约82亿美元全股票；仍待监管与交割条件</x:v>
+      </x:c>
       <x:c r="E51" s="2"/>
       <x:c r="F51" s="2"/>
       <x:c r="G51" s="2"/>
@@ -2632,10 +2738,10 @@
       <x:c r="O51" s="2"/>
     </x:row>
     <x:row r="52">
-      <x:c r="A52" s="2"/>
-      <x:c r="B52" s="2"/>
-      <x:c r="C52" s="2"/>
-      <x:c r="D52" s="2"/>
+      <x:c r="A52"/>
+      <x:c r="B52"/>
+      <x:c r="C52"/>
+      <x:c r="D52"/>
       <x:c r="E52" s="2"/>
       <x:c r="F52" s="2"/>
       <x:c r="G52" s="2"/>
@@ -2649,10 +2755,10 @@
       <x:c r="O52" s="2"/>
     </x:row>
     <x:row r="53">
-      <x:c r="A53" s="2"/>
-      <x:c r="B53" s="2"/>
-      <x:c r="C53" s="2"/>
-      <x:c r="D53" s="2"/>
+      <x:c r="A53"/>
+      <x:c r="B53"/>
+      <x:c r="C53"/>
+      <x:c r="D53"/>
       <x:c r="E53" s="2"/>
       <x:c r="F53" s="2"/>
       <x:c r="G53" s="2"/>
@@ -2786,7 +2892,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R39bdcc3e8f274e8a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f845e5189884edf"/>
 </x:worksheet>
 </file>
 
@@ -2959,10 +3065,10 @@
         <x:v>事件视觉传感、软件、伙伴相机生态及Mantara整机</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>Sony IMX636／637伙伴相机已有现货、系列生产或发货证据。OpenMV同时列出400美元GENX320模组与500美元多光谱事件相机模组；后者把GENX320与1MP／120 FPS彩色全局快门传感器同步集成，检索时两款均售罄。6月推出Mantara与Hearth。</x:v>
+        <x:v>Sony IMX636／637伙伴相机已有现货、系列生产或发货证据。法国工商／BODACC转载记录显示公司于2024年10月进入司法重整，法院在2026年5月5日批准重整计划；6月15日公司宣布2000万欧元融资并推出Mantara与Hearth，转向事件传感器、软件和反无人机全栈系统。</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
-        <x:v>事件相机生态已越过样片，但商品页、价格和售罄状态不等于当前供货、销量、终端采用或Prophesee收入。多光谱模组证明事件流与彩色帧已有现成集成入口，不证明世界模型训练或SNN芯片采用；Mantara仅有公司现场验证口径。OpenEB仍公开，但公司已宣布OpenEB与独立Metavision SDK结束生命周期；Hearth公开迁移包和客户部署待核。</x:v>
+        <x:v>重整计划获批和融资说明公司继续经营，但融资不等于收入或经营风险消失。事件相机商品页、价格和伙伴发货不等于Prophesee传感器销量、终端采用或收入；Mantara商业化与现场验证为公司口径，缺具名采购、部署数量、合同和验收。OpenEB与独立Metavision SDK已宣布结束生命周期；Hearth公开迁移包仍未找到。</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
         <x:v>Prophesee、IDS、LUCID与OpenMV官方产品／商店页；Prophesee资源与迁移公告，检索2026-10-02；事实、厂商宣称、分析和未知分列</x:v>
@@ -4135,16 +4241,34 @@
       <x:c r="N38" s="2"/>
       <x:c r="O38" s="2"/>
     </x:row>
-    <x:row r="39" ht="92" customHeight="1">
-      <x:c r="A39" s="3"/>
-      <x:c r="B39" s="3"/>
-      <x:c r="C39" s="3"/>
-      <x:c r="D39" s="3"/>
-      <x:c r="E39" s="3"/>
-      <x:c r="F39" s="3"/>
-      <x:c r="G39" s="3"/>
-      <x:c r="H39" s="3"/>
-      <x:c r="I39" s="3"/>
+    <x:row r="39" ht="74" customHeight="1">
+      <x:c r="A39" s="3" t="str">
+        <x:v>C038</x:v>
+      </x:c>
+      <x:c r="B39" s="3" t="str">
+        <x:v>ModelCat（原Eta Compute）</x:v>
+      </x:c>
+      <x:c r="C39" s="3" t="str">
+        <x:v>相邻替代</x:v>
+      </x:c>
+      <x:c r="D39" s="3" t="str">
+        <x:v>硬件感知的边缘AI模型构建、重定向与实机验证软件</x:v>
+      </x:c>
+      <x:c r="E39" s="3" t="str">
+        <x:v>Eta Compute于2025年8月宣布更名ModelCat；当前官网和公司说明把核心定位转为AI-in-the-Loop模型构建平台。NXP官方资料将eIQ Model Creator列为ModelCat合作产品，并明确该工具采用订阅收费。</x:v>
+      </x:c>
+      <x:c r="F39" s="3" t="str">
+        <x:v>当前公开产品是软件平台，不是自研神经拟态芯片；历史ECM3532／TENSAI硅片不能当作当前芯片供应。订阅入口和合作关系不证明客户规模、收入或模型性能宣称。</x:v>
+      </x:c>
+      <x:c r="G39" s="3" t="str">
+        <x:v>ModelCat更名与当前产品说明、NXP eIQ FAQ；检索2026-10-02</x:v>
+      </x:c>
+      <x:c r="H39" s="3" t="str">
+        <x:v>https://modelcat.ai/blog/why-we-changed-our-name-to-modelcat</x:v>
+      </x:c>
+      <x:c r="I39" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J39" s="2"/>
       <x:c r="K39" s="2"/>
       <x:c r="L39" s="2"/>
@@ -4523,7 +4647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R54a83612ea1d4456"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a47bf84c9c4ec5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5918,17 +6042,37 @@
       <x:c r="N40" s="2"/>
       <x:c r="O40" s="2"/>
     </x:row>
-    <x:row r="41" ht="88" customHeight="1">
-      <x:c r="A41" s="3"/>
-      <x:c r="B41" s="3"/>
-      <x:c r="C41" s="3"/>
-      <x:c r="D41" s="3"/>
-      <x:c r="E41" s="3"/>
-      <x:c r="F41" s="3"/>
-      <x:c r="G41" s="3"/>
-      <x:c r="H41" s="3"/>
-      <x:c r="I41" s="3"/>
-      <x:c r="J41" s="3"/>
+    <x:row r="41" ht="68" customHeight="1">
+      <x:c r="A41" s="3" t="str">
+        <x:v>P040</x:v>
+      </x:c>
+      <x:c r="B41" s="3" t="str">
+        <x:v>ModelCat／NXP</x:v>
+      </x:c>
+      <x:c r="C41" s="3" t="str">
+        <x:v>eIQ Model Creator</x:v>
+      </x:c>
+      <x:c r="D41" s="3" t="str">
+        <x:v>开发平台</x:v>
+      </x:c>
+      <x:c r="E41" s="3" t="str">
+        <x:v>ModelCat官方发布与NXP eIQ资料交叉确认当前软件、支持NXP MCU／MPU系列及订阅收费入口</x:v>
+      </x:c>
+      <x:c r="F41" s="4" t="d">
+        <x:v>2025-09-09T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G41" s="4" t="d">
+        <x:v>2025-09-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H41" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I41" s="3" t="str">
+        <x:v>软件可用与订阅收费不等于已核客户数量或收入；生成模型指标为厂商宣称。ModelCat当前无自研SNN／类脑芯片证据</x:v>
+      </x:c>
+      <x:c r="J41" s="3" t="str">
+        <x:v>https://modelcat.ai/blog/modelcat-tm-launches-eiq-r-model-creator-to-turbocharge-ai-model-development-for-nxp-devices</x:v>
+      </x:c>
       <x:c r="K41" s="2"/>
       <x:c r="L41" s="2"/>
       <x:c r="M41" s="2"/>
@@ -6273,7 +6417,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfcf8c1dd5c1a47ab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R930963e0e9d74cf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6326,25 +6470,25 @@
     </x:row>
     <x:row r="2" ht="66" customHeight="1">
       <x:c r="A2" s="151" t="str">
-        <x:v>T018</x:v>
-      </x:c>
-      <x:c r="B2" s="152" t="str">
-        <x:v>2025-03（仅月份）</x:v>
+        <x:v>T028</x:v>
+      </x:c>
+      <x:c r="B2" s="152" t="d">
+        <x:v>2024-10-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C2" s="152" t="d">
-        <x:v>2025-06-04T00:00:00.000Z</x:v>
+        <x:v>2024-10-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D2" s="151" t="str">
-        <x:v>Sandia／SpiNNcloud</x:v>
+        <x:v>Prophesee</x:v>
       </x:c>
       <x:c r="E2" s="151" t="str">
-        <x:v>Braunfels到货并完成科研部署</x:v>
+        <x:v>法国法院启动司法重整程序</x:v>
       </x:c>
       <x:c r="F2" s="151" t="str">
-        <x:v>事件只确认月份；Sandia确认初始热流随机游走模拟。研究试验平台，不是终端规模量产或供应商收入</x:v>
+        <x:v>工商／BODACC转载记录确认2024-09-17停止付款、10月15日启动重整；2026-05-05法院批准重整计划。重整不等于清算或公司退出，融资与后续经营需分开记录</x:v>
       </x:c>
       <x:c r="G2" s="151" t="str">
-        <x:v>https://www.sandia.gov/research/news/brain-based-computing-for-nuclear-deterrence-solutions/</x:v>
+        <x:v>https://www.pappers.fr/entreprise/prophesee-800681892</x:v>
       </x:c>
       <x:c r="H2" s="2"/>
       <x:c r="I2" s="2"/>
@@ -6357,25 +6501,25 @@
     </x:row>
     <x:row r="3" ht="66" customHeight="1">
       <x:c r="A3" s="151" t="str">
-        <x:v>T012</x:v>
-      </x:c>
-      <x:c r="B3" s="152" t="d">
-        <x:v>2025-07-22T00:00:00.000Z</x:v>
+        <x:v>T018</x:v>
+      </x:c>
+      <x:c r="B3" s="152" t="str">
+        <x:v>2025-03（仅月份）</x:v>
       </x:c>
       <x:c r="C3" s="152" t="d">
-        <x:v>2025-07-22T00:00:00.000Z</x:v>
+        <x:v>2025-06-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D3" s="151" t="str">
-        <x:v>Hailo</x:v>
+        <x:v>Sandia／SpiNNcloud</x:v>
       </x:c>
       <x:c r="E3" s="151" t="str">
-        <x:v>Hailo-10H商业可用并接受全球订单</x:v>
+        <x:v>Braunfels到货并完成科研部署</x:v>
       </x:c>
       <x:c r="F3" s="151" t="str">
-        <x:v>厂商GA与订单入口；不等于终端设计定点、销量或收入</x:v>
+        <x:v>事件只确认月份；Sandia确认初始热流随机游走模拟。研究试验平台，不是终端规模量产或供应商收入</x:v>
       </x:c>
       <x:c r="G3" s="151" t="str">
-        <x:v>https://hailo.ai/company-overview/newsroom/news/hailo-announces-general-availability-of-hailo-10h-edge-ai-accelerator-with-generative-ai-capabilities/</x:v>
+        <x:v>https://www.sandia.gov/research/news/brain-based-computing-for-nuclear-deterrence-solutions/</x:v>
       </x:c>
       <x:c r="H3" s="2"/>
       <x:c r="I3" s="2"/>
@@ -6388,25 +6532,25 @@
     </x:row>
     <x:row r="4" ht="66" customHeight="1">
       <x:c r="A4" s="151" t="str">
-        <x:v>T019</x:v>
-      </x:c>
-      <x:c r="B4" s="152" t="str">
-        <x:v>2025-10（仅月份）</x:v>
+        <x:v>T012</x:v>
+      </x:c>
+      <x:c r="B4" s="152" t="d">
+        <x:v>2025-07-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C4" s="152" t="d">
-        <x:v>2025-10-28T00:00:00.000Z</x:v>
+        <x:v>2025-07-22T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D4" s="151" t="str">
-        <x:v>莱比锡大学／SpiNNcloud</x:v>
+        <x:v>Hailo</x:v>
       </x:c>
       <x:c r="E4" s="151" t="str">
-        <x:v>类脑科研系统投入运行</x:v>
+        <x:v>Hailo-10H商业可用并接受全球订单</x:v>
       </x:c>
       <x:c r="F4" s="151" t="str">
-        <x:v>事件只确认月份；约400万欧元为科研设施资助，不是采购额或供应商收入。药物项目采用int8 DNN，不能等同SNN片上学习</x:v>
+        <x:v>厂商GA与订单入口；不等于终端设计定点、销量或收入</x:v>
       </x:c>
       <x:c r="G4" s="151" t="str">
-        <x:v>https://www.uni-leipzig.de/newsdetail/artikel/vom-gehirn-inspiriert-supercomputer-staerkt-ki-forschung-an-der-universitaet-leipzig-2025-10-28</x:v>
+        <x:v>https://hailo.ai/company-overview/newsroom/news/hailo-announces-general-availability-of-hailo-10h-edge-ai-accelerator-with-generative-ai-capabilities/</x:v>
       </x:c>
       <x:c r="H4" s="2"/>
       <x:c r="I4" s="2"/>
@@ -6419,25 +6563,25 @@
     </x:row>
     <x:row r="5" ht="66" customHeight="1">
       <x:c r="A5" s="151" t="str">
-        <x:v>T001</x:v>
+        <x:v>T029</x:v>
       </x:c>
       <x:c r="B5" s="152" t="d">
-        <x:v>2026-02-04T00:00:00.000Z</x:v>
+        <x:v>2025-08-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C5" s="152" t="d">
-        <x:v>2026-02-04T00:00:00.000Z</x:v>
+        <x:v>2025-08-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D5" s="151" t="str">
-        <x:v>Honda／Mythic</x:v>
+        <x:v>Eta Compute／ModelCat</x:v>
       </x:c>
       <x:c r="E5" s="151" t="str">
-        <x:v>投资与车载SoC联合研发</x:v>
+        <x:v>更名并转向AI-in-the-Loop模型构建软件</x:v>
       </x:c>
       <x:c r="F5" s="151" t="str">
-        <x:v>未来联合研发，不是车型量产</x:v>
+        <x:v>当前ModelCat和NXP资料确认软件与订阅产品；历史超低功耗神经拟态芯片履历不能当作当前自研硅供应</x:v>
       </x:c>
       <x:c r="G5" s="151" t="str">
-        <x:v>https://global.honda/en/topics/2026/c_2026-02-04eng.html</x:v>
+        <x:v>https://modelcat.ai/blog/why-we-changed-our-name-to-modelcat</x:v>
       </x:c>
       <x:c r="H5" s="2"/>
       <x:c r="I5" s="2"/>
@@ -6450,25 +6594,25 @@
     </x:row>
     <x:row r="6" ht="66" customHeight="1">
       <x:c r="A6" s="151" t="str">
-        <x:v>T026</x:v>
-      </x:c>
-      <x:c r="B6" s="152" t="d">
-        <x:v>2026-02-25T00:00:00.000Z</x:v>
+        <x:v>T019</x:v>
+      </x:c>
+      <x:c r="B6" s="152" t="str">
+        <x:v>2025-10（仅月份）</x:v>
       </x:c>
       <x:c r="C6" s="152" t="d">
-        <x:v>2026-03-02T00:00:00.000Z</x:v>
+        <x:v>2025-10-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D6" s="151" t="str">
-        <x:v>Forschungszentrum Jülich／SpiNNcloud</x:v>
+        <x:v>莱比锡大学／SpiNNcloud</x:v>
       </x:c>
       <x:c r="E6" s="151" t="str">
-        <x:v>336万欧元SpiNNaker2公共采购合同签订</x:v>
+        <x:v>类脑科研系统投入运行</x:v>
       </x:c>
       <x:c r="F6" s="151" t="str">
-        <x:v>公共采购结果确认合同授予值、数量1套、单一投标且无分包；合同不等于已付款、交付验收或当期收入确认</x:v>
+        <x:v>事件只确认月份；约400万欧元为科研设施资助，不是采购额或供应商收入。药物项目采用int8 DNN，不能等同SNN片上学习</x:v>
       </x:c>
       <x:c r="G6" s="151" t="str">
-        <x:v>https://ted.europa.eu/en/notice/-/detail/141500-2026</x:v>
+        <x:v>https://www.uni-leipzig.de/newsdetail/artikel/vom-gehirn-inspiriert-supercomputer-staerkt-ki-forschung-an-der-universitaet-leipzig-2025-10-28</x:v>
       </x:c>
       <x:c r="H6" s="2"/>
       <x:c r="I6" s="2"/>
@@ -6481,25 +6625,25 @@
     </x:row>
     <x:row r="7" ht="66" customHeight="1">
       <x:c r="A7" s="151" t="str">
-        <x:v>T022</x:v>
+        <x:v>T001</x:v>
       </x:c>
       <x:c r="B7" s="152" t="d">
-        <x:v>2026-02-26T00:00:00.000Z</x:v>
+        <x:v>2026-02-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C7" s="152" t="d">
-        <x:v>2026-02-26T00:00:00.000Z</x:v>
+        <x:v>2026-02-04T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D7" s="151" t="str">
-        <x:v>Aspirare Semi</x:v>
+        <x:v>Honda／Mythic</x:v>
       </x:c>
       <x:c r="E7" s="151" t="str">
-        <x:v>模拟计算电路专利申请公开</x:v>
+        <x:v>投资与车载SoC联合研发</x:v>
       </x:c>
       <x:c r="F7" s="151" t="str">
-        <x:v>确认主体与知识产权路线，不证明ASIC实现、量产或收入</x:v>
+        <x:v>未来联合研发，不是车型量产</x:v>
       </x:c>
       <x:c r="G7" s="151" t="str">
-        <x:v>https://patents.google.com/patent/US20260057197A1/en</x:v>
+        <x:v>https://global.honda/en/topics/2026/c_2026-02-04eng.html</x:v>
       </x:c>
       <x:c r="H7" s="2"/>
       <x:c r="I7" s="2"/>
@@ -6512,25 +6656,25 @@
     </x:row>
     <x:row r="8" ht="66" customHeight="1">
       <x:c r="A8" s="151" t="str">
-        <x:v>T002</x:v>
+        <x:v>T026</x:v>
       </x:c>
       <x:c r="B8" s="152" t="d">
-        <x:v>2026-03-12T00:00:00.000Z</x:v>
+        <x:v>2026-02-25T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C8" s="152" t="d">
-        <x:v>2026-03-26T00:00:00.000Z</x:v>
+        <x:v>2026-03-02T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D8" s="151" t="str">
-        <x:v>Innatera／Joya</x:v>
+        <x:v>Forschungszentrum Jülich／SpiNNcloud</x:v>
       </x:c>
       <x:c r="E8" s="151" t="str">
-        <x:v>EdgeCore模块发布</x:v>
+        <x:v>336万欧元SpiNNaker2公共采购合同签订</x:v>
       </x:c>
       <x:c r="F8" s="151" t="str">
-        <x:v>可集成客户模块，销量未知</x:v>
+        <x:v>公共采购结果确认合同授予值、数量1套、单一投标且无分包；合同不等于已付款、交付验收或当期收入确认</x:v>
       </x:c>
       <x:c r="G8" s="151" t="str">
-        <x:v>https://www.innatera.com/newsroom/joya-design-takes-neuromorphic-chip-from-design-to-device-with-first-innatera-powered-consumer-audio-product-at-awe-china/</x:v>
+        <x:v>https://ted.europa.eu/en/notice/-/detail/141500-2026</x:v>
       </x:c>
       <x:c r="H8" s="2"/>
       <x:c r="I8" s="2"/>
@@ -6543,25 +6687,25 @@
     </x:row>
     <x:row r="9" ht="66" customHeight="1">
       <x:c r="A9" s="151" t="str">
-        <x:v>T021</x:v>
+        <x:v>T022</x:v>
       </x:c>
       <x:c r="B9" s="152" t="d">
-        <x:v>2026-03-17T00:00:00.000Z</x:v>
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C9" s="152" t="d">
-        <x:v>2026-03-17T00:00:00.000Z</x:v>
+        <x:v>2026-02-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D9" s="151" t="str">
-        <x:v>Mythic／Microchip SST</x:v>
+        <x:v>Aspirare Semi</x:v>
       </x:c>
       <x:c r="E9" s="151" t="str">
-        <x:v>下一代APU选择memBrain／SuperFlash</x:v>
+        <x:v>模拟计算电路专利申请公开</x:v>
       </x:c>
       <x:c r="F9" s="151" t="str">
-        <x:v>供应链／IP选型，不证明Vanguard流片、样片或交付；能效数字为厂商宣称</x:v>
+        <x:v>确认主体与知识产权路线，不证明ASIC实现、量产或收入</x:v>
       </x:c>
       <x:c r="G9" s="151" t="str">
-        <x:v>https://www.microchip.com/en-us/about/news-releases/products/mythic-selects-membrain-technology-from-sst-for-its-next-gen-ultra-low-power-apus</x:v>
+        <x:v>https://patents.google.com/patent/US20260057197A1/en</x:v>
       </x:c>
       <x:c r="H9" s="2"/>
       <x:c r="I9" s="2"/>
@@ -6574,23 +6718,25 @@
     </x:row>
     <x:row r="10" ht="66" customHeight="1">
       <x:c r="A10" s="151" t="str">
-        <x:v>T025</x:v>
+        <x:v>T002</x:v>
       </x:c>
       <x:c r="B10" s="152" t="d">
-        <x:v>2026-05-13T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C10" s="152"/>
+        <x:v>2026-03-12T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C10" s="152" t="d">
+        <x:v>2026-03-26T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="D10" s="151" t="str">
-        <x:v>Intel／Lava</x:v>
+        <x:v>Innatera／Joya</x:v>
       </x:c>
       <x:c r="E10" s="151" t="str">
-        <x:v>官方仓库归档、只读；下一代Loihi与新SDK在开发</x:v>
+        <x:v>EdgeCore模块发布</x:v>
       </x:c>
       <x:c r="F10" s="151" t="str">
-        <x:v>归档日期可核；README发布日期未知。新SDK为路线，未证明交付、量产或退出研究。</x:v>
+        <x:v>可集成客户模块，销量未知</x:v>
       </x:c>
       <x:c r="G10" s="151" t="str">
-        <x:v>https://github.com/lava-nc/lava</x:v>
+        <x:v>https://www.innatera.com/newsroom/joya-design-takes-neuromorphic-chip-from-design-to-device-with-first-innatera-powered-consumer-audio-product-at-awe-china/</x:v>
       </x:c>
       <x:c r="H10" s="2"/>
       <x:c r="I10" s="2"/>
@@ -6603,25 +6749,25 @@
     </x:row>
     <x:row r="11" ht="66" customHeight="1">
       <x:c r="A11" s="151" t="str">
-        <x:v>T003</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="B11" s="152" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
+        <x:v>2026-03-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C11" s="152" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
+        <x:v>2026-03-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D11" s="151" t="str">
-        <x:v>Mythic</x:v>
+        <x:v>Mythic／Microchip SST</x:v>
       </x:c>
       <x:c r="E11" s="151" t="str">
-        <x:v>收购Videantis</x:v>
+        <x:v>下一代APU选择memBrain／SuperFlash</x:v>
       </x:c>
       <x:c r="F11" s="151" t="str">
-        <x:v>被收购数字IP装机不计作模拟APU销量</x:v>
+        <x:v>供应链／IP选型，不证明Vanguard流片、样片或交付；能效数字为厂商宣称</x:v>
       </x:c>
       <x:c r="G11" s="151" t="str">
-        <x:v>https://www.mythic.ai/newsroom/Blog%20Post%20Title%20One-3zaa9-zlxng-67tfc-lbgbx</x:v>
+        <x:v>https://www.microchip.com/en-us/about/news-releases/products/mythic-selects-membrain-technology-from-sst-for-its-next-gen-ultra-low-power-apus</x:v>
       </x:c>
       <x:c r="H11" s="2"/>
       <x:c r="I11" s="2"/>
@@ -6634,25 +6780,23 @@
     </x:row>
     <x:row r="12" ht="66" customHeight="1">
       <x:c r="A12" s="151" t="str">
-        <x:v>T013</x:v>
+        <x:v>T025</x:v>
       </x:c>
       <x:c r="B12" s="152" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C12" s="152" t="d">
-        <x:v>2026-05-19T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>2026-05-13T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C12" s="152"/>
       <x:c r="D12" s="151" t="str">
-        <x:v>BrainChip／ASICLAND</x:v>
+        <x:v>Intel／Lava</x:v>
       </x:c>
       <x:c r="E12" s="151" t="str">
-        <x:v>签署Akida IP分销许可</x:v>
+        <x:v>官方仓库归档、只读；下一代Loihi与新SDK在开发</x:v>
       </x:c>
       <x:c r="F12" s="151" t="str">
-        <x:v>可做评估许可和MPW；客户生产许可需BrainChip另批并支付生产许可费，未披露金额或已确认收入</x:v>
+        <x:v>归档日期可核；README发布日期未知。新SDK为路线，未证明交付、量产或退出研究。</x:v>
       </x:c>
       <x:c r="G12" s="151" t="str">
-        <x:v>https://brainchip.com/press/brainchip-strikes-ip-licensing-deal-with-asicland/</x:v>
+        <x:v>https://github.com/lava-nc/lava</x:v>
       </x:c>
       <x:c r="H12" s="2"/>
       <x:c r="I12" s="2"/>
@@ -6665,25 +6809,25 @@
     </x:row>
     <x:row r="13" ht="66" customHeight="1">
       <x:c r="A13" s="151" t="str">
-        <x:v>T004</x:v>
+        <x:v>T003</x:v>
       </x:c>
       <x:c r="B13" s="152" t="d">
-        <x:v>2026-06-15T00:00:00.000Z</x:v>
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C13" s="152" t="d">
-        <x:v>2026-06-15T00:00:00.000Z</x:v>
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D13" s="151" t="str">
-        <x:v>Prophesee</x:v>
+        <x:v>Mythic</x:v>
       </x:c>
       <x:c r="E13" s="151" t="str">
-        <x:v>Mantara／Hearth发布</x:v>
+        <x:v>收购Videantis</x:v>
       </x:c>
       <x:c r="F13" s="151" t="str">
-        <x:v>厂商现场验证与软件迁移公告</x:v>
+        <x:v>被收购数字IP装机不计作模拟APU销量</x:v>
       </x:c>
       <x:c r="G13" s="151" t="str">
-        <x:v>https://www.prophesee.ai/2026/06/15/prophesee-launches-mantara-event-based-drone-detection/</x:v>
+        <x:v>https://www.mythic.ai/newsroom/Blog%20Post%20Title%20One-3zaa9-zlxng-67tfc-lbgbx</x:v>
       </x:c>
       <x:c r="H13" s="2"/>
       <x:c r="I13" s="2"/>
@@ -6696,25 +6840,25 @@
     </x:row>
     <x:row r="14" ht="66" customHeight="1">
       <x:c r="A14" s="151" t="str">
-        <x:v>T005</x:v>
+        <x:v>T013</x:v>
       </x:c>
       <x:c r="B14" s="152" t="d">
-        <x:v>2026-06-29T00:00:00.000Z</x:v>
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C14" s="152" t="d">
-        <x:v>2026-06-29T00:00:00.000Z</x:v>
+        <x:v>2026-05-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D14" s="151" t="str">
-        <x:v>Innatera</x:v>
+        <x:v>BrainChip／ASICLAND</x:v>
       </x:c>
       <x:c r="E14" s="151" t="str">
-        <x:v>Synfire 0.0.2 Beta发布</x:v>
+        <x:v>签署Akida IP分销许可</x:v>
       </x:c>
       <x:c r="F14" s="151" t="str">
-        <x:v>可安装，生产部署未知</x:v>
+        <x:v>可做评估许可和MPW；客户生产许可需BrainChip另批并支付生产许可费，未披露金额或已确认收入</x:v>
       </x:c>
       <x:c r="G14" s="151" t="str">
-        <x:v>https://pypi.org/project/synfire/</x:v>
+        <x:v>https://brainchip.com/press/brainchip-strikes-ip-licensing-deal-with-asicland/</x:v>
       </x:c>
       <x:c r="H14" s="2"/>
       <x:c r="I14" s="2"/>
@@ -6727,25 +6871,25 @@
     </x:row>
     <x:row r="15" ht="66" customHeight="1">
       <x:c r="A15" s="151" t="str">
-        <x:v>T023</x:v>
+        <x:v>T004</x:v>
       </x:c>
       <x:c r="B15" s="152" t="d">
-        <x:v>2026-07-16T00:00:00.000Z</x:v>
+        <x:v>2026-06-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C15" s="152" t="d">
-        <x:v>2026-07-16T00:00:00.000Z</x:v>
+        <x:v>2026-06-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D15" s="151" t="str">
-        <x:v>千觉机器人</x:v>
+        <x:v>Prophesee</x:v>
       </x:c>
       <x:c r="E15" s="151" t="str">
-        <x:v>发布X-TouchMind V1与TacVerse 1k</x:v>
+        <x:v>Mantara／Hearth发布并宣布2000万欧元融资</x:v>
       </x:c>
       <x:c r="F15" s="151" t="str">
-        <x:v>公司发布与展会演示；数据下载、权重、客户验收和收入未核</x:v>
+        <x:v>司法重整计划获批后，公司转向反无人机全栈系统并融资；现场验证、商业化与迁移兼容为厂商口径。融资不等于收入，未见具名采购、合同、验收或部署数量</x:v>
       </x:c>
       <x:c r="G15" s="151" t="str">
-        <x:v>https://www.xenserobotics.com/article/387/detail/25</x:v>
+        <x:v>https://www.prophesee.ai/2026/06/15/prophesee-launches-mantara-event-based-drone-detection/</x:v>
       </x:c>
       <x:c r="H15" s="2"/>
       <x:c r="I15" s="2"/>
@@ -6758,25 +6902,25 @@
     </x:row>
     <x:row r="16" ht="66" customHeight="1">
       <x:c r="A16" s="151" t="str">
-        <x:v>T010</x:v>
+        <x:v>T005</x:v>
       </x:c>
       <x:c r="B16" s="152" t="d">
-        <x:v>2026-07-17T00:00:00.000Z</x:v>
+        <x:v>2026-06-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C16" s="152" t="d">
-        <x:v>2026-07-17T00:00:00.000Z</x:v>
+        <x:v>2026-06-29T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D16" s="151" t="str">
-        <x:v>他山科技</x:v>
+        <x:v>Innatera</x:v>
       </x:c>
       <x:c r="E16" s="151" t="str">
-        <x:v>E10A动态触觉芯片公开发布／演示</x:v>
+        <x:v>Synfire 0.0.2 Beta发布</x:v>
       </x:c>
       <x:c r="F16" s="151" t="str">
-        <x:v>ASC转换为厂商披露，E10A量产未知</x:v>
+        <x:v>可安装，生产部署未知</x:v>
       </x:c>
       <x:c r="G16" s="151" t="str">
-        <x:v>https://www3.xinhuanet.com/tech/20260717/d66a7bb7dcf8414baeab73d6499b785e/c.html</x:v>
+        <x:v>https://pypi.org/project/synfire/</x:v>
       </x:c>
       <x:c r="H16" s="64"/>
       <x:c r="I16" s="65"/>
@@ -6789,25 +6933,25 @@
     </x:row>
     <x:row r="17" ht="66" customHeight="1">
       <x:c r="A17" s="151" t="str">
-        <x:v>T015</x:v>
+        <x:v>T023</x:v>
       </x:c>
       <x:c r="B17" s="152" t="d">
-        <x:v>2026-07-21T00:00:00.000Z</x:v>
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C17" s="152" t="d">
-        <x:v>2026-07-28T00:00:00.000Z</x:v>
+        <x:v>2026-07-16T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D17" s="151" t="str">
-        <x:v>World Labs／SceniX</x:v>
+        <x:v>千觉机器人</x:v>
       </x:c>
       <x:c r="E17" s="151" t="str">
-        <x:v>World Labs收购机器人仿真公司SceniX</x:v>
+        <x:v>发布X-TouchMind V1与TacVerse 1k</x:v>
       </x:c>
       <x:c r="F17" s="151" t="str">
-        <x:v>World Labs称SceniX R2S2R把真实任务转为可控仿真用于策略训练和评估；结果为公司展示，未独立复现，未披露交易金额或客户收入</x:v>
+        <x:v>公司发布与展会演示；数据下载、权重、客户验收和收入未核</x:v>
       </x:c>
       <x:c r="G17" s="151" t="str">
-        <x:v>https://www.worldlabs.ai/blog/real-to-sim-to-real</x:v>
+        <x:v>https://www.xenserobotics.com/article/387/detail/25</x:v>
       </x:c>
       <x:c r="H17" s="67"/>
       <x:c r="I17" s="68"/>
@@ -6820,25 +6964,25 @@
     </x:row>
     <x:row r="18" ht="66" customHeight="1">
       <x:c r="A18" s="151" t="str">
-        <x:v>T006</x:v>
+        <x:v>T010</x:v>
       </x:c>
       <x:c r="B18" s="152" t="d">
-        <x:v>2026-07-28T00:00:00.000Z</x:v>
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C18" s="152" t="d">
-        <x:v>2026-07-28T00:00:00.000Z</x:v>
+        <x:v>2026-07-17T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D18" s="151" t="str">
-        <x:v>BrainChip</x:v>
+        <x:v>他山科技</x:v>
       </x:c>
       <x:c r="E18" s="151" t="str">
-        <x:v>AKD1500 M.2模块可购</x:v>
+        <x:v>E10A动态触觉芯片公开发布／演示</x:v>
       </x:c>
       <x:c r="F18" s="151" t="str">
-        <x:v>开发模块，不等于终端销量</x:v>
+        <x:v>ASC转换为厂商披露，E10A量产未知</x:v>
       </x:c>
       <x:c r="G18" s="151" t="str">
-        <x:v>https://investor.brainchip.com/press/brainchip-akd1500-now-available-in-compact-m-2-form-factor-enabling-fanless-edge-ai-in-industrial-and-commercial-designs/</x:v>
+        <x:v>https://www3.xinhuanet.com/tech/20260717/d66a7bb7dcf8414baeab73d6499b785e/c.html</x:v>
       </x:c>
       <x:c r="H18" s="67"/>
       <x:c r="I18" s="68"/>
@@ -6851,25 +6995,25 @@
     </x:row>
     <x:row r="19" ht="66" customHeight="1">
       <x:c r="A19" s="151" t="str">
-        <x:v>T014</x:v>
+        <x:v>T015</x:v>
       </x:c>
       <x:c r="B19" s="152" t="d">
-        <x:v>2026-08-13T00:00:00.000Z</x:v>
+        <x:v>2026-07-21T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C19" s="152" t="d">
-        <x:v>2026-08-13T00:00:00.000Z</x:v>
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D19" s="151" t="str">
-        <x:v>BrainChip／Orama.AOI</x:v>
+        <x:v>World Labs／SceniX</x:v>
       </x:c>
       <x:c r="E19" s="151" t="str">
-        <x:v>发布工业检测参考部署合作</x:v>
+        <x:v>World Labs收购机器人仿真公司SceniX</x:v>
       </x:c>
       <x:c r="F19" s="151" t="str">
-        <x:v>伙伴称已优化模型并形成参考部署／生产就绪方案；未披露终端工厂、采购额、出货量或收入</x:v>
+        <x:v>World Labs称SceniX R2S2R把真实任务转为可控仿真用于策略训练和评估；结果为公司展示，未独立复现，未披露交易金额或客户收入</x:v>
       </x:c>
       <x:c r="G19" s="151" t="str">
-        <x:v>https://brainchip.com/press/brainchip-partners-with-orama-aoi-for-ai-fueled-defect-detection/</x:v>
+        <x:v>https://www.worldlabs.ai/blog/real-to-sim-to-real</x:v>
       </x:c>
       <x:c r="H19" s="67"/>
       <x:c r="I19" s="68"/>
@@ -6882,23 +7026,25 @@
     </x:row>
     <x:row r="20" ht="66" customHeight="1">
       <x:c r="A20" s="151" t="str">
-        <x:v>T024</x:v>
-      </x:c>
-      <x:c r="B20" s="152"/>
+        <x:v>T006</x:v>
+      </x:c>
+      <x:c r="B20" s="152" t="d">
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="C20" s="152" t="d">
-        <x:v>2026-08-24T00:00:00.000Z</x:v>
+        <x:v>2026-07-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D20" s="151" t="str">
-        <x:v>他山科技／E10A</x:v>
+        <x:v>BrainChip</x:v>
       </x:c>
       <x:c r="E20" s="151" t="str">
-        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
+        <x:v>AKD1500 M.2模块可购</x:v>
       </x:c>
       <x:c r="F20" s="151" t="str">
-        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
+        <x:v>开发模块，不等于终端销量</x:v>
       </x:c>
       <x:c r="G20" s="151" t="str">
-        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
+        <x:v>https://investor.brainchip.com/press/brainchip-akd1500-now-available-in-compact-m-2-form-factor-enabling-fanless-edge-ai-in-industrial-and-commercial-designs/</x:v>
       </x:c>
       <x:c r="H20" s="67"/>
       <x:c r="I20" s="68"/>
@@ -6911,23 +7057,25 @@
     </x:row>
     <x:row r="21" ht="66" customHeight="1">
       <x:c r="A21" s="151" t="str">
-        <x:v>T011</x:v>
-      </x:c>
-      <x:c r="B21" s="152"/>
+        <x:v>T014</x:v>
+      </x:c>
+      <x:c r="B21" s="152" t="d">
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="C21" s="152" t="d">
-        <x:v>2026-08-26T00:00:00.000Z</x:v>
+        <x:v>2026-08-13T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D21" s="151" t="str">
-        <x:v>奥比中光／他山</x:v>
+        <x:v>BrainChip／Orama.AOI</x:v>
       </x:c>
       <x:c r="E21" s="151" t="str">
-        <x:v>TS-ECHO视触无本体数采合作</x:v>
+        <x:v>发布工业检测参考部署合作</x:v>
       </x:c>
       <x:c r="F21" s="151" t="str">
-        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
+        <x:v>伙伴称已优化模型并形成参考部署／生产就绪方案；未披露终端工厂、采购额、出货量或收入</x:v>
       </x:c>
       <x:c r="G21" s="151" t="str">
-        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
+        <x:v>https://brainchip.com/press/brainchip-partners-with-orama-aoi-for-ai-fueled-defect-detection/</x:v>
       </x:c>
       <x:c r="H21" s="67"/>
       <x:c r="I21" s="68"/>
@@ -6940,25 +7088,23 @@
     </x:row>
     <x:row r="22" ht="66" customHeight="1">
       <x:c r="A22" s="151" t="str">
-        <x:v>T027</x:v>
-      </x:c>
-      <x:c r="B22" s="152" t="str">
-        <x:v>2026-08（仅月份）</x:v>
-      </x:c>
+        <x:v>T024</x:v>
+      </x:c>
+      <x:c r="B22" s="152"/>
       <x:c r="C22" s="152" t="d">
         <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D22" s="151" t="str">
-        <x:v>维泛智能</x:v>
+        <x:v>他山科技／E10A</x:v>
       </x:c>
       <x:c r="E22" s="151" t="str">
-        <x:v>披露过亿元种子+轮融资</x:v>
+        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
       </x:c>
       <x:c r="F22" s="151" t="str">
-        <x:v>据公司向钛媒体披露；与2026年5月数亿元种子轮分开。融资拟用于量产芯片、BrainOS与OmniRT产品化，不等于收入、量产或客户付款</x:v>
+        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
       </x:c>
       <x:c r="G22" s="151" t="str">
-        <x:v>https://www.tmtpost.com/8113528.html</x:v>
+        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
       </x:c>
       <x:c r="H22" s="67"/>
       <x:c r="I22" s="68"/>
@@ -6971,25 +7117,23 @@
     </x:row>
     <x:row r="23" ht="66" customHeight="1">
       <x:c r="A23" s="151" t="str">
-        <x:v>T007</x:v>
-      </x:c>
-      <x:c r="B23" s="152" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>T011</x:v>
+      </x:c>
+      <x:c r="B23" s="152"/>
       <x:c r="C23" s="152" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D23" s="151" t="str">
-        <x:v>MemryX／Express LUCK</x:v>
+        <x:v>奥比中光／他山</x:v>
       </x:c>
       <x:c r="E23" s="151" t="str">
-        <x:v>生产线部署</x:v>
+        <x:v>TS-ECHO视触无本体数采合作</x:v>
       </x:c>
       <x:c r="F23" s="151" t="str">
-        <x:v>具名部署联合稿，采购金额未知</x:v>
+        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
       </x:c>
       <x:c r="G23" s="151" t="str">
-        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
+        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
       </x:c>
       <x:c r="H23" s="67"/>
       <x:c r="I23" s="68"/>
@@ -7002,25 +7146,25 @@
     </x:row>
     <x:row r="24" ht="66" customHeight="1">
       <x:c r="A24" s="151" t="str">
-        <x:v>T017</x:v>
-      </x:c>
-      <x:c r="B24" s="152" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
+        <x:v>T027</x:v>
+      </x:c>
+      <x:c r="B24" s="152" t="str">
+        <x:v>2026-08（仅月份）</x:v>
       </x:c>
       <x:c r="C24" s="152" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D24" s="151" t="str">
-        <x:v>具脑磐石 EBKernel</x:v>
+        <x:v>维泛智能</x:v>
       </x:c>
       <x:c r="E24" s="151" t="str">
-        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
+        <x:v>披露过亿元种子+轮融资</x:v>
       </x:c>
       <x:c r="F24" s="151" t="str">
-        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
+        <x:v>据公司向钛媒体披露；与2026年5月数亿元种子轮分开。融资拟用于量产芯片、BrainOS与OmniRT产品化，不等于收入、量产或客户付款</x:v>
       </x:c>
       <x:c r="G24" s="151" t="str">
-        <x:v>https://www.ebkernel.com/</x:v>
+        <x:v>https://www.tmtpost.com/8113528.html</x:v>
       </x:c>
       <x:c r="H24" s="67"/>
       <x:c r="I24" s="68"/>
@@ -7033,25 +7177,25 @@
     </x:row>
     <x:row r="25" ht="66" customHeight="1">
       <x:c r="A25" s="151" t="str">
-        <x:v>T008</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="B25" s="152" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C25" s="152" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D25" s="151" t="str">
-        <x:v>AnalogAI</x:v>
+        <x:v>MemryX／Express LUCK</x:v>
       </x:c>
       <x:c r="E25" s="151" t="str">
-        <x:v>选用SST memBrain SAGE IP</x:v>
+        <x:v>生产线部署</x:v>
       </x:c>
       <x:c r="F25" s="151" t="str">
-        <x:v>IP选型，无流片证据</x:v>
+        <x:v>具名部署联合稿，采购金额未知</x:v>
       </x:c>
       <x:c r="G25" s="151" t="str">
-        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
+        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
       </x:c>
       <x:c r="H25" s="67"/>
       <x:c r="I25" s="68"/>
@@ -7064,23 +7208,25 @@
     </x:row>
     <x:row r="26" ht="66" customHeight="1">
       <x:c r="A26" s="151" t="str">
-        <x:v>T020</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="B26" s="152" t="d">
-        <x:v>2026-09-23T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C26" s="152"/>
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C26" s="152" t="d">
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="D26" s="151" t="str">
-        <x:v>SpiNNcloud／py-spinnaker2</x:v>
+        <x:v>具脑磐石 EBKernel</x:v>
       </x:c>
       <x:c r="E26" s="151" t="str">
-        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
+        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
       </x:c>
       <x:c r="F26" s="151" t="str">
-        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
+        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
       </x:c>
       <x:c r="G26" s="151" t="str">
-        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
+        <x:v>https://www.ebkernel.com/</x:v>
       </x:c>
       <x:c r="H26" s="67"/>
       <x:c r="I26" s="68"/>
@@ -7093,25 +7239,25 @@
     </x:row>
     <x:row r="27" ht="66" customHeight="1">
       <x:c r="A27" s="151" t="str">
-        <x:v>T016</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="B27" s="152" t="d">
-        <x:v>2026-09-26T00:00:00.000Z</x:v>
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C27" s="152" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D27" s="151" t="str">
-        <x:v>AMD／World Labs</x:v>
+        <x:v>AnalogAI</x:v>
       </x:c>
       <x:c r="E27" s="151" t="str">
-        <x:v>签署约82亿美元全股票收购协议</x:v>
+        <x:v>选用SST memBrain SAGE IP</x:v>
       </x:c>
       <x:c r="F27" s="151" t="str">
-        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
+        <x:v>IP选型，无流片证据</x:v>
       </x:c>
       <x:c r="G27" s="151" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
+        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
       </x:c>
       <x:c r="H27" s="67"/>
       <x:c r="I27" s="68"/>
@@ -7124,25 +7270,23 @@
     </x:row>
     <x:row r="28" ht="66" customHeight="1">
       <x:c r="A28" s="151" t="str">
-        <x:v>T009</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="B28" s="152" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C28" s="152" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>2026-09-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C28" s="152"/>
       <x:c r="D28" s="151" t="str">
-        <x:v>POLYN</x:v>
+        <x:v>SpiNNcloud／py-spinnaker2</x:v>
       </x:c>
       <x:c r="E28" s="151" t="str">
-        <x:v>TMS工程节点供客户评估</x:v>
+        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
       </x:c>
       <x:c r="F28" s="151" t="str">
-        <x:v>未具名评估方，非量产</x:v>
+        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
       </x:c>
       <x:c r="G28" s="151" t="str">
-        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
       </x:c>
       <x:c r="H28" s="67"/>
       <x:c r="I28" s="68"/>
@@ -7153,14 +7297,28 @@
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="2"/>
     </x:row>
-    <x:row r="29" ht="30" customHeight="1">
-      <x:c r="A29" s="78"/>
-      <x:c r="B29" s="79"/>
-      <x:c r="C29" s="79"/>
-      <x:c r="D29" s="80"/>
-      <x:c r="E29" s="80"/>
-      <x:c r="F29" s="80"/>
-      <x:c r="G29" s="80"/>
+    <x:row r="29" ht="66" customHeight="1">
+      <x:c r="A29" s="78" t="str">
+        <x:v>T016</x:v>
+      </x:c>
+      <x:c r="B29" s="83" t="d">
+        <x:v>2026-09-26T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C29" s="83" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D29" s="80" t="str">
+        <x:v>AMD／World Labs</x:v>
+      </x:c>
+      <x:c r="E29" s="80" t="str">
+        <x:v>签署约82亿美元全股票收购协议</x:v>
+      </x:c>
+      <x:c r="F29" s="80" t="str">
+        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
+      </x:c>
+      <x:c r="G29" s="80" t="str">
+        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
+      </x:c>
       <x:c r="H29" s="67"/>
       <x:c r="I29" s="68"/>
       <x:c r="J29" s="2"/>
@@ -7170,16 +7328,28 @@
       <x:c r="N29" s="2"/>
       <x:c r="O29" s="2"/>
     </x:row>
-    <x:row r="30" ht="30" customHeight="1">
+    <x:row r="30" ht="66" customHeight="1">
       <x:c r="A30" s="102" t="str">
-        <x:v>半年收入</x:v>
-      </x:c>
-      <x:c r="B30" s="103"/>
-      <x:c r="C30" s="103"/>
-      <x:c r="D30" s="104"/>
-      <x:c r="E30" s="80"/>
-      <x:c r="F30" s="80"/>
-      <x:c r="G30" s="80"/>
+        <x:v>T009</x:v>
+      </x:c>
+      <x:c r="B30" s="123" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C30" s="123" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D30" s="104" t="str">
+        <x:v>POLYN</x:v>
+      </x:c>
+      <x:c r="E30" s="80" t="str">
+        <x:v>TMS工程节点供客户评估</x:v>
+      </x:c>
+      <x:c r="F30" s="80" t="str">
+        <x:v>未具名评估方，非量产</x:v>
+      </x:c>
+      <x:c r="G30" s="80" t="str">
+        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+      </x:c>
       <x:c r="H30" s="67"/>
       <x:c r="I30" s="68"/>
       <x:c r="J30" s="2"/>
@@ -7190,18 +7360,10 @@
       <x:c r="O30" s="2"/>
     </x:row>
     <x:row r="31" ht="28" customHeight="1">
-      <x:c r="A31" s="153" t="str">
-        <x:v>构成</x:v>
-      </x:c>
-      <x:c r="B31" s="154" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C31" s="154" t="str">
-        <x:v>2026 H1</x:v>
-      </x:c>
-      <x:c r="D31" s="155" t="str">
-        <x:v>来源</x:v>
-      </x:c>
+      <x:c r="A31" s="168"/>
+      <x:c r="B31" s="169"/>
+      <x:c r="C31" s="169"/>
+      <x:c r="D31" s="170"/>
       <x:c r="E31" s="80"/>
       <x:c r="F31" s="80"/>
       <x:c r="G31" s="80"/>
@@ -7215,18 +7377,12 @@
       <x:c r="O31" s="2"/>
     </x:row>
     <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="78" t="str">
-        <x:v>许可</x:v>
-      </x:c>
-      <x:c r="B32" s="79" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C32" s="79" t="n">
-        <x:v>613826</x:v>
-      </x:c>
-      <x:c r="D32" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
-      </x:c>
+      <x:c r="A32" s="102" t="str">
+        <x:v>半年收入</x:v>
+      </x:c>
+      <x:c r="B32" s="103"/>
+      <x:c r="C32" s="103"/>
+      <x:c r="D32" s="104"/>
       <x:c r="E32" s="80"/>
       <x:c r="F32" s="80"/>
       <x:c r="G32" s="80"/>
@@ -7239,18 +7395,18 @@
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="2"/>
     </x:row>
-    <x:row r="33" ht="26" customHeight="1">
-      <x:c r="A33" s="78" t="str">
-        <x:v>产品</x:v>
-      </x:c>
-      <x:c r="B33" s="79" t="n">
-        <x:v>19184</x:v>
-      </x:c>
-      <x:c r="C33" s="79" t="n">
-        <x:v>110362</x:v>
-      </x:c>
-      <x:c r="D33" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
+    <x:row r="33" ht="28" customHeight="1">
+      <x:c r="A33" s="178" t="str">
+        <x:v>构成</x:v>
+      </x:c>
+      <x:c r="B33" s="179" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C33" s="179" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D33" s="180" t="str">
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="E33" s="80"/>
       <x:c r="F33" s="80"/>
@@ -7266,13 +7422,13 @@
     </x:row>
     <x:row r="34" ht="26" customHeight="1">
       <x:c r="A34" s="78" t="str">
-        <x:v>开发服务</x:v>
+        <x:v>许可</x:v>
       </x:c>
       <x:c r="B34" s="79" t="n">
-        <x:v>1004395</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C34" s="79" t="n">
-        <x:v>498557</x:v>
+        <x:v>613826</x:v>
       </x:c>
       <x:c r="D34" s="80" t="str">
         <x:v>半年报Note 3</x:v>
@@ -7291,18 +7447,16 @@
     </x:row>
     <x:row r="35" ht="26" customHeight="1">
       <x:c r="A35" s="76" t="str">
-        <x:v>合计</x:v>
+        <x:v>产品</x:v>
       </x:c>
       <x:c r="B35" s="86" t="n">
-        <x:f>SUM(B32:B34)</x:f>
-        <x:v>1023579</x:v>
+        <x:v>19184</x:v>
       </x:c>
       <x:c r="C35" s="86" t="n">
-        <x:f>SUM(C32:C34)</x:f>
-        <x:v>1222745</x:v>
+        <x:v>110362</x:v>
       </x:c>
       <x:c r="D35" s="77" t="str">
-        <x:v>监管半年报</x:v>
+        <x:v>半年报Note 3</x:v>
       </x:c>
       <x:c r="E35" s="77"/>
       <x:c r="F35" s="77"/>
@@ -7316,11 +7470,19 @@
       <x:c r="N35" s="2"/>
       <x:c r="O35" s="2"/>
     </x:row>
-    <x:row r="36" ht="72" customHeight="1">
-      <x:c r="A36" s="78"/>
-      <x:c r="B36" s="80"/>
-      <x:c r="C36" s="80"/>
-      <x:c r="D36" s="83"/>
+    <x:row r="36" ht="26" customHeight="1">
+      <x:c r="A36" s="78" t="str">
+        <x:v>开发服务</x:v>
+      </x:c>
+      <x:c r="B36" s="79" t="n">
+        <x:v>1004395</x:v>
+      </x:c>
+      <x:c r="C36" s="79" t="n">
+        <x:v>498557</x:v>
+      </x:c>
+      <x:c r="D36" s="83" t="str">
+        <x:v>半年报Note 3</x:v>
+      </x:c>
       <x:c r="E36" s="80"/>
       <x:c r="F36" s="80"/>
       <x:c r="G36" s="80"/>
@@ -7333,18 +7495,20 @@
       <x:c r="N36" s="2"/>
       <x:c r="O36" s="2"/>
     </x:row>
-    <x:row r="37" ht="28" customHeight="1">
-      <x:c r="A37" s="153" t="str">
-        <x:v>现金与客户指标</x:v>
-      </x:c>
-      <x:c r="B37" s="155" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C37" s="155" t="str">
-        <x:v>2026 H1</x:v>
-      </x:c>
-      <x:c r="D37" s="156" t="str">
-        <x:v>边界</x:v>
+    <x:row r="37" ht="26" customHeight="1">
+      <x:c r="A37" s="132" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B37" s="134" t="n">
+        <x:f>SUM(B34:B36)</x:f>
+        <x:v>1023579</x:v>
+      </x:c>
+      <x:c r="C37" s="134" t="n">
+        <x:f>SUM(C34:C36)</x:f>
+        <x:v>1222745</x:v>
+      </x:c>
+      <x:c r="D37" s="124" t="str">
+        <x:v>监管半年报</x:v>
       </x:c>
       <x:c r="E37" s="118"/>
       <x:c r="F37" s="118"/>
@@ -7359,18 +7523,10 @@
       <x:c r="O37" s="2"/>
     </x:row>
     <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="78" t="str">
-        <x:v>客户收款</x:v>
-      </x:c>
-      <x:c r="B38" s="79" t="n">
-        <x:v>1522026</x:v>
-      </x:c>
-      <x:c r="C38" s="79" t="n">
-        <x:v>813247</x:v>
-      </x:c>
-      <x:c r="D38" s="83" t="str">
-        <x:v>现金流，不等于收入</x:v>
-      </x:c>
+      <x:c r="A38" s="78"/>
+      <x:c r="B38" s="79"/>
+      <x:c r="C38" s="79"/>
+      <x:c r="D38" s="83"/>
       <x:c r="E38" s="80"/>
       <x:c r="F38" s="80"/>
       <x:c r="G38" s="80"/>
@@ -7383,18 +7539,18 @@
       <x:c r="N38" s="2"/>
       <x:c r="O38" s="2"/>
     </x:row>
-    <x:row r="39" ht="30" customHeight="1">
-      <x:c r="A39" s="78" t="str">
-        <x:v>经营现金净流出</x:v>
-      </x:c>
-      <x:c r="B39" s="79" t="n">
-        <x:v>6990176</x:v>
-      </x:c>
-      <x:c r="C39" s="79" t="n">
-        <x:v>11253495</x:v>
-      </x:c>
-      <x:c r="D39" s="83" t="str">
-        <x:v>按流出绝对值展示</x:v>
+    <x:row r="39" ht="28" customHeight="1">
+      <x:c r="A39" s="178" t="str">
+        <x:v>现金与客户指标</x:v>
+      </x:c>
+      <x:c r="B39" s="179" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C39" s="179" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D39" s="182" t="str">
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="E39" s="80"/>
       <x:c r="F39" s="80"/>
@@ -7410,16 +7566,16 @@
     </x:row>
     <x:row r="40" ht="30" customHeight="1">
       <x:c r="A40" s="78" t="str">
-        <x:v>期末现金及现金等价物</x:v>
+        <x:v>客户收款</x:v>
       </x:c>
       <x:c r="B40" s="79" t="n">
-        <x:v>13458121</x:v>
+        <x:v>1522026</x:v>
       </x:c>
       <x:c r="C40" s="79" t="n">
-        <x:v>20304971</x:v>
+        <x:v>813247</x:v>
       </x:c>
       <x:c r="D40" s="80" t="str">
-        <x:v>各年6月30日</x:v>
+        <x:v>现金流，不等于收入</x:v>
       </x:c>
       <x:c r="E40" s="80"/>
       <x:c r="F40" s="80"/>
@@ -7435,16 +7591,16 @@
     </x:row>
     <x:row r="41" ht="30" customHeight="1">
       <x:c r="A41" s="132" t="str">
-        <x:v>&gt;10%客户收入合计</x:v>
+        <x:v>经营现金净流出</x:v>
       </x:c>
       <x:c r="B41" s="134" t="n">
-        <x:v>809706</x:v>
+        <x:v>6990176</x:v>
       </x:c>
       <x:c r="C41" s="134" t="n">
-        <x:v>983780</x:v>
+        <x:v>11253495</x:v>
       </x:c>
       <x:c r="D41" s="133" t="str">
-        <x:v>2026约占H1收入80.5%</x:v>
+        <x:v>按流出绝对值展示</x:v>
       </x:c>
       <x:c r="E41" s="80"/>
       <x:c r="F41" s="80"/>
@@ -7460,14 +7616,16 @@
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="105" t="str">
-        <x:v>首批AKD1500生产批次</x:v>
-      </x:c>
-      <x:c r="B42" s="79"/>
+        <x:v>期末现金及现金等价物</x:v>
+      </x:c>
+      <x:c r="B42" s="79" t="n">
+        <x:v>13458121</x:v>
+      </x:c>
       <x:c r="C42" s="79" t="n">
-        <x:v>2000</x:v>
+        <x:v>20304971</x:v>
       </x:c>
       <x:c r="D42" s="80" t="str">
-        <x:v>颗；公司收到，不是客户出货</x:v>
+        <x:v>各年6月30日</x:v>
       </x:c>
       <x:c r="E42" s="80"/>
       <x:c r="F42" s="80"/>
@@ -7481,11 +7639,19 @@
       <x:c r="N42" s="2"/>
       <x:c r="O42" s="2"/>
     </x:row>
-    <x:row r="43" ht="44" customHeight="1">
-      <x:c r="A43" s="105"/>
-      <x:c r="B43" s="80"/>
-      <x:c r="C43" s="80"/>
-      <x:c r="D43" s="83"/>
+    <x:row r="43" ht="30" customHeight="1">
+      <x:c r="A43" s="105" t="str">
+        <x:v>&gt;10%客户收入合计</x:v>
+      </x:c>
+      <x:c r="B43" s="79" t="n">
+        <x:v>809706</x:v>
+      </x:c>
+      <x:c r="C43" s="79" t="n">
+        <x:v>983780</x:v>
+      </x:c>
+      <x:c r="D43" s="83" t="str">
+        <x:v>2026约占H1收入80.5%</x:v>
+      </x:c>
       <x:c r="E43" s="80"/>
       <x:c r="F43" s="80"/>
       <x:c r="G43" s="80"/>
@@ -7498,15 +7664,17 @@
       <x:c r="N43" s="2"/>
       <x:c r="O43" s="2"/>
     </x:row>
-    <x:row r="44" ht="34" customHeight="1">
+    <x:row r="44" ht="30" customHeight="1">
       <x:c r="A44" s="105" t="str">
-        <x:v>来源</x:v>
-      </x:c>
-      <x:c r="B44" s="80" t="str">
-        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
-      </x:c>
-      <x:c r="C44" s="80"/>
-      <x:c r="D44" s="83"/>
+        <x:v>首批AKD1500生产批次</x:v>
+      </x:c>
+      <x:c r="B44" s="79"/>
+      <x:c r="C44" s="79" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D44" s="83" t="str">
+        <x:v>颗；公司收到，不是客户出货</x:v>
+      </x:c>
       <x:c r="E44" s="80"/>
       <x:c r="F44" s="80"/>
       <x:c r="G44" s="80"/>
@@ -7520,12 +7688,8 @@
       <x:c r="O44" s="2"/>
     </x:row>
     <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="106" t="str">
-        <x:v>边界</x:v>
-      </x:c>
-      <x:c r="B45" s="107" t="str">
-        <x:v>BrainChip财务数据来自监管半年报；SpiNNcloud 336万欧元为公共采购合同授予值，不计入BrainChip收入图，也不等于SpiNNcloud已付款或确认收入。</x:v>
-      </x:c>
+      <x:c r="A45" s="106"/>
+      <x:c r="B45" s="107"/>
       <x:c r="C45" s="107"/>
       <x:c r="D45" s="125"/>
       <x:c r="E45" s="107"/>
@@ -7540,9 +7704,13 @@
       <x:c r="N45" s="2"/>
       <x:c r="O45" s="2"/>
     </x:row>
-    <x:row r="46" ht="64" customHeight="1">
-      <x:c r="A46" s="4"/>
-      <x:c r="B46" s="3"/>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="4" t="str">
+        <x:v>来源</x:v>
+      </x:c>
+      <x:c r="B46" s="3" t="str">
+        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
+      </x:c>
       <x:c r="C46" s="3"/>
       <x:c r="D46" s="4"/>
       <x:c r="E46" s="3"/>
@@ -7557,34 +7725,20 @@
       <x:c r="N46" s="2"/>
       <x:c r="O46" s="2"/>
     </x:row>
-    <x:row r="47" ht="64" customHeight="1">
+    <x:row r="47" ht="34" customHeight="1">
       <x:c r="A47" s="4" t="str">
-        <x:v>研究编号</x:v>
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>研究主体</x:v>
-      </x:c>
-      <x:c r="C47" s="3" t="str">
-        <x:v>路线</x:v>
-      </x:c>
-      <x:c r="D47" s="4" t="str">
-        <x:v>发布日期</x:v>
-      </x:c>
-      <x:c r="E47" s="3" t="str">
-        <x:v>证据类型</x:v>
-      </x:c>
-      <x:c r="F47" s="3" t="str">
-        <x:v>作者报告指标</x:v>
-      </x:c>
-      <x:c r="G47" s="3" t="str">
-        <x:v>边界</x:v>
-      </x:c>
-      <x:c r="H47" s="3" t="str">
-        <x:v>原始URL</x:v>
-      </x:c>
-      <x:c r="I47" s="4" t="str">
-        <x:v>检索日期</x:v>
-      </x:c>
+        <x:v>BrainChip财务数据来自监管半年报；SpiNNcloud 336万欧元为公共采购合同授予值，不计入BrainChip收入图，也不等于SpiNNcloud已付款或确认收入。</x:v>
+      </x:c>
+      <x:c r="C47" s="3"/>
+      <x:c r="D47" s="4"/>
+      <x:c r="E47" s="3"/>
+      <x:c r="F47" s="3"/>
+      <x:c r="G47" s="3"/>
+      <x:c r="H47" s="3"/>
+      <x:c r="I47" s="4"/>
       <x:c r="J47" s="2"/>
       <x:c r="K47" s="2"/>
       <x:c r="L47" s="2"/>
@@ -7593,33 +7747,15 @@
       <x:c r="O47" s="2"/>
     </x:row>
     <x:row r="48" ht="82" customHeight="1">
-      <x:c r="A48" s="3" t="str">
-        <x:v>R001</x:v>
-      </x:c>
-      <x:c r="B48" s="3" t="str">
-        <x:v>GelNeuro／中科院自动化所</x:v>
-      </x:c>
-      <x:c r="C48" s="3" t="str">
-        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
-      </x:c>
-      <x:c r="D48" s="4" t="d">
-        <x:v>2026-07-06T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="E48" s="3" t="str">
-        <x:v>作者预印本实机研究结果，未独立复现</x:v>
-      </x:c>
-      <x:c r="F48" s="3" t="str">
-        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
-      </x:c>
-      <x:c r="G48" s="3" t="str">
-        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
-      </x:c>
-      <x:c r="H48" s="3" t="str">
-        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
-      </x:c>
-      <x:c r="I48" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
-      </x:c>
+      <x:c r="A48" s="3"/>
+      <x:c r="B48" s="3"/>
+      <x:c r="C48" s="3"/>
+      <x:c r="D48" s="4"/>
+      <x:c r="E48" s="3"/>
+      <x:c r="F48" s="3"/>
+      <x:c r="G48" s="3"/>
+      <x:c r="H48" s="3"/>
+      <x:c r="I48" s="4"/>
       <x:c r="J48" s="2"/>
       <x:c r="K48" s="2"/>
       <x:c r="L48" s="2"/>
@@ -7629,31 +7765,31 @@
     </x:row>
     <x:row r="49" ht="82" customHeight="1">
       <x:c r="A49" s="3" t="str">
-        <x:v>R002</x:v>
+        <x:v>研究编号</x:v>
       </x:c>
       <x:c r="B49" s="3" t="str">
-        <x:v>SpikingTac／中科院自动化所</x:v>
+        <x:v>研究主体</x:v>
       </x:c>
       <x:c r="C49" s="3" t="str">
-        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
-      </x:c>
-      <x:c r="D49" s="4" t="d">
-        <x:v>2026-02-27T00:00:00.000Z</x:v>
+        <x:v>路线</x:v>
+      </x:c>
+      <x:c r="D49" s="4" t="str">
+        <x:v>发布日期</x:v>
       </x:c>
       <x:c r="E49" s="3" t="str">
-        <x:v>作者预印本研究样机，未独立复现</x:v>
+        <x:v>证据类型</x:v>
       </x:c>
       <x:c r="F49" s="3" t="str">
-        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
+        <x:v>作者报告指标</x:v>
       </x:c>
       <x:c r="G49" s="3" t="str">
-        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="H49" s="3" t="str">
-        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
-      </x:c>
-      <x:c r="I49" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>原始URL</x:v>
+      </x:c>
+      <x:c r="I49" s="4" t="str">
+        <x:v>检索日期</x:v>
       </x:c>
       <x:c r="J49" s="2"/>
       <x:c r="K49" s="2"/>
@@ -7664,28 +7800,28 @@
     </x:row>
     <x:row r="50" ht="82" customHeight="1">
       <x:c r="A50" s="3" t="str">
-        <x:v>R003</x:v>
+        <x:v>R001</x:v>
       </x:c>
       <x:c r="B50" s="3" t="str">
-        <x:v>OmniVTA／NUS、CASIA等</x:v>
+        <x:v>GelNeuro／中科院自动化所</x:v>
       </x:c>
       <x:c r="C50" s="3" t="str">
-        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
+        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
       </x:c>
       <x:c r="D50" s="4" t="d">
-        <x:v>2026-03-19T00:00:00.000Z</x:v>
+        <x:v>2026-07-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E50" s="3" t="str">
-        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
+        <x:v>作者预印本实机研究结果，未独立复现</x:v>
       </x:c>
       <x:c r="F50" s="3" t="str">
-        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
+        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
       </x:c>
       <x:c r="G50" s="3" t="str">
-        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
+        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
       </x:c>
       <x:c r="H50" s="3" t="str">
-        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
+        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
       </x:c>
       <x:c r="I50" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7699,28 +7835,28 @@
     </x:row>
     <x:row r="51" ht="82" customHeight="1">
       <x:c r="A51" s="3" t="str">
-        <x:v>R004</x:v>
+        <x:v>R002</x:v>
       </x:c>
       <x:c r="B51" s="3" t="str">
-        <x:v>Event-VLA／上海科技大学等</x:v>
+        <x:v>SpikingTac／中科院自动化所</x:v>
       </x:c>
       <x:c r="C51" s="3" t="str">
-        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
+        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
       </x:c>
       <x:c r="D51" s="4" t="d">
-        <x:v>2026-06-28T00:00:00.000Z</x:v>
+        <x:v>2026-02-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E51" s="3" t="str">
-        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
+        <x:v>作者预印本研究样机，未独立复现</x:v>
       </x:c>
       <x:c r="F51" s="3" t="str">
-        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
+        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
       </x:c>
       <x:c r="G51" s="3" t="str">
-        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
+        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
       </x:c>
       <x:c r="H51" s="3" t="str">
-        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
+        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
       </x:c>
       <x:c r="I51" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7734,28 +7870,28 @@
     </x:row>
     <x:row r="52" ht="82" customHeight="1">
       <x:c r="A52" s="4" t="str">
-        <x:v>R005</x:v>
+        <x:v>R003</x:v>
       </x:c>
       <x:c r="B52" s="3" t="str">
-        <x:v>TouchWorld／研究团队</x:v>
+        <x:v>OmniVTA／NUS、CASIA等</x:v>
       </x:c>
       <x:c r="C52" s="3" t="str">
-        <x:v>预测式＋反应式触觉基础模型</x:v>
+        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
       </x:c>
       <x:c r="D52" s="4" t="d">
-        <x:v>2026-07-08T00:00:00.000Z</x:v>
+        <x:v>2026-03-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E52" s="3" t="str">
-        <x:v>作者预印本研究；未独立复现</x:v>
+        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
       </x:c>
       <x:c r="F52" s="3" t="str">
-        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
+        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
       </x:c>
       <x:c r="G52" s="3" t="str">
-        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
+        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
       </x:c>
       <x:c r="H52" s="3" t="str">
-        <x:v>https://arxiv.org/abs/2607.07287</x:v>
+        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
       </x:c>
       <x:c r="I52" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7769,28 +7905,28 @@
     </x:row>
     <x:row r="53" ht="82" customHeight="1">
       <x:c r="A53" s="4" t="str">
-        <x:v>R006</x:v>
+        <x:v>R004</x:v>
       </x:c>
       <x:c r="B53" s="3" t="str">
-        <x:v>CLP-SNN／LMU、Intel等</x:v>
+        <x:v>Event-VLA／上海科技大学等</x:v>
       </x:c>
       <x:c r="C53" s="3" t="str">
-        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
       </x:c>
       <x:c r="D53" s="4" t="d">
-        <x:v>2026-05-05T00:00:00.000Z</x:v>
+        <x:v>2026-06-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E53" s="3" t="str">
-        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
       </x:c>
       <x:c r="F53" s="3" t="str">
-        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
       </x:c>
       <x:c r="G53" s="3" t="str">
-        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
       </x:c>
       <x:c r="H53" s="3" t="str">
-        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
       </x:c>
       <x:c r="I53" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7802,16 +7938,34 @@
       <x:c r="N53" s="2"/>
       <x:c r="O53" s="2"/>
     </x:row>
-    <x:row r="54" ht="50" customHeight="1">
-      <x:c r="A54" s="11"/>
-      <x:c r="B54" s="2"/>
-      <x:c r="C54" s="2"/>
-      <x:c r="D54" s="2"/>
-      <x:c r="E54" s="2"/>
-      <x:c r="F54" s="2"/>
-      <x:c r="G54" s="2"/>
-      <x:c r="H54" s="2"/>
-      <x:c r="I54" s="2"/>
+    <x:row r="54" ht="82" customHeight="1">
+      <x:c r="A54" s="4" t="str">
+        <x:v>R005</x:v>
+      </x:c>
+      <x:c r="B54" s="3" t="str">
+        <x:v>TouchWorld／研究团队</x:v>
+      </x:c>
+      <x:c r="C54" s="3" t="str">
+        <x:v>预测式＋反应式触觉基础模型</x:v>
+      </x:c>
+      <x:c r="D54" s="4" t="d">
+        <x:v>2026-07-08T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E54" s="3" t="str">
+        <x:v>作者预印本研究；未独立复现</x:v>
+      </x:c>
+      <x:c r="F54" s="3" t="str">
+        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
+      </x:c>
+      <x:c r="G54" s="3" t="str">
+        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
+      </x:c>
+      <x:c r="H54" s="3" t="str">
+        <x:v>https://arxiv.org/abs/2607.07287</x:v>
+      </x:c>
+      <x:c r="I54" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J54" s="2"/>
       <x:c r="K54" s="2"/>
       <x:c r="L54" s="2"/>
@@ -7819,16 +7973,34 @@
       <x:c r="N54" s="2"/>
       <x:c r="O54" s="2"/>
     </x:row>
-    <x:row r="55" ht="50" customHeight="1">
-      <x:c r="A55" s="11"/>
-      <x:c r="B55" s="2"/>
-      <x:c r="C55" s="2"/>
-      <x:c r="D55" s="2"/>
-      <x:c r="E55" s="2"/>
-      <x:c r="F55" s="2"/>
-      <x:c r="G55" s="2"/>
-      <x:c r="H55" s="2"/>
-      <x:c r="I55" s="2"/>
+    <x:row r="55" ht="82" customHeight="1">
+      <x:c r="A55" s="4" t="str">
+        <x:v>R006</x:v>
+      </x:c>
+      <x:c r="B55" s="3" t="str">
+        <x:v>CLP-SNN／LMU、Intel等</x:v>
+      </x:c>
+      <x:c r="C55" s="3" t="str">
+        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+      </x:c>
+      <x:c r="D55" s="4" t="d">
+        <x:v>2026-05-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E55" s="3" t="str">
+        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+      </x:c>
+      <x:c r="F55" s="3" t="str">
+        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+      </x:c>
+      <x:c r="G55" s="3" t="str">
+        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+      </x:c>
+      <x:c r="H55" s="3" t="str">
+        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+      </x:c>
+      <x:c r="I55" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J55" s="2"/>
       <x:c r="K55" s="2"/>
       <x:c r="L55" s="2"/>
@@ -7924,8 +8096,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra950f82ed62346bc"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0c7a631d9754f9a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56888d6d35b443b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra53cf51e3d8840a5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Akida multi-card orchestration evidence
Update the mobile report, traceable data and workbook to 38 companies, 42 product records and 30 events. Add Symphony Community Akida Bundle and AkidaTag with deployment, pre-order and revenue boundaries.
</commit_message>
<xml_diff>
--- a/market-evidence.xlsx
+++ b/market-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="R537b605574be4760"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="Raff751be60c14ce2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="R7a810256b33f471f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="R7bedf60f1bec451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="Ra8714f0ffee949fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="R95736d4aaddf4fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="Rf867912933864b09"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="Rbfc9847b51f04f85"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,7 +21,7 @@
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
     <x:numFmt numFmtId="202" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="10">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -68,8 +68,14 @@
       <x:color rgb="FF222222"/>
       <x:name val="Noto Sans SC"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Noto Sans SC"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="28">
+  <x:fills count="32">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -206,6 +212,26 @@
         <x:fgColor rgb="FF23445C"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F6C8A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF23445C"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="9">
     <x:border/>
@@ -241,7 +267,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="186">
+  <x:cellXfs count="205">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -714,6 +740,55 @@
     <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="3" fillId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1259,7 +1334,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3bba0f9f16954405"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R70da2afa31b54948"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1289,7 +1364,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4b7f94dbe09b4ab0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1b4b96a18045418b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1319,7 +1394,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3549f9c9096d4b63"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd82942c26f9416c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1346,7 +1421,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J41" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductEvidence" displayName="ProductEvidence" ref="A1:J43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1364,7 +1439,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G30" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="事件日期"/>
@@ -1379,7 +1454,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A49:I55" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A50:I56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="研究编号"/>
     <x:tableColumn id="2" name="研究主体"/>
@@ -1642,7 +1717,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-02小公司、退出收购与路线转向复核。38个主体、40组产品、29项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
+        <x:v>2026-10-03核心SNN、多卡调度与常开感知复核。38个主体、42组产品、30项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -1837,8 +1912,8 @@
         <x:v>方案／研发</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A13)</x:f>
-        <x:v>7</x:v>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A13)</x:f>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="2"/>
       <x:c r="D13" s="2"/>
@@ -1859,7 +1934,7 @@
         <x:v>研究／原型</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A14)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A14)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C14" s="2"/>
@@ -1881,7 +1956,7 @@
         <x:v>工程样片</x:v>
       </x:c>
       <x:c r="B15" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A15)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A15)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C15" s="2"/>
@@ -1903,7 +1978,7 @@
         <x:v>IP／商务接洽</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A16)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A16)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C16" s="2"/>
@@ -1925,8 +2000,8 @@
         <x:v>开发平台</x:v>
       </x:c>
       <x:c r="B17" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A17)</x:f>
-        <x:v>2</x:v>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A17)</x:f>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C17" s="2"/>
       <x:c r="D17" s="2"/>
@@ -1947,7 +2022,7 @@
         <x:v>客户评估／模块</x:v>
       </x:c>
       <x:c r="B18" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A18)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A18)</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="C18" s="2"/>
@@ -1969,7 +2044,7 @@
         <x:v>可采购硬件</x:v>
       </x:c>
       <x:c r="B19" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A19)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A19)</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="2"/>
@@ -1991,7 +2066,7 @@
         <x:v>商品页／售罄</x:v>
       </x:c>
       <x:c r="B20" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A20)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A20)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C20" s="2"/>
@@ -2013,7 +2088,7 @@
         <x:v>生产／部署声明</x:v>
       </x:c>
       <x:c r="B21" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A21)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A21)</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="C21" s="2"/>
@@ -2035,7 +2110,7 @@
         <x:v>发布／演示</x:v>
       </x:c>
       <x:c r="B22" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A22)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A22)</x:f>
         <x:v>2</x:v>
       </x:c>
       <x:c r="C22" s="2"/>
@@ -2057,7 +2132,7 @@
         <x:v>已签公共采购合同／科研部署</x:v>
       </x:c>
       <x:c r="B23" s="2" t="n">
-        <x:f>COUNTIF('产品阶段'!$D$2:$D$41,A23)</x:f>
+        <x:f>COUNTIF('产品阶段'!$D$2:$D$43,A23)</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="C23" s="2"/>
@@ -2121,15 +2196,15 @@
         <x:v>许可</x:v>
       </x:c>
       <x:c r="B26" s="5" t="n">
-        <x:f>'事件与财务'!B34</x:f>
+        <x:f>'事件与财务'!B35</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="C26" s="5" t="n">
-        <x:f>'事件与财务'!C34</x:f>
+        <x:f>'事件与财务'!C35</x:f>
         <x:v>613826</x:v>
       </x:c>
       <x:c r="D26" s="6" t="n">
-        <x:f>C26/'事件与财务'!C37</x:f>
+        <x:f>C26/'事件与财务'!C38</x:f>
         <x:v>0.5020065508343932</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
@@ -2149,15 +2224,15 @@
         <x:v>产品</x:v>
       </x:c>
       <x:c r="B27" s="5" t="n">
-        <x:f>'事件与财务'!B35</x:f>
+        <x:f>'事件与财务'!B36</x:f>
         <x:v>19184</x:v>
       </x:c>
       <x:c r="C27" s="5" t="n">
-        <x:f>'事件与财务'!C35</x:f>
+        <x:f>'事件与财务'!C36</x:f>
         <x:v>110362</x:v>
       </x:c>
       <x:c r="D27" s="6" t="n">
-        <x:f>C27/'事件与财务'!C37</x:f>
+        <x:f>C27/'事件与财务'!C38</x:f>
         <x:v>0.09025757619127454</x:v>
       </x:c>
       <x:c r="E27" s="2"/>
@@ -2177,15 +2252,15 @@
         <x:v>开发服务</x:v>
       </x:c>
       <x:c r="B28" s="5" t="n">
-        <x:f>'事件与财务'!B36</x:f>
+        <x:f>'事件与财务'!B37</x:f>
         <x:v>1004395</x:v>
       </x:c>
       <x:c r="C28" s="5" t="n">
-        <x:f>'事件与财务'!C36</x:f>
+        <x:f>'事件与财务'!C37</x:f>
         <x:v>498557</x:v>
       </x:c>
       <x:c r="D28" s="6" t="n">
-        <x:f>C28/'事件与财务'!C37</x:f>
+        <x:f>C28/'事件与财务'!C38</x:f>
         <x:v>0.40773587297433234</x:v>
       </x:c>
       <x:c r="E28" s="2"/>
@@ -2421,16 +2496,16 @@
       <x:c r="O38" s="2"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
-      <x:c r="A39" s="185" t="str">
+      <x:c r="A39" s="204" t="str">
         <x:v>可核商业化合同</x:v>
       </x:c>
-      <x:c r="B39" s="185" t="str">
+      <x:c r="B39" s="204" t="str">
         <x:v>签约日</x:v>
       </x:c>
-      <x:c r="C39" s="185" t="str">
+      <x:c r="C39" s="204" t="str">
         <x:v>合同授予值</x:v>
       </x:c>
-      <x:c r="D39" s="185" t="str">
+      <x:c r="D39" s="204" t="str">
         <x:v>边界</x:v>
       </x:c>
       <x:c r="E39" s="2"/>
@@ -2513,16 +2588,16 @@
       <x:c r="O42" s="2"/>
     </x:row>
     <x:row r="43" ht="42" customHeight="1">
-      <x:c r="A43" s="185" t="str">
+      <x:c r="A43" s="204" t="str">
         <x:v>并购与退出追溯</x:v>
       </x:c>
-      <x:c r="B43" s="185" t="str">
+      <x:c r="B43" s="204" t="str">
         <x:v>日期</x:v>
       </x:c>
-      <x:c r="C43" s="185" t="str">
+      <x:c r="C43" s="204" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="D43" s="185" t="str">
+      <x:c r="D43" s="204" t="str">
         <x:v>证据边界</x:v>
       </x:c>
       <x:c r="E43" s="2"/>
@@ -2892,7 +2967,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f845e5189884edf"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda340d1e09ab4669"/>
 </x:worksheet>
 </file>
 
@@ -2957,22 +3032,22 @@
         <x:v>硬件与平台</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>全数字事件驱动Akida；芯片、M.2／PCIe模块、第三方开发板及IP</x:v>
+        <x:v>全数字事件驱动Akida；芯片、M.2／PCIe模块、第三方开发板、开放调度软件及IP</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>监管半年报确认首批2,000颗AKD1500已收货并进入商业规模制造；最终产量因良率低于预期预计略低于计划。ASICLAND取得非独家IP分销许可，Orama.AOI被公司称为工业检测参考部署。</x:v>
+        <x:v>监管半年报确认首批2,000颗AKD1500已收货并进入商业规模制造；最终产量因良率低于预期预计略低于计划。2026年8月20日发布Apache 2.0许可的Symphony Community Akida Bundle，可在IBM Spectrum Symphony Community Edition下调度多张Akida卡；9月公开AkidaTag预订入口。</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
-        <x:v>2,000颗是BrainChip收到的首批生产批次，不是已核实客户出货；良率问题仍在分析。ASICLAND的生产许可需逐客户另行批准并付费；Orama为伙伴公告，未披露终端工厂、订单、数量或收入。AKD1500单独收入、版税和客户名单未知。</x:v>
+        <x:v>2,000颗是BrainChip收到的首批生产批次，不是已核实客户出货；良率问题仍在分析。Symphony代码与参考机结果可查，但属于BrainChip维护的社区包，不是IBM产品公告，也未披露企业客户部署、合同或收入。AkidaTag仍为预订／早期接入，价格、交付时间、硬件配置和客户未知。</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>BrainChip 2026半年报（监管文件、独立审阅）及ASICLAND／Orama官方公告；事实、发行人宣称和分析边界分列</x:v>
+        <x:v>BrainChip 2026半年报（监管文件、独立审阅）、BrainChip官方发布、公开GitHub仓库及IBM Community技术博客；事实、发行人宣称和分析边界分列</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
         <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
       </x:c>
       <x:c r="I2" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J2" s="2"/>
       <x:c r="K2" s="2"/>
@@ -4647,7 +4722,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0a47bf84c9c4ec5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf45ebfc9427f4f76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6079,34 +6154,70 @@
       <x:c r="N41" s="2"/>
       <x:c r="O41" s="2"/>
     </x:row>
-    <x:row r="42" ht="88" customHeight="1">
-      <x:c r="A42" s="3"/>
-      <x:c r="B42" s="3"/>
-      <x:c r="C42" s="3"/>
-      <x:c r="D42" s="3"/>
-      <x:c r="E42" s="3"/>
-      <x:c r="F42" s="3"/>
-      <x:c r="G42" s="3"/>
-      <x:c r="H42" s="3"/>
-      <x:c r="I42" s="3"/>
-      <x:c r="J42" s="3"/>
+    <x:row r="42" ht="68" customHeight="1">
+      <x:c r="A42" s="3" t="str">
+        <x:v>P041</x:v>
+      </x:c>
+      <x:c r="B42" s="3" t="str">
+        <x:v>BrainChip</x:v>
+      </x:c>
+      <x:c r="C42" s="3" t="str">
+        <x:v>Symphony Community Akida Bundle</x:v>
+      </x:c>
+      <x:c r="D42" s="3" t="str">
+        <x:v>开发平台</x:v>
+      </x:c>
+      <x:c r="E42" s="3" t="str">
+        <x:v>BrainChip发布＋Apache 2.0公开仓库＋IBM Community技术博客交叉确认</x:v>
+      </x:c>
+      <x:c r="F42" s="4" t="d">
+        <x:v>2026-08-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="G42" s="4" t="d">
+        <x:v>2026-08-20T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="H42" s="4" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I42" s="3" t="str">
+        <x:v>公开代码要求真实Akida硬件并给出8张AKD1500 M.2参考机配置；性能与精度来自公司参考机，未独立复现。社区包不是IBM产品公告，也未见企业客户、合同、SLA或收入</x:v>
+      </x:c>
+      <x:c r="J42" s="3" t="str">
+        <x:v>https://github.com/Brainchip-Inc/symphony-akida</x:v>
+      </x:c>
       <x:c r="K42" s="2"/>
       <x:c r="L42" s="2"/>
       <x:c r="M42" s="2"/>
       <x:c r="N42" s="2"/>
       <x:c r="O42" s="2"/>
     </x:row>
-    <x:row r="43" ht="88" customHeight="1">
-      <x:c r="A43" s="3"/>
-      <x:c r="B43" s="3"/>
-      <x:c r="C43" s="3"/>
-      <x:c r="D43" s="3"/>
-      <x:c r="E43" s="3"/>
-      <x:c r="F43" s="3"/>
-      <x:c r="G43" s="3"/>
-      <x:c r="H43" s="3"/>
-      <x:c r="I43" s="3"/>
-      <x:c r="J43" s="3"/>
+    <x:row r="43" ht="68" customHeight="1">
+      <x:c r="A43" s="3" t="str">
+        <x:v>P042</x:v>
+      </x:c>
+      <x:c r="B43" s="3" t="str">
+        <x:v>BrainChip</x:v>
+      </x:c>
+      <x:c r="C43" s="3" t="str">
+        <x:v>AkidaTag常开感知平台</x:v>
+      </x:c>
+      <x:c r="D43" s="3" t="str">
+        <x:v>方案／研发</x:v>
+      </x:c>
+      <x:c r="E43" s="3" t="str">
+        <x:v>公司产品页与预订入口；页面标注2026-09-29更新</x:v>
+      </x:c>
+      <x:c r="F43" s="4"/>
+      <x:c r="G43" s="4"/>
+      <x:c r="H43" s="4" t="d">
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="I43" s="3" t="str">
+        <x:v>当前仅可预订／申请早期接入；厂商宣称支持常开多模态和本地自学习，尚未核到价格、交付时间、完整硬件配置、第三方实测、具名客户或收入</x:v>
+      </x:c>
+      <x:c r="J43" s="3" t="str">
+        <x:v>https://brainchip.com/akida-tag/</x:v>
+      </x:c>
       <x:c r="K43" s="2"/>
       <x:c r="L43" s="2"/>
       <x:c r="M43" s="2"/>
@@ -6417,7 +6528,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R930963e0e9d74cf2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f61a696b93e45f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7088,23 +7199,25 @@
     </x:row>
     <x:row r="22" ht="66" customHeight="1">
       <x:c r="A22" s="151" t="str">
-        <x:v>T024</x:v>
-      </x:c>
-      <x:c r="B22" s="152"/>
+        <x:v>T030</x:v>
+      </x:c>
+      <x:c r="B22" s="152" t="d">
+        <x:v>2026-08-20T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="C22" s="152" t="d">
-        <x:v>2026-08-24T00:00:00.000Z</x:v>
+        <x:v>2026-08-20T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D22" s="151" t="str">
-        <x:v>他山科技／E10A</x:v>
+        <x:v>BrainChip／Symphony Community Akida Bundle</x:v>
       </x:c>
       <x:c r="E22" s="151" t="str">
-        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
+        <x:v>发布面向多卡Akida的开源异构调度软件包</x:v>
       </x:c>
       <x:c r="F22" s="151" t="str">
-        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
+        <x:v>官方发布与公开仓库确认Apache-2.0代码、8张AKD1500 M.2加3张AKD1000 PCIe参考配置及三类演示；当前仓库明确要求真实Akida硬件，结果为厂商参考复现而非独立基准。IBM Community文章仅为社区作者交叉说明，不等于IBM产品采用；未披露企业客户部署、付费合同、SLA或收入</x:v>
       </x:c>
       <x:c r="G22" s="151" t="str">
-        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
+        <x:v>https://brainchip.com/press/brainchip-launches-symphony-community-edition-akida-bundle/</x:v>
       </x:c>
       <x:c r="H22" s="67"/>
       <x:c r="I22" s="68"/>
@@ -7117,23 +7230,23 @@
     </x:row>
     <x:row r="23" ht="66" customHeight="1">
       <x:c r="A23" s="151" t="str">
-        <x:v>T011</x:v>
+        <x:v>T024</x:v>
       </x:c>
       <x:c r="B23" s="152"/>
       <x:c r="C23" s="152" t="d">
-        <x:v>2026-08-26T00:00:00.000Z</x:v>
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D23" s="151" t="str">
-        <x:v>奥比中光／他山</x:v>
+        <x:v>他山科技／E10A</x:v>
       </x:c>
       <x:c r="E23" s="151" t="str">
-        <x:v>TS-ECHO视触无本体数采合作</x:v>
+        <x:v>公司人员称E10A已完成流片并联合开发感控灵巧手</x:v>
       </x:c>
       <x:c r="F23" s="151" t="str">
-        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
+        <x:v>媒体采访转述；流片不等于回片、工程样片、客户验证、量产或收入</x:v>
       </x:c>
       <x:c r="G23" s="151" t="str">
-        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
+        <x:v>https://caifuhao.eastmoney.com/news/20260824025726767924920</x:v>
       </x:c>
       <x:c r="H23" s="67"/>
       <x:c r="I23" s="68"/>
@@ -7146,25 +7259,23 @@
     </x:row>
     <x:row r="24" ht="66" customHeight="1">
       <x:c r="A24" s="151" t="str">
-        <x:v>T027</x:v>
-      </x:c>
-      <x:c r="B24" s="152" t="str">
-        <x:v>2026-08（仅月份）</x:v>
-      </x:c>
+        <x:v>T011</x:v>
+      </x:c>
+      <x:c r="B24" s="152"/>
       <x:c r="C24" s="152" t="d">
-        <x:v>2026-08-24T00:00:00.000Z</x:v>
+        <x:v>2026-08-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D24" s="151" t="str">
-        <x:v>维泛智能</x:v>
+        <x:v>奥比中光／他山</x:v>
       </x:c>
       <x:c r="E24" s="151" t="str">
-        <x:v>披露过亿元种子+轮融资</x:v>
+        <x:v>TS-ECHO视触无本体数采合作</x:v>
       </x:c>
       <x:c r="F24" s="151" t="str">
-        <x:v>据公司向钛媒体披露；与2026年5月数亿元种子轮分开。融资拟用于量产芯片、BrainOS与OmniRT产品化，不等于收入、量产或客户付款</x:v>
+        <x:v>合作方确认签约，具体签约日未知；非验收／付费交付</x:v>
       </x:c>
       <x:c r="G24" s="151" t="str">
-        <x:v>https://www.tmtpost.com/8113528.html</x:v>
+        <x:v>https://www.orbbec.com/news/orbbec-and-tashan-technology-form-strategic-partnership-to-advance-vision-tactile-data-collection-solutions/</x:v>
       </x:c>
       <x:c r="H24" s="67"/>
       <x:c r="I24" s="68"/>
@@ -7177,25 +7288,25 @@
     </x:row>
     <x:row r="25" ht="66" customHeight="1">
       <x:c r="A25" s="151" t="str">
-        <x:v>T007</x:v>
-      </x:c>
-      <x:c r="B25" s="152" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
+        <x:v>T027</x:v>
+      </x:c>
+      <x:c r="B25" s="152" t="str">
+        <x:v>2026-08（仅月份）</x:v>
       </x:c>
       <x:c r="C25" s="152" t="d">
-        <x:v>2026-08-31T00:00:00.000Z</x:v>
+        <x:v>2026-08-24T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D25" s="151" t="str">
-        <x:v>MemryX／Express LUCK</x:v>
+        <x:v>维泛智能</x:v>
       </x:c>
       <x:c r="E25" s="151" t="str">
-        <x:v>生产线部署</x:v>
+        <x:v>披露过亿元种子+轮融资</x:v>
       </x:c>
       <x:c r="F25" s="151" t="str">
-        <x:v>具名部署联合稿，采购金额未知</x:v>
+        <x:v>据公司向钛媒体披露；与2026年5月数亿元种子轮分开。融资拟用于量产芯片、BrainOS与OmniRT产品化，不等于收入、量产或客户付款</x:v>
       </x:c>
       <x:c r="G25" s="151" t="str">
-        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
+        <x:v>https://www.tmtpost.com/8113528.html</x:v>
       </x:c>
       <x:c r="H25" s="67"/>
       <x:c r="I25" s="68"/>
@@ -7208,25 +7319,25 @@
     </x:row>
     <x:row r="26" ht="66" customHeight="1">
       <x:c r="A26" s="151" t="str">
-        <x:v>T017</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="B26" s="152" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C26" s="152" t="d">
-        <x:v>2026-09-14T00:00:00.000Z</x:v>
+        <x:v>2026-08-31T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D26" s="151" t="str">
-        <x:v>具脑磐石 EBKernel</x:v>
+        <x:v>MemryX／Express LUCK</x:v>
       </x:c>
       <x:c r="E26" s="151" t="str">
-        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
+        <x:v>生产线部署</x:v>
       </x:c>
       <x:c r="F26" s="151" t="str">
-        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
+        <x:v>具名部署联合稿，采购金额未知</x:v>
       </x:c>
       <x:c r="G26" s="151" t="str">
-        <x:v>https://www.ebkernel.com/</x:v>
+        <x:v>https://memryx.ai/news/express-luck-selects-memryx-for-ai-enabled-smart-manufacturing-operations/</x:v>
       </x:c>
       <x:c r="H26" s="67"/>
       <x:c r="I26" s="68"/>
@@ -7239,25 +7350,25 @@
     </x:row>
     <x:row r="27" ht="66" customHeight="1">
       <x:c r="A27" s="151" t="str">
-        <x:v>T008</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="B27" s="152" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C27" s="152" t="d">
-        <x:v>2026-09-15T00:00:00.000Z</x:v>
+        <x:v>2026-09-14T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D27" s="151" t="str">
-        <x:v>AnalogAI</x:v>
+        <x:v>具脑磐石 EBKernel</x:v>
       </x:c>
       <x:c r="E27" s="151" t="str">
-        <x:v>选用SST memBrain SAGE IP</x:v>
+        <x:v>Cog-WM 1.0发布并公开四种交付形态</x:v>
       </x:c>
       <x:c r="F27" s="151" t="str">
-        <x:v>IP选型，无流片证据</x:v>
+        <x:v>官网明确许可、模组、行业方案和RaaS；客户现场为公司／媒体宣称，未披露具名付费客户、合同、验收或收入，节能幅度未实测</x:v>
       </x:c>
       <x:c r="G27" s="151" t="str">
-        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
+        <x:v>https://www.ebkernel.com/</x:v>
       </x:c>
       <x:c r="H27" s="67"/>
       <x:c r="I27" s="68"/>
@@ -7270,23 +7381,25 @@
     </x:row>
     <x:row r="28" ht="66" customHeight="1">
       <x:c r="A28" s="151" t="str">
-        <x:v>T020</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="B28" s="152" t="d">
-        <x:v>2026-09-23T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C28" s="152"/>
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C28" s="152" t="d">
+        <x:v>2026-09-15T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="D28" s="151" t="str">
-        <x:v>SpiNNcloud／py-spinnaker2</x:v>
+        <x:v>AnalogAI</x:v>
       </x:c>
       <x:c r="E28" s="151" t="str">
-        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
+        <x:v>选用SST memBrain SAGE IP</x:v>
       </x:c>
       <x:c r="F28" s="151" t="str">
-        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
+        <x:v>IP选型，无流片证据</x:v>
       </x:c>
       <x:c r="G28" s="151" t="str">
-        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
+        <x:v>https://ir.microchip.com/news-events/press-releases/detail/1414/analogai-selects-membrain-sage-intellectual-property-from-silicon-storage-technology-for-its-first-real-world-edge-ai-processors</x:v>
       </x:c>
       <x:c r="H28" s="67"/>
       <x:c r="I28" s="68"/>
@@ -7299,25 +7412,23 @@
     </x:row>
     <x:row r="29" ht="66" customHeight="1">
       <x:c r="A29" s="78" t="str">
-        <x:v>T016</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="B29" s="83" t="d">
-        <x:v>2026-09-26T00:00:00.000Z</x:v>
-      </x:c>
-      <x:c r="C29" s="83" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
-      </x:c>
+        <x:v>2026-09-23T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C29" s="83"/>
       <x:c r="D29" s="80" t="str">
-        <x:v>AMD／World Labs</x:v>
+        <x:v>SpiNNcloud／py-spinnaker2</x:v>
       </x:c>
       <x:c r="E29" s="80" t="str">
-        <x:v>签署约82亿美元全股票收购协议</x:v>
+        <x:v>v0.8.2标签记录首次公开Docker镜像</x:v>
       </x:c>
       <x:c r="F29" s="80" t="str">
-        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
+        <x:v>日期是标签关联提交日期；发布说明、当前文档和Docker Hub确认公开镜像存在，未核首个实际推送日，未复现规模化训练</x:v>
       </x:c>
       <x:c r="G29" s="80" t="str">
-        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
+        <x:v>https://gitlab.com/spinnaker2/py-spinnaker2/-/tags</x:v>
       </x:c>
       <x:c r="H29" s="67"/>
       <x:c r="I29" s="68"/>
@@ -7330,25 +7441,25 @@
     </x:row>
     <x:row r="30" ht="66" customHeight="1">
       <x:c r="A30" s="102" t="str">
-        <x:v>T009</x:v>
+        <x:v>T016</x:v>
       </x:c>
       <x:c r="B30" s="123" t="d">
-        <x:v>2026-09-28T00:00:00.000Z</x:v>
+        <x:v>2026-09-26T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="C30" s="123" t="d">
         <x:v>2026-09-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="D30" s="104" t="str">
-        <x:v>POLYN</x:v>
+        <x:v>AMD／World Labs</x:v>
       </x:c>
       <x:c r="E30" s="80" t="str">
-        <x:v>TMS工程节点供客户评估</x:v>
+        <x:v>签署约82亿美元全股票收购协议</x:v>
       </x:c>
       <x:c r="F30" s="80" t="str">
-        <x:v>未具名评估方，非量产</x:v>
+        <x:v>AMD拟收购World Labs全部股权，预计2026年底完成；交易仍待监管批准和惯例条件，不是已完成收购，也不证明World Labs采用类脑芯片</x:v>
       </x:c>
       <x:c r="G30" s="80" t="str">
-        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+        <x:v>https://www.sec.gov/Archives/edgar/data/2488/000000248826000182/amd-20260926.htm</x:v>
       </x:c>
       <x:c r="H30" s="67"/>
       <x:c r="I30" s="68"/>
@@ -7359,14 +7470,28 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="28" customHeight="1">
-      <x:c r="A31" s="168"/>
-      <x:c r="B31" s="169"/>
-      <x:c r="C31" s="169"/>
-      <x:c r="D31" s="170"/>
-      <x:c r="E31" s="80"/>
-      <x:c r="F31" s="80"/>
-      <x:c r="G31" s="80"/>
+    <x:row r="31" ht="66" customHeight="1">
+      <x:c r="A31" s="132" t="str">
+        <x:v>T009</x:v>
+      </x:c>
+      <x:c r="B31" s="124" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C31" s="124" t="d">
+        <x:v>2026-09-28T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D31" s="133" t="str">
+        <x:v>POLYN</x:v>
+      </x:c>
+      <x:c r="E31" s="80" t="str">
+        <x:v>TMS工程节点供客户评估</x:v>
+      </x:c>
+      <x:c r="F31" s="80" t="str">
+        <x:v>未具名评估方，非量产</x:v>
+      </x:c>
+      <x:c r="G31" s="80" t="str">
+        <x:v>https://polyn.ai/polyn-delivers-first-vibrosense-tms-engineering-sensor-nodes-for-customer-evaluation/</x:v>
+      </x:c>
       <x:c r="H31" s="67"/>
       <x:c r="I31" s="68"/>
       <x:c r="J31" s="2"/>
@@ -7377,9 +7502,7 @@
       <x:c r="O31" s="2"/>
     </x:row>
     <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="102" t="str">
-        <x:v>半年收入</x:v>
-      </x:c>
+      <x:c r="A32" s="102"/>
       <x:c r="B32" s="103"/>
       <x:c r="C32" s="103"/>
       <x:c r="D32" s="104"/>
@@ -7396,18 +7519,12 @@
       <x:c r="O32" s="2"/>
     </x:row>
     <x:row r="33" ht="28" customHeight="1">
-      <x:c r="A33" s="178" t="str">
-        <x:v>构成</x:v>
-      </x:c>
-      <x:c r="B33" s="179" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C33" s="179" t="str">
-        <x:v>2026 H1</x:v>
-      </x:c>
-      <x:c r="D33" s="180" t="str">
-        <x:v>来源</x:v>
-      </x:c>
+      <x:c r="A33" s="193" t="str">
+        <x:v>半年收入</x:v>
+      </x:c>
+      <x:c r="B33" s="194"/>
+      <x:c r="C33" s="194"/>
+      <x:c r="D33" s="195"/>
       <x:c r="E33" s="80"/>
       <x:c r="F33" s="80"/>
       <x:c r="G33" s="80"/>
@@ -7420,18 +7537,18 @@
       <x:c r="N33" s="2"/>
       <x:c r="O33" s="2"/>
     </x:row>
-    <x:row r="34" ht="26" customHeight="1">
-      <x:c r="A34" s="78" t="str">
-        <x:v>许可</x:v>
-      </x:c>
-      <x:c r="B34" s="79" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="C34" s="79" t="n">
-        <x:v>613826</x:v>
-      </x:c>
-      <x:c r="D34" s="80" t="str">
-        <x:v>半年报Note 3</x:v>
+    <x:row r="34" ht="28" customHeight="1">
+      <x:c r="A34" s="199" t="str">
+        <x:v>构成</x:v>
+      </x:c>
+      <x:c r="B34" s="200" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C34" s="200" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D34" s="201" t="str">
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="E34" s="80"/>
       <x:c r="F34" s="80"/>
@@ -7447,13 +7564,13 @@
     </x:row>
     <x:row r="35" ht="26" customHeight="1">
       <x:c r="A35" s="76" t="str">
-        <x:v>产品</x:v>
+        <x:v>许可</x:v>
       </x:c>
       <x:c r="B35" s="86" t="n">
-        <x:v>19184</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="C35" s="86" t="n">
-        <x:v>110362</x:v>
+        <x:v>613826</x:v>
       </x:c>
       <x:c r="D35" s="77" t="str">
         <x:v>半年报Note 3</x:v>
@@ -7472,13 +7589,13 @@
     </x:row>
     <x:row r="36" ht="26" customHeight="1">
       <x:c r="A36" s="78" t="str">
-        <x:v>开发服务</x:v>
+        <x:v>产品</x:v>
       </x:c>
       <x:c r="B36" s="79" t="n">
-        <x:v>1004395</x:v>
+        <x:v>19184</x:v>
       </x:c>
       <x:c r="C36" s="79" t="n">
-        <x:v>498557</x:v>
+        <x:v>110362</x:v>
       </x:c>
       <x:c r="D36" s="83" t="str">
         <x:v>半年报Note 3</x:v>
@@ -7497,18 +7614,16 @@
     </x:row>
     <x:row r="37" ht="26" customHeight="1">
       <x:c r="A37" s="132" t="str">
-        <x:v>合计</x:v>
+        <x:v>开发服务</x:v>
       </x:c>
       <x:c r="B37" s="134" t="n">
-        <x:f>SUM(B34:B36)</x:f>
-        <x:v>1023579</x:v>
+        <x:v>1004395</x:v>
       </x:c>
       <x:c r="C37" s="134" t="n">
-        <x:f>SUM(C34:C36)</x:f>
-        <x:v>1222745</x:v>
+        <x:v>498557</x:v>
       </x:c>
       <x:c r="D37" s="124" t="str">
-        <x:v>监管半年报</x:v>
+        <x:v>半年报Note 3</x:v>
       </x:c>
       <x:c r="E37" s="118"/>
       <x:c r="F37" s="118"/>
@@ -7522,11 +7637,21 @@
       <x:c r="N37" s="2"/>
       <x:c r="O37" s="2"/>
     </x:row>
-    <x:row r="38" ht="30" customHeight="1">
-      <x:c r="A38" s="78"/>
-      <x:c r="B38" s="79"/>
-      <x:c r="C38" s="79"/>
-      <x:c r="D38" s="83"/>
+    <x:row r="38" ht="26" customHeight="1">
+      <x:c r="A38" s="78" t="str">
+        <x:v>合计</x:v>
+      </x:c>
+      <x:c r="B38" s="79" t="n">
+        <x:f>SUM(B35:B37)</x:f>
+        <x:v>1023579</x:v>
+      </x:c>
+      <x:c r="C38" s="79" t="n">
+        <x:f>SUM(C35:C37)</x:f>
+        <x:v>1222745</x:v>
+      </x:c>
+      <x:c r="D38" s="83" t="str">
+        <x:v>监管半年报</x:v>
+      </x:c>
       <x:c r="E38" s="80"/>
       <x:c r="F38" s="80"/>
       <x:c r="G38" s="80"/>
@@ -7540,18 +7665,10 @@
       <x:c r="O38" s="2"/>
     </x:row>
     <x:row r="39" ht="28" customHeight="1">
-      <x:c r="A39" s="178" t="str">
-        <x:v>现金与客户指标</x:v>
-      </x:c>
-      <x:c r="B39" s="179" t="str">
-        <x:v>2025 H1</x:v>
-      </x:c>
-      <x:c r="C39" s="179" t="str">
-        <x:v>2026 H1</x:v>
-      </x:c>
-      <x:c r="D39" s="182" t="str">
-        <x:v>边界</x:v>
-      </x:c>
+      <x:c r="A39" s="132"/>
+      <x:c r="B39" s="134"/>
+      <x:c r="C39" s="134"/>
+      <x:c r="D39" s="124"/>
       <x:c r="E39" s="80"/>
       <x:c r="F39" s="80"/>
       <x:c r="G39" s="80"/>
@@ -7564,18 +7681,18 @@
       <x:c r="N39" s="2"/>
       <x:c r="O39" s="2"/>
     </x:row>
-    <x:row r="40" ht="30" customHeight="1">
-      <x:c r="A40" s="78" t="str">
-        <x:v>客户收款</x:v>
-      </x:c>
-      <x:c r="B40" s="79" t="n">
-        <x:v>1522026</x:v>
-      </x:c>
-      <x:c r="C40" s="79" t="n">
-        <x:v>813247</x:v>
-      </x:c>
-      <x:c r="D40" s="80" t="str">
-        <x:v>现金流，不等于收入</x:v>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="199" t="str">
+        <x:v>现金与客户指标</x:v>
+      </x:c>
+      <x:c r="B40" s="200" t="str">
+        <x:v>2025 H1</x:v>
+      </x:c>
+      <x:c r="C40" s="200" t="str">
+        <x:v>2026 H1</x:v>
+      </x:c>
+      <x:c r="D40" s="201" t="str">
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="E40" s="80"/>
       <x:c r="F40" s="80"/>
@@ -7591,16 +7708,16 @@
     </x:row>
     <x:row r="41" ht="30" customHeight="1">
       <x:c r="A41" s="132" t="str">
-        <x:v>经营现金净流出</x:v>
+        <x:v>客户收款</x:v>
       </x:c>
       <x:c r="B41" s="134" t="n">
-        <x:v>6990176</x:v>
+        <x:v>1522026</x:v>
       </x:c>
       <x:c r="C41" s="134" t="n">
-        <x:v>11253495</x:v>
+        <x:v>813247</x:v>
       </x:c>
       <x:c r="D41" s="133" t="str">
-        <x:v>按流出绝对值展示</x:v>
+        <x:v>现金流，不等于收入</x:v>
       </x:c>
       <x:c r="E41" s="80"/>
       <x:c r="F41" s="80"/>
@@ -7616,16 +7733,16 @@
     </x:row>
     <x:row r="42" ht="30" customHeight="1">
       <x:c r="A42" s="105" t="str">
-        <x:v>期末现金及现金等价物</x:v>
+        <x:v>经营现金净流出</x:v>
       </x:c>
       <x:c r="B42" s="79" t="n">
-        <x:v>13458121</x:v>
+        <x:v>6990176</x:v>
       </x:c>
       <x:c r="C42" s="79" t="n">
-        <x:v>20304971</x:v>
+        <x:v>11253495</x:v>
       </x:c>
       <x:c r="D42" s="80" t="str">
-        <x:v>各年6月30日</x:v>
+        <x:v>按流出绝对值展示</x:v>
       </x:c>
       <x:c r="E42" s="80"/>
       <x:c r="F42" s="80"/>
@@ -7641,16 +7758,16 @@
     </x:row>
     <x:row r="43" ht="30" customHeight="1">
       <x:c r="A43" s="105" t="str">
-        <x:v>&gt;10%客户收入合计</x:v>
+        <x:v>期末现金及现金等价物</x:v>
       </x:c>
       <x:c r="B43" s="79" t="n">
-        <x:v>809706</x:v>
+        <x:v>13458121</x:v>
       </x:c>
       <x:c r="C43" s="79" t="n">
-        <x:v>983780</x:v>
+        <x:v>20304971</x:v>
       </x:c>
       <x:c r="D43" s="83" t="str">
-        <x:v>2026约占H1收入80.5%</x:v>
+        <x:v>各年6月30日</x:v>
       </x:c>
       <x:c r="E43" s="80"/>
       <x:c r="F43" s="80"/>
@@ -7666,14 +7783,16 @@
     </x:row>
     <x:row r="44" ht="30" customHeight="1">
       <x:c r="A44" s="105" t="str">
-        <x:v>首批AKD1500生产批次</x:v>
-      </x:c>
-      <x:c r="B44" s="79"/>
+        <x:v>&gt;10%客户收入合计</x:v>
+      </x:c>
+      <x:c r="B44" s="79" t="n">
+        <x:v>809706</x:v>
+      </x:c>
       <x:c r="C44" s="79" t="n">
-        <x:v>2000</x:v>
+        <x:v>983780</x:v>
       </x:c>
       <x:c r="D44" s="83" t="str">
-        <x:v>颗；公司收到，不是客户出货</x:v>
+        <x:v>2026约占H1收入80.5%</x:v>
       </x:c>
       <x:c r="E44" s="80"/>
       <x:c r="F44" s="80"/>
@@ -7687,11 +7806,17 @@
       <x:c r="N44" s="2"/>
       <x:c r="O44" s="2"/>
     </x:row>
-    <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="106"/>
-      <x:c r="B45" s="107"/>
-      <x:c r="C45" s="107"/>
-      <x:c r="D45" s="125"/>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="106" t="str">
+        <x:v>首批AKD1500生产批次</x:v>
+      </x:c>
+      <x:c r="B45" s="186"/>
+      <x:c r="C45" s="186" t="n">
+        <x:v>2000</x:v>
+      </x:c>
+      <x:c r="D45" s="125" t="str">
+        <x:v>颗；公司收到，不是客户出货</x:v>
+      </x:c>
       <x:c r="E45" s="107"/>
       <x:c r="F45" s="107"/>
       <x:c r="G45" s="107"/>
@@ -7705,12 +7830,8 @@
       <x:c r="O45" s="2"/>
     </x:row>
     <x:row r="46" ht="34" customHeight="1">
-      <x:c r="A46" s="4" t="str">
-        <x:v>来源</x:v>
-      </x:c>
-      <x:c r="B46" s="3" t="str">
-        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
-      </x:c>
+      <x:c r="A46" s="4"/>
+      <x:c r="B46" s="3"/>
       <x:c r="C46" s="3"/>
       <x:c r="D46" s="4"/>
       <x:c r="E46" s="3"/>
@@ -7727,10 +7848,10 @@
     </x:row>
     <x:row r="47" ht="34" customHeight="1">
       <x:c r="A47" s="4" t="str">
-        <x:v>边界</x:v>
+        <x:v>来源</x:v>
       </x:c>
       <x:c r="B47" s="3" t="str">
-        <x:v>BrainChip财务数据来自监管半年报；SpiNNcloud 336万欧元为公共采购合同授予值，不计入BrainChip收入图，也不等于SpiNNcloud已付款或确认收入。</x:v>
+        <x:v>https://investor.brainchip.com/wp-content/uploads/2026/09/2026-08-26-June-2026-half-yearly-report.pdf</x:v>
       </x:c>
       <x:c r="C47" s="3"/>
       <x:c r="D47" s="4"/>
@@ -7746,9 +7867,13 @@
       <x:c r="N47" s="2"/>
       <x:c r="O47" s="2"/>
     </x:row>
-    <x:row r="48" ht="82" customHeight="1">
-      <x:c r="A48" s="3"/>
-      <x:c r="B48" s="3"/>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="3" t="str">
+        <x:v>边界</x:v>
+      </x:c>
+      <x:c r="B48" s="3" t="str">
+        <x:v>BrainChip财务数据来自监管半年报；SpiNNcloud 336万欧元为公共采购合同授予值，不计入BrainChip收入图，也不等于SpiNNcloud已付款或确认收入。</x:v>
+      </x:c>
       <x:c r="C48" s="3"/>
       <x:c r="D48" s="4"/>
       <x:c r="E48" s="3"/>
@@ -7764,33 +7889,15 @@
       <x:c r="O48" s="2"/>
     </x:row>
     <x:row r="49" ht="82" customHeight="1">
-      <x:c r="A49" s="3" t="str">
-        <x:v>研究编号</x:v>
-      </x:c>
-      <x:c r="B49" s="3" t="str">
-        <x:v>研究主体</x:v>
-      </x:c>
-      <x:c r="C49" s="3" t="str">
-        <x:v>路线</x:v>
-      </x:c>
-      <x:c r="D49" s="4" t="str">
-        <x:v>发布日期</x:v>
-      </x:c>
-      <x:c r="E49" s="3" t="str">
-        <x:v>证据类型</x:v>
-      </x:c>
-      <x:c r="F49" s="3" t="str">
-        <x:v>作者报告指标</x:v>
-      </x:c>
-      <x:c r="G49" s="3" t="str">
-        <x:v>边界</x:v>
-      </x:c>
-      <x:c r="H49" s="3" t="str">
-        <x:v>原始URL</x:v>
-      </x:c>
-      <x:c r="I49" s="4" t="str">
-        <x:v>检索日期</x:v>
-      </x:c>
+      <x:c r="A49" s="3"/>
+      <x:c r="B49" s="3"/>
+      <x:c r="C49" s="3"/>
+      <x:c r="D49" s="4"/>
+      <x:c r="E49" s="3"/>
+      <x:c r="F49" s="3"/>
+      <x:c r="G49" s="3"/>
+      <x:c r="H49" s="3"/>
+      <x:c r="I49" s="4"/>
       <x:c r="J49" s="2"/>
       <x:c r="K49" s="2"/>
       <x:c r="L49" s="2"/>
@@ -7800,31 +7907,31 @@
     </x:row>
     <x:row r="50" ht="82" customHeight="1">
       <x:c r="A50" s="3" t="str">
-        <x:v>R001</x:v>
+        <x:v>研究编号</x:v>
       </x:c>
       <x:c r="B50" s="3" t="str">
-        <x:v>GelNeuro／中科院自动化所</x:v>
+        <x:v>研究主体</x:v>
       </x:c>
       <x:c r="C50" s="3" t="str">
-        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
-      </x:c>
-      <x:c r="D50" s="4" t="d">
-        <x:v>2026-07-06T00:00:00.000Z</x:v>
+        <x:v>路线</x:v>
+      </x:c>
+      <x:c r="D50" s="4" t="str">
+        <x:v>发布日期</x:v>
       </x:c>
       <x:c r="E50" s="3" t="str">
-        <x:v>作者预印本实机研究结果，未独立复现</x:v>
+        <x:v>证据类型</x:v>
       </x:c>
       <x:c r="F50" s="3" t="str">
-        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
+        <x:v>作者报告指标</x:v>
       </x:c>
       <x:c r="G50" s="3" t="str">
-        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
+        <x:v>边界</x:v>
       </x:c>
       <x:c r="H50" s="3" t="str">
-        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
-      </x:c>
-      <x:c r="I50" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>原始URL</x:v>
+      </x:c>
+      <x:c r="I50" s="4" t="str">
+        <x:v>检索日期</x:v>
       </x:c>
       <x:c r="J50" s="2"/>
       <x:c r="K50" s="2"/>
@@ -7835,28 +7942,28 @@
     </x:row>
     <x:row r="51" ht="82" customHeight="1">
       <x:c r="A51" s="3" t="str">
-        <x:v>R002</x:v>
+        <x:v>R001</x:v>
       </x:c>
       <x:c r="B51" s="3" t="str">
-        <x:v>SpikingTac／中科院自动化所</x:v>
+        <x:v>GelNeuro／中科院自动化所</x:v>
       </x:c>
       <x:c r="C51" s="3" t="str">
-        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
+        <x:v>GelSight Mini前端＋Speck2f DVS／SCNN直接推理</x:v>
       </x:c>
       <x:c r="D51" s="4" t="d">
-        <x:v>2026-02-27T00:00:00.000Z</x:v>
+        <x:v>2026-07-06T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E51" s="3" t="str">
-        <x:v>作者预印本研究样机，未独立复现</x:v>
+        <x:v>作者预印本实机研究结果，未独立复现</x:v>
       </x:c>
       <x:c r="F51" s="3" t="str">
-        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
+        <x:v>15类纹理；96.3%；80ms窗口；板级活动19.6mW</x:v>
       </x:c>
       <x:c r="G51" s="3" t="str">
-        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
+        <x:v>离线PC训练；不是完整机器人功耗、在线学习、真实客户或世界模型训练</x:v>
       </x:c>
       <x:c r="H51" s="3" t="str">
-        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
+        <x:v>https://arxiv.org/html/2607.05241v1</x:v>
       </x:c>
       <x:c r="I51" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7870,28 +7977,28 @@
     </x:row>
     <x:row r="52" ht="82" customHeight="1">
       <x:c r="A52" s="4" t="str">
-        <x:v>R003</x:v>
+        <x:v>R002</x:v>
       </x:c>
       <x:c r="B52" s="3" t="str">
-        <x:v>OmniVTA／NUS、CASIA等</x:v>
+        <x:v>SpikingTac／中科院自动化所</x:v>
       </x:c>
       <x:c r="C52" s="3" t="str">
-        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
+        <x:v>独立事件相机＋动态状态图与迟滞补偿</x:v>
       </x:c>
       <x:c r="D52" s="4" t="d">
-        <x:v>2026-03-19T00:00:00.000Z</x:v>
+        <x:v>2026-02-27T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E52" s="3" t="str">
-        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
+        <x:v>作者预印本研究样机，未独立复现</x:v>
       </x:c>
       <x:c r="F52" s="3" t="str">
-        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
+        <x:v>感知1000Hz、跟踪350Hz；实验碰撞后过冲6.2mm</x:v>
       </x:c>
       <x:c r="G52" s="3" t="str">
-        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
+        <x:v>动态事件状态处理不自动等于SNN芯片；无商业出货／收入证据</x:v>
       </x:c>
       <x:c r="H52" s="3" t="str">
-        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
+        <x:v>https://arxiv.org/html/2602.23654v1</x:v>
       </x:c>
       <x:c r="I52" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7905,28 +8012,28 @@
     </x:row>
     <x:row r="53" ht="82" customHeight="1">
       <x:c r="A53" s="4" t="str">
-        <x:v>R004</x:v>
+        <x:v>R003</x:v>
       </x:c>
       <x:c r="B53" s="3" t="str">
-        <x:v>Event-VLA／上海科技大学等</x:v>
+        <x:v>OmniVTA／NUS、CASIA等</x:v>
       </x:c>
       <x:c r="C53" s="3" t="str">
-        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
+        <x:v>视触觉世界模型＋60Hz触觉反射闭环</x:v>
       </x:c>
       <x:c r="D53" s="4" t="d">
-        <x:v>2026-06-28T00:00:00.000Z</x:v>
+        <x:v>2026-03-19T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E53" s="3" t="str">
-        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
+        <x:v>作者预印本、项目页与真机实验；未独立复现</x:v>
       </x:c>
       <x:c r="F53" s="3" t="str">
-        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
+        <x:v>21,879轨迹、86任务、100+物体；六类接触任务真机评估</x:v>
       </x:c>
       <x:c r="G53" s="3" t="str">
-        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
+        <x:v>采用Xense、GelSight Mini、Tac3D、Daimon等常规触觉，不是事件触觉或SNN芯片；代码／数据仅称将公开</x:v>
       </x:c>
       <x:c r="H53" s="3" t="str">
-        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
+        <x:v>https://arxiv.org/html/2603.19201v3</x:v>
       </x:c>
       <x:c r="I53" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7940,28 +8047,28 @@
     </x:row>
     <x:row r="54" ht="82" customHeight="1">
       <x:c r="A54" s="4" t="str">
-        <x:v>R005</x:v>
+        <x:v>R004</x:v>
       </x:c>
       <x:c r="B54" s="3" t="str">
-        <x:v>TouchWorld／研究团队</x:v>
+        <x:v>Event-VLA／上海科技大学等</x:v>
       </x:c>
       <x:c r="C54" s="3" t="str">
-        <x:v>预测式＋反应式触觉基础模型</x:v>
+        <x:v>DAVIS事件相机＋VLA动作条件事件融合</x:v>
       </x:c>
       <x:c r="D54" s="4" t="d">
-        <x:v>2026-07-08T00:00:00.000Z</x:v>
+        <x:v>2026-06-28T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E54" s="3" t="str">
-        <x:v>作者预印本研究；未独立复现</x:v>
+        <x:v>作者预印本真机研究；Franka Research 3与真实事件相机，未独立复现</x:v>
       </x:c>
       <x:c r="F54" s="3" t="str">
-        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
+        <x:v>80次示范、4任务；作者报近暗环境平均成功率52.5%，正常光72.5%</x:v>
       </x:c>
       <x:c r="G54" s="3" t="str">
-        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
+        <x:v>事件视觉而非触觉；VLA动作模型而非明确世界模型；小样本研究，RTX 4090服务器，无专用类脑芯片</x:v>
       </x:c>
       <x:c r="H54" s="3" t="str">
-        <x:v>https://arxiv.org/abs/2607.07287</x:v>
+        <x:v>https://arxiv.org/html/2606.29384v1</x:v>
       </x:c>
       <x:c r="I54" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -7975,28 +8082,28 @@
     </x:row>
     <x:row r="55" ht="82" customHeight="1">
       <x:c r="A55" s="4" t="str">
-        <x:v>R006</x:v>
+        <x:v>R005</x:v>
       </x:c>
       <x:c r="B55" s="3" t="str">
-        <x:v>CLP-SNN／LMU、Intel等</x:v>
+        <x:v>TouchWorld／研究团队</x:v>
       </x:c>
       <x:c r="C55" s="3" t="str">
-        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+        <x:v>预测式＋反应式触觉基础模型</x:v>
       </x:c>
       <x:c r="D55" s="4" t="d">
-        <x:v>2026-05-05T00:00:00.000Z</x:v>
+        <x:v>2026-07-08T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="E55" s="3" t="str">
-        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+        <x:v>作者预印本研究；未独立复现</x:v>
       </x:c>
       <x:c r="F55" s="3" t="str">
-        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+        <x:v>6项灵巧操作任务；作者报65.0%干净条件、53.7%扰动条件</x:v>
       </x:c>
       <x:c r="G55" s="3" t="str">
-        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+        <x:v>使用压力手套／常规触觉适配，不是事件触觉或SNN芯片；商业客户、代码和部署未知</x:v>
       </x:c>
       <x:c r="H55" s="3" t="str">
-        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+        <x:v>https://arxiv.org/abs/2607.07287</x:v>
       </x:c>
       <x:c r="I55" s="4" t="d">
         <x:v>2026-10-02T00:00:00.000Z</x:v>
@@ -8008,16 +8115,34 @@
       <x:c r="N55" s="2"/>
       <x:c r="O55" s="2"/>
     </x:row>
-    <x:row r="56" ht="50" customHeight="1">
-      <x:c r="A56" s="11"/>
-      <x:c r="B56" s="2"/>
-      <x:c r="C56" s="2"/>
-      <x:c r="D56" s="2"/>
-      <x:c r="E56" s="2"/>
-      <x:c r="F56" s="2"/>
-      <x:c r="G56" s="2"/>
-      <x:c r="H56" s="2"/>
-      <x:c r="I56" s="2"/>
+    <x:row r="56" ht="82" customHeight="1">
+      <x:c r="A56" s="4" t="str">
+        <x:v>R006</x:v>
+      </x:c>
+      <x:c r="B56" s="3" t="str">
+        <x:v>CLP-SNN／LMU、Intel等</x:v>
+      </x:c>
+      <x:c r="C56" s="3" t="str">
+        <x:v>Loihi2原型分配与片上写入；完整自适应规则仅仿真</x:v>
+      </x:c>
+      <x:c r="D56" s="4" t="d">
+        <x:v>2026-05-05T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="E56" s="3" t="str">
+        <x:v>作者论文v2 Methods及代码；实机科研，未独立复现</x:v>
+      </x:c>
+      <x:c r="F56" s="3" t="str">
+        <x:v>作者报学习模块0.33ms／0.05mJ；硬件为原型写入一次后冻结，错误时新增原型</x:v>
+      </x:c>
+      <x:c r="G56" s="3" t="str">
+        <x:v>主机GPU冻结EfficientNet-B0提取1280维特征；不含特征提取与IO。完整自适应／元可塑性未完整上芯；实机代码需联系作者，依赖专有Lava-Loihi。初稿2025-11-03；v2提交2026-05-05，HTML题头另标8月24日，不替代版本日期。非客户出货／收入。</x:v>
+      </x:c>
+      <x:c r="H56" s="3" t="str">
+        <x:v>https://arxiv.org/html/2511.01553v2</x:v>
+      </x:c>
+      <x:c r="I56" s="4" t="d">
+        <x:v>2026-10-02T00:00:00.000Z</x:v>
+      </x:c>
       <x:c r="J56" s="2"/>
       <x:c r="K56" s="2"/>
       <x:c r="L56" s="2"/>
@@ -8096,8 +8221,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56888d6d35b443b3"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra53cf51e3d8840a5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4921207f21dc4a2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfc7aa281e3a4397"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Mythic India engineering expansion evidence
Add the September 29 Bengaluru CoE event, current RTL/DV/PD/DFT evidence, cross-region mapping, and synchronized downloadable evidence. Preserve the no-tapeout/no-sample boundary for Vanguard.
</commit_message>
<xml_diff>
--- a/market-evidence.xlsx
+++ b/market-evidence.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="Ra8714f0ffee949fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="R95736d4aaddf4fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="Rf867912933864b09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="Rbfc9847b51f04f85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="图表汇总" sheetId="1" r:id="Rf2226dd950404beb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="主体证据" sheetId="2" r:id="R502b7028995b496d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="产品阶段" sheetId="3" r:id="R80136088471748f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="事件与财务" sheetId="4" r:id="Rbda4958cd7fe4bf8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1334,7 +1334,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R70da2afa31b54948"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rfb9ddd9452134289"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1364,7 +1364,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1b4b96a18045418b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9a55a93431824990"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1394,7 +1394,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd82942c26f9416c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rba98c557ff7c4b3f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1404,7 +1404,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CompanyEvidence" displayName="CompanyEvidence" ref="A1:I39" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="编号"/>
     <x:tableColumn id="2" name="主体"/>
@@ -1439,21 +1439,6 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="EventEvidence" displayName="EventEvidence" ref="A1:G31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="7">
-    <x:tableColumn id="1" name="编号"/>
-    <x:tableColumn id="2" name="事件日期"/>
-    <x:tableColumn id="3" name="发布日期"/>
-    <x:tableColumn id="4" name="主体"/>
-    <x:tableColumn id="5" name="事件"/>
-    <x:tableColumn id="6" name="证据边界"/>
-    <x:tableColumn id="7" name="原始URL"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TactileResearch" displayName="TactileResearch" ref="A50:I56" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="研究编号"/>
@@ -1465,6 +1450,21 @@
     <x:tableColumn id="7" name="边界"/>
     <x:tableColumn id="8" name="原始URL"/>
     <x:tableColumn id="9" name="检索日期"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="EventEvidence" displayName="EventEvidence" ref="A1:G32" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="7">
+    <x:tableColumn id="1" name="编号"/>
+    <x:tableColumn id="2" name="事件日期"/>
+    <x:tableColumn id="3" name="发布日期"/>
+    <x:tableColumn id="4" name="主体"/>
+    <x:tableColumn id="5" name="事件"/>
+    <x:tableColumn id="6" name="证据边界"/>
+    <x:tableColumn id="7" name="原始URL"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -1717,7 +1717,7 @@
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="2" t="str">
-        <x:v>2026-10-03核心SNN、多卡调度与常开感知复核。38个主体、42组产品、30项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
+        <x:v>2026-10-03模拟AI、存算与数据流复核。38个主体、42组产品、31项事件、6项科研记录。样本覆盖，不代表市场份额。</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -2967,7 +2967,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda340d1e09ab4669"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cdb8fe5c6334b80"/>
 </x:worksheet>
 </file>
 
@@ -3021,7 +3021,7 @@
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
     </x:row>
-    <x:row r="2" ht="74" customHeight="1">
+    <x:row r="2" ht="70" customHeight="1">
       <x:c r="A2" s="3" t="str">
         <x:v>C001</x:v>
       </x:c>
@@ -3056,7 +3056,7 @@
       <x:c r="N2" s="2"/>
       <x:c r="O2" s="2"/>
     </x:row>
-    <x:row r="3" ht="74" customHeight="1">
+    <x:row r="3" ht="70" customHeight="1">
       <x:c r="A3" s="3" t="str">
         <x:v>C002</x:v>
       </x:c>
@@ -3091,7 +3091,7 @@
       <x:c r="N3" s="2"/>
       <x:c r="O3" s="2"/>
     </x:row>
-    <x:row r="4" ht="74" customHeight="1">
+    <x:row r="4" ht="70" customHeight="1">
       <x:c r="A4" s="3" t="str">
         <x:v>C003</x:v>
       </x:c>
@@ -3105,19 +3105,19 @@
         <x:v>Speck感算一体SNN、Aeveon高速视觉路线、iniVation事件相机及Rigi神经信号采集</x:v>
       </x:c>
       <x:c r="E4" s="3" t="str">
-        <x:v>2024年2月1日SynSense宣布母公司收购iniVation 100%股份；苏黎世实体继续运营并服务原客户。2026年参投方另确认数亿元B轮及视觉产品批量订单口径。</x:v>
+        <x:v>2024年2月1日SynSense宣布母公司收购iniVation 100%股份；苏黎世实体继续运营并服务原客户。Aeveon于2026年6月24日发布；当前产品页披露最高1000 fps、VGA、约1 ms、多模态输出、3.4×3.4 mm与1-lane MIPI CSI-2等厂商规格。2026年参投方另确认数亿元B轮及视觉产品批量订单口径。</x:v>
       </x:c>
       <x:c r="F4" s="3" t="str">
-        <x:v>iniVation已不是独立所有权主体，但仍保留运营实体和产品品牌；交易金额未披露。2026批量订单未披露型号、客户、数量、金额、交付或收入，不能直接映射为Aeveon、Speck或iniVation相机。</x:v>
+        <x:v>iniVation已不是独立所有权主体，但仍保留运营实体和产品品牌；交易金额未披露。Aeveon的Product Resources仍标为Coming soon，未见公开数据表、开发板、价格、库存、生产状态或具名客户。2026批量订单未披露型号、客户、数量、金额、交付或收入，不能直接映射为Aeveon、Speck或iniVation相机。</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>SynSense 2024-02-01收购公告及参投方2026-07-14文章；所有权、运营延续和订单宣称分列</x:v>
+        <x:v>SynSense收购公告、Aeveon发布与产品页、参投方融资文章；所有权、产品规格、运营延续与订单宣称分列</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>https://www.synsense.ai/synsense-and-inivation-join-forces-to-form-leading-neuromorphic-technology-provider/</x:v>
+        <x:v>https://www.synsense.ai/products/aeveon_eye/</x:v>
       </x:c>
       <x:c r="I4" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J4" s="2"/>
       <x:c r="K4" s="2"/>
@@ -3126,7 +3126,7 @@
       <x:c r="N4" s="2"/>
       <x:c r="O4" s="2"/>
     </x:row>
-    <x:row r="5" ht="74" customHeight="1">
+    <x:row r="5" ht="70" customHeight="1">
       <x:c r="A5" s="3" t="str">
         <x:v>C004</x:v>
       </x:c>
@@ -3161,7 +3161,7 @@
       <x:c r="N5" s="2"/>
       <x:c r="O5" s="2"/>
     </x:row>
-    <x:row r="6" ht="74" customHeight="1">
+    <x:row r="6" ht="70" customHeight="1">
       <x:c r="A6" s="3" t="str">
         <x:v>C005</x:v>
       </x:c>
@@ -3196,7 +3196,7 @@
       <x:c r="N6" s="2"/>
       <x:c r="O6" s="2"/>
     </x:row>
-    <x:row r="7" ht="74" customHeight="1">
+    <x:row r="7" ht="70" customHeight="1">
       <x:c r="A7" s="3" t="str">
         <x:v>C006</x:v>
       </x:c>
@@ -3231,7 +3231,7 @@
       <x:c r="N7" s="2"/>
       <x:c r="O7" s="2"/>
     </x:row>
-    <x:row r="8" ht="74" customHeight="1">
+    <x:row r="8" ht="70" customHeight="1">
       <x:c r="A8" s="3" t="str">
         <x:v>C007</x:v>
       </x:c>
@@ -3266,7 +3266,7 @@
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="2"/>
     </x:row>
-    <x:row r="9" ht="74" customHeight="1">
+    <x:row r="9" ht="70" customHeight="1">
       <x:c r="A9" s="3" t="str">
         <x:v>C008</x:v>
       </x:c>
@@ -3301,7 +3301,7 @@
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="2"/>
     </x:row>
-    <x:row r="10" ht="74" customHeight="1">
+    <x:row r="10" ht="70" customHeight="1">
       <x:c r="A10" s="3" t="str">
         <x:v>C009</x:v>
       </x:c>
@@ -3336,7 +3336,7 @@
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
     </x:row>
-    <x:row r="11" ht="74" customHeight="1">
+    <x:row r="11" ht="70" customHeight="1">
       <x:c r="A11" s="3" t="str">
         <x:v>C010</x:v>
       </x:c>
@@ -3371,7 +3371,7 @@
       <x:c r="N11" s="2"/>
       <x:c r="O11" s="2"/>
     </x:row>
-    <x:row r="12" ht="74" customHeight="1">
+    <x:row r="12" ht="70" customHeight="1">
       <x:c r="A12" s="3" t="str">
         <x:v>C011</x:v>
       </x:c>
@@ -3406,7 +3406,7 @@
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="2"/>
     </x:row>
-    <x:row r="13" ht="74" customHeight="1">
+    <x:row r="13" ht="70" customHeight="1">
       <x:c r="A13" s="3" t="str">
         <x:v>C012</x:v>
       </x:c>
@@ -3441,7 +3441,7 @@
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="2"/>
     </x:row>
-    <x:row r="14" ht="74" customHeight="1">
+    <x:row r="14" ht="70" customHeight="1">
       <x:c r="A14" s="3" t="str">
         <x:v>C013</x:v>
       </x:c>
@@ -3476,7 +3476,7 @@
       <x:c r="N14" s="2"/>
       <x:c r="O14" s="2"/>
     </x:row>
-    <x:row r="15" ht="74" customHeight="1">
+    <x:row r="15" ht="70" customHeight="1">
       <x:c r="A15" s="3" t="str">
         <x:v>C014</x:v>
       </x:c>
@@ -3511,7 +3511,7 @@
       <x:c r="N15" s="2"/>
       <x:c r="O15" s="2"/>
     </x:row>
-    <x:row r="16" ht="74" customHeight="1">
+    <x:row r="16" ht="70" customHeight="1">
       <x:c r="A16" s="3" t="str">
         <x:v>C015</x:v>
       </x:c>
@@ -3546,7 +3546,7 @@
       <x:c r="N16" s="2"/>
       <x:c r="O16" s="2"/>
     </x:row>
-    <x:row r="17" ht="74" customHeight="1">
+    <x:row r="17" ht="70" customHeight="1">
       <x:c r="A17" s="3" t="str">
         <x:v>C016</x:v>
       </x:c>
@@ -3581,7 +3581,7 @@
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
     </x:row>
-    <x:row r="18" ht="74" customHeight="1">
+    <x:row r="18" ht="70" customHeight="1">
       <x:c r="A18" s="3" t="str">
         <x:v>C017</x:v>
       </x:c>
@@ -3616,7 +3616,7 @@
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="2"/>
     </x:row>
-    <x:row r="19" ht="74" customHeight="1">
+    <x:row r="19" ht="70" customHeight="1">
       <x:c r="A19" s="3" t="str">
         <x:v>C018</x:v>
       </x:c>
@@ -3651,7 +3651,7 @@
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="2"/>
     </x:row>
-    <x:row r="20" ht="74" customHeight="1">
+    <x:row r="20" ht="70" customHeight="1">
       <x:c r="A20" s="3" t="str">
         <x:v>C019</x:v>
       </x:c>
@@ -3686,7 +3686,7 @@
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="2"/>
     </x:row>
-    <x:row r="21" ht="74" customHeight="1">
+    <x:row r="21" ht="70" customHeight="1">
       <x:c r="A21" s="3" t="str">
         <x:v>C020</x:v>
       </x:c>
@@ -3721,7 +3721,7 @@
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="2"/>
     </x:row>
-    <x:row r="22" ht="74" customHeight="1">
+    <x:row r="22" ht="70" customHeight="1">
       <x:c r="A22" s="3" t="str">
         <x:v>C021</x:v>
       </x:c>
@@ -3756,7 +3756,7 @@
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="2"/>
     </x:row>
-    <x:row r="23" ht="74" customHeight="1">
+    <x:row r="23" ht="70" customHeight="1">
       <x:c r="A23" s="3" t="str">
         <x:v>C022</x:v>
       </x:c>
@@ -3791,7 +3791,7 @@
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="2"/>
     </x:row>
-    <x:row r="24" ht="74" customHeight="1">
+    <x:row r="24" ht="70" customHeight="1">
       <x:c r="A24" s="3" t="str">
         <x:v>C023</x:v>
       </x:c>
@@ -3826,7 +3826,7 @@
       <x:c r="N24" s="2"/>
       <x:c r="O24" s="2"/>
     </x:row>
-    <x:row r="25" ht="74" customHeight="1">
+    <x:row r="25" ht="70" customHeight="1">
       <x:c r="A25" s="3" t="str">
         <x:v>C024</x:v>
       </x:c>
@@ -3861,7 +3861,7 @@
       <x:c r="N25" s="2"/>
       <x:c r="O25" s="2"/>
     </x:row>
-    <x:row r="26" ht="74" customHeight="1">
+    <x:row r="26" ht="70" customHeight="1">
       <x:c r="A26" s="3" t="str">
         <x:v>C025</x:v>
       </x:c>
@@ -3896,7 +3896,7 @@
       <x:c r="N26" s="2"/>
       <x:c r="O26" s="2"/>
     </x:row>
-    <x:row r="27" ht="74" customHeight="1">
+    <x:row r="27" ht="70" customHeight="1">
       <x:c r="A27" s="3" t="str">
         <x:v>C026</x:v>
       </x:c>
@@ -3931,7 +3931,7 @@
       <x:c r="N27" s="2"/>
       <x:c r="O27" s="2"/>
     </x:row>
-    <x:row r="28" ht="74" customHeight="1">
+    <x:row r="28" ht="70" customHeight="1">
       <x:c r="A28" s="3" t="str">
         <x:v>C027</x:v>
       </x:c>
@@ -3945,19 +3945,19 @@
         <x:v>M1模拟CIM APU；Vanguard混合模拟／数字APU；Starlight传感集成；Mead 3D NAND大模型路线；Videantis数字IP</x:v>
       </x:c>
       <x:c r="E28" s="3" t="str">
-        <x:v>M1可申请评估；Vanguard计划2027可用并披露GF 28nm模拟die＋TSMC N5A数字die；Microchip／SST确认下一代APU选用memBrain／SuperFlash；Starlight与Mead均标注在研</x:v>
+        <x:v>M1可申请评估；Vanguard计划2027可用并披露GF 28nm模拟die＋TSMC N5A数字die；Microchip／SST确认下一代APU选用memBrain／SuperFlash。2026年9月29日Mythic宣布班加罗尔CoE，称团队已参与模拟核心前端、混合物理设计和车规DFT；当前招聘页可见RTL、验证、物理设计与DFT岗位</x:v>
       </x:c>
       <x:c r="F28" s="3" t="str">
-        <x:v>Vanguard未见投片、样片、客户或交付；Starlight现有演示运行于M1硅片，未证实集成传感器；Mead未见3D NAND硅片。所有高能效数字均为厂商口径</x:v>
+        <x:v>Vanguard未见投片、样片、客户或交付；Mythic所称Lockheed Martin战术边缘验证未见Lockheed对应硬件、任务或结果披露；Starlight现有演示运行于M1硅片，未证实集成传感器；Mead未见3D NAND硅片。所有高能效数字均为厂商口径</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Mythic产品页与Microchip／SST 2026-03-17公告，检索2026-10-02；供应链选型不等于流片</x:v>
+        <x:v>Mythic 2026-09-29班加罗尔CoE公告、当前官方岗位页、产品页及Microchip／SST公告；组织扩张与厂商验证口径不等于投片、样片或交付</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>https://www.mythic.ai/vanguard</x:v>
+        <x:v>https://www.mythic.ai/newsroom/mythic-bengaluru-centre-of-excellence</x:v>
       </x:c>
       <x:c r="I28" s="4" t="d">
-        <x:v>2026-10-02T00:00:00.000Z</x:v>
+        <x:v>2026-10-03T00:00:00.000Z</x:v>
       </x:c>
       <x:c r="J28" s="2"/>
       <x:c r="K28" s="2"/>
@@ -3966,7 +3966,7 @@
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="2"/>
     </x:row>
-    <x:row r="29" ht="74" customHeight="1">
+    <x:row r="29" ht="70" customHeight="1">
       <x:c r="A29" s="3" t="str">
         <x:v>C028</x:v>
       </x:c>
@@ -4001,7 +4001,7 @@
       <x:c r="N29" s="2"/>
       <x:c r="O29" s="2"/>
     </x:row>
-    <x:row r="30" ht="74" customHeight="1">
+    <x:row r="30" ht="70" customHeight="1">
       <x:c r="A30" s="3" t="str">
         <x:v>C029</x:v>
       </x:c>
@@ -4036,7 +4036,7 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="74" customHeight="1">
+    <x:row r="31" ht="70" customHeight="1">
       <x:c r="A31" s="3" t="str">
         <x:v>C030</x:v>
       </x:c>
@@ -4071,7 +4071,7 @@
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="2"/>
     </x:row>
-    <x:row r="32" ht="74" customHeight="1">
+    <x:row r="32" ht="70" customHeight="1">
       <x:c r="A32" s="3" t="str">
         <x:v>C031</x:v>
       </x:c>
@@ -4106,7 +4106,7 @@
       <x:c r="N32" s="2"/>
       <x:c r="O32" s="2"/>
     </x:row>
-    <x:row r="33" ht="74" customHeight="1">
+    <x:row r="33" ht="70" customHeight="1">
       <x:c r="A33" s="3" t="str">
         <x:v>C032</x:v>
       </x:c>
@@ -4141,7 +4141,7 @@
       <x:c r="N33" s="2"/>
       <x:c r="O33" s="2"/>
     </x:row>
-    <x:row r="34" ht="74" customHeight="1">
+    <x:row r="34" ht="70" customHeight="1">
       <x:c r="A34" s="3" t="str">
         <x:v>C033</x:v>
       </x:c>
@@ -4176,7 +4176,7 @@
       <x:c r="N34" s="2"/>
       <x:c r="O34" s="2"/>
     </x:row>
-    <x:row r="35" ht="74" customHeight="1">
+    <x:row r="35" ht="70" customHeight="1">
       <x:c r="A35" s="3" t="str">
         <x:v>C034</x:v>
       </x:c>
@@ -4211,7 +4211,7 @@
       <x:c r="N35" s="2"/>
       <x:c r="O35" s="2"/>
     </x:row>
-    <x:row r="36" ht="74" customHeight="1">
+    <x:row r="36" ht="70" customHeight="1">
       <x:c r="A36" s="3" t="str">
         <x:v>C035</x:v>
       </x:c>
@@ -4246,7 +4246,7 @@
       <x:c r="N36" s="2"/>
       <x:c r="O36" s="2"/>
     </x:row>
-    <x:row r="37" ht="74" customHeight="1">
+    <x:row r="37" ht="70" customHeight="1">
       <x:c r="A37" s="3" t="str">
         <x:v>C036</x:v>
       </x:c>
@@ -4281,7 +4281,7 @@
       <x:c r="N37" s="2"/>
       <x:c r="O37" s="2"/>
     </x:row>
-    <x:row r="38" ht="74" customHeight="1">
+    <x:row r="38" ht="70" customHeight="1">
       <x:c r="A38" s="3" t="str">
         <x:v>C037</x:v>
       </x:c>
@@ -4316,7 +4316,7 @@
       <x:c r="N38" s="2"/>
       <x:c r="O38" s="2"/>
     </x:row>
-    <x:row r="39" ht="74" customHeight="1">
+    <x:row r="39" ht="70" customHeight="1">
       <x:c r="A39" s="3" t="str">
         <x:v>C038</x:v>
       </x:c>
@@ -4722,7 +4722,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf45ebfc9427f4f76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf4c8e0062e348ef"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6528,7 +6528,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f61a696b93e45f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9c508ba257e4d7f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6579,7 +6579,7 @@
       <x:c r="N1" s="2"/>
       <x:c r="O1" s="2"/>
     </x:row>
-    <x:row r="2" ht="66" customHeight="1">
+    <x:row r="2" ht="60" customHeight="1">
       <x:c r="A2" s="151" t="str">
         <x:v>T028</x:v>
       </x:c>
@@ -6610,7 +6610,7 @@
       <x:c r="N2" s="2"/>
       <x:c r="O2" s="2"/>
     </x:row>
-    <x:row r="3" ht="66" customHeight="1">
+    <x:row r="3" ht="60" customHeight="1">
       <x:c r="A3" s="151" t="str">
         <x:v>T018</x:v>
       </x:c>
@@ -6641,7 +6641,7 @@
       <x:c r="N3" s="2"/>
       <x:c r="O3" s="2"/>
     </x:row>
-    <x:row r="4" ht="66" customHeight="1">
+    <x:row r="4" ht="60" customHeight="1">
       <x:c r="A4" s="151" t="str">
         <x:v>T012</x:v>
       </x:c>
@@ -6672,7 +6672,7 @@
       <x:c r="N4" s="2"/>
       <x:c r="O4" s="2"/>
     </x:row>
-    <x:row r="5" ht="66" customHeight="1">
+    <x:row r="5" ht="60" customHeight="1">
       <x:c r="A5" s="151" t="str">
         <x:v>T029</x:v>
       </x:c>
@@ -6703,7 +6703,7 @@
       <x:c r="N5" s="2"/>
       <x:c r="O5" s="2"/>
     </x:row>
-    <x:row r="6" ht="66" customHeight="1">
+    <x:row r="6" ht="60" customHeight="1">
       <x:c r="A6" s="151" t="str">
         <x:v>T019</x:v>
       </x:c>
@@ -6734,7 +6734,7 @@
       <x:c r="N6" s="2"/>
       <x:c r="O6" s="2"/>
     </x:row>
-    <x:row r="7" ht="66" customHeight="1">
+    <x:row r="7" ht="60" customHeight="1">
       <x:c r="A7" s="151" t="str">
         <x:v>T001</x:v>
       </x:c>
@@ -6765,7 +6765,7 @@
       <x:c r="N7" s="2"/>
       <x:c r="O7" s="2"/>
     </x:row>
-    <x:row r="8" ht="66" customHeight="1">
+    <x:row r="8" ht="60" customHeight="1">
       <x:c r="A8" s="151" t="str">
         <x:v>T026</x:v>
       </x:c>
@@ -6796,7 +6796,7 @@
       <x:c r="N8" s="2"/>
       <x:c r="O8" s="2"/>
     </x:row>
-    <x:row r="9" ht="66" customHeight="1">
+    <x:row r="9" ht="60" customHeight="1">
       <x:c r="A9" s="151" t="str">
         <x:v>T022</x:v>
       </x:c>
@@ -6827,7 +6827,7 @@
       <x:c r="N9" s="2"/>
       <x:c r="O9" s="2"/>
     </x:row>
-    <x:row r="10" ht="66" customHeight="1">
+    <x:row r="10" ht="60" customHeight="1">
       <x:c r="A10" s="151" t="str">
         <x:v>T002</x:v>
       </x:c>
@@ -6858,7 +6858,7 @@
       <x:c r="N10" s="2"/>
       <x:c r="O10" s="2"/>
     </x:row>
-    <x:row r="11" ht="66" customHeight="1">
+    <x:row r="11" ht="60" customHeight="1">
       <x:c r="A11" s="151" t="str">
         <x:v>T021</x:v>
       </x:c>
@@ -6889,7 +6889,7 @@
       <x:c r="N11" s="2"/>
       <x:c r="O11" s="2"/>
     </x:row>
-    <x:row r="12" ht="66" customHeight="1">
+    <x:row r="12" ht="60" customHeight="1">
       <x:c r="A12" s="151" t="str">
         <x:v>T025</x:v>
       </x:c>
@@ -6918,7 +6918,7 @@
       <x:c r="N12" s="2"/>
       <x:c r="O12" s="2"/>
     </x:row>
-    <x:row r="13" ht="66" customHeight="1">
+    <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" s="151" t="str">
         <x:v>T003</x:v>
       </x:c>
@@ -6949,7 +6949,7 @@
       <x:c r="N13" s="2"/>
       <x:c r="O13" s="2"/>
     </x:row>
-    <x:row r="14" ht="66" customHeight="1">
+    <x:row r="14" ht="60" customHeight="1">
       <x:c r="A14" s="151" t="str">
         <x:v>T013</x:v>
       </x:c>
@@ -6980,7 +6980,7 @@
       <x:c r="N14" s="2"/>
       <x:c r="O14" s="2"/>
     </x:row>
-    <x:row r="15" ht="66" customHeight="1">
+    <x:row r="15" ht="60" customHeight="1">
       <x:c r="A15" s="151" t="str">
         <x:v>T004</x:v>
       </x:c>
@@ -7011,7 +7011,7 @@
       <x:c r="N15" s="2"/>
       <x:c r="O15" s="2"/>
     </x:row>
-    <x:row r="16" ht="66" customHeight="1">
+    <x:row r="16" ht="60" customHeight="1">
       <x:c r="A16" s="151" t="str">
         <x:v>T005</x:v>
       </x:c>
@@ -7042,7 +7042,7 @@
       <x:c r="N16" s="2"/>
       <x:c r="O16" s="2"/>
     </x:row>
-    <x:row r="17" ht="66" customHeight="1">
+    <x:row r="17" ht="60" customHeight="1">
       <x:c r="A17" s="151" t="str">
         <x:v>T023</x:v>
       </x:c>
@@ -7073,7 +7073,7 @@
       <x:c r="N17" s="2"/>
       <x:c r="O17" s="2"/>
     </x:row>
-    <x:row r="18" ht="66" customHeight="1">
+    <x:row r="18" ht="60" customHeight="1">
       <x:c r="A18" s="151" t="str">
         <x:v>T010</x:v>
       </x:c>
@@ -7104,7 +7104,7 @@
       <x:c r="N18" s="2"/>
       <x:c r="O18" s="2"/>
     </x:row>
-    <x:row r="19" ht="66" customHeight="1">
+    <x:row r="19" ht="60" customHeight="1">
       <x:c r="A19" s="151" t="str">
         <x:v>T015</x:v>
       </x:c>
@@ -7135,7 +7135,7 @@
       <x:c r="N19" s="2"/>
       <x:c r="O19" s="2"/>
     </x:row>
-    <x:row r="20" ht="66" customHeight="1">
+    <x:row r="20" ht="60" customHeight="1">
       <x:c r="A20" s="151" t="str">
         <x:v>T006</x:v>
       </x:c>
@@ -7166,7 +7166,7 @@
       <x:c r="N20" s="2"/>
       <x:c r="O20" s="2"/>
     </x:row>
-    <x:row r="21" ht="66" customHeight="1">
+    <x:row r="21" ht="60" customHeight="1">
       <x:c r="A21" s="151" t="str">
         <x:v>T014</x:v>
       </x:c>
@@ -7197,7 +7197,7 @@
       <x:c r="N21" s="2"/>
       <x:c r="O21" s="2"/>
     </x:row>
-    <x:row r="22" ht="66" customHeight="1">
+    <x:row r="22" ht="60" customHeight="1">
       <x:c r="A22" s="151" t="str">
         <x:v>T030</x:v>
       </x:c>
@@ -7228,7 +7228,7 @@
       <x:c r="N22" s="2"/>
       <x:c r="O22" s="2"/>
     </x:row>
-    <x:row r="23" ht="66" customHeight="1">
+    <x:row r="23" ht="60" customHeight="1">
       <x:c r="A23" s="151" t="str">
         <x:v>T024</x:v>
       </x:c>
@@ -7257,7 +7257,7 @@
       <x:c r="N23" s="2"/>
       <x:c r="O23" s="2"/>
     </x:row>
-    <x:row r="24" ht="66" customHeight="1">
+    <x:row r="24" ht="60" customHeight="1">
       <x:c r="A24" s="151" t="str">
         <x:v>T011</x:v>
       </x:c>
@@ -7286,7 +7286,7 @@
       <x:c r="N24" s="2"/>
       <x:c r="O24" s="2"/>
     </x:row>
-    <x:row r="25" ht="66" customHeight="1">
+    <x:row r="25" ht="60" customHeight="1">
       <x:c r="A25" s="151" t="str">
         <x:v>T027</x:v>
       </x:c>
@@ -7317,7 +7317,7 @@
       <x:c r="N25" s="2"/>
       <x:c r="O25" s="2"/>
     </x:row>
-    <x:row r="26" ht="66" customHeight="1">
+    <x:row r="26" ht="60" customHeight="1">
       <x:c r="A26" s="151" t="str">
         <x:v>T007</x:v>
       </x:c>
@@ -7348,7 +7348,7 @@
       <x:c r="N26" s="2"/>
       <x:c r="O26" s="2"/>
     </x:row>
-    <x:row r="27" ht="66" customHeight="1">
+    <x:row r="27" ht="60" customHeight="1">
       <x:c r="A27" s="151" t="str">
         <x:v>T017</x:v>
       </x:c>
@@ -7379,7 +7379,7 @@
       <x:c r="N27" s="2"/>
       <x:c r="O27" s="2"/>
     </x:row>
-    <x:row r="28" ht="66" customHeight="1">
+    <x:row r="28" ht="60" customHeight="1">
       <x:c r="A28" s="151" t="str">
         <x:v>T008</x:v>
       </x:c>
@@ -7410,7 +7410,7 @@
       <x:c r="N28" s="2"/>
       <x:c r="O28" s="2"/>
     </x:row>
-    <x:row r="29" ht="66" customHeight="1">
+    <x:row r="29" ht="60" customHeight="1">
       <x:c r="A29" s="78" t="str">
         <x:v>T020</x:v>
       </x:c>
@@ -7439,7 +7439,7 @@
       <x:c r="N29" s="2"/>
       <x:c r="O29" s="2"/>
     </x:row>
-    <x:row r="30" ht="66" customHeight="1">
+    <x:row r="30" ht="60" customHeight="1">
       <x:c r="A30" s="102" t="str">
         <x:v>T016</x:v>
       </x:c>
@@ -7470,7 +7470,7 @@
       <x:c r="N30" s="2"/>
       <x:c r="O30" s="2"/>
     </x:row>
-    <x:row r="31" ht="66" customHeight="1">
+    <x:row r="31" ht="60" customHeight="1">
       <x:c r="A31" s="132" t="str">
         <x:v>T009</x:v>
       </x:c>
@@ -7501,14 +7501,28 @@
       <x:c r="N31" s="2"/>
       <x:c r="O31" s="2"/>
     </x:row>
-    <x:row r="32" ht="26" customHeight="1">
-      <x:c r="A32" s="102"/>
-      <x:c r="B32" s="103"/>
-      <x:c r="C32" s="103"/>
-      <x:c r="D32" s="104"/>
-      <x:c r="E32" s="80"/>
-      <x:c r="F32" s="80"/>
-      <x:c r="G32" s="80"/>
+    <x:row r="32" ht="60" customHeight="1">
+      <x:c r="A32" s="102" t="str">
+        <x:v>T031</x:v>
+      </x:c>
+      <x:c r="B32" s="123" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="C32" s="123" t="d">
+        <x:v>2026-09-29T00:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="D32" s="104" t="str">
+        <x:v>Mythic</x:v>
+      </x:c>
+      <x:c r="E32" s="80" t="str">
+        <x:v>在班加罗尔设立CoE并扩展Vanguard研发团队</x:v>
+      </x:c>
+      <x:c r="F32" s="80" t="str">
+        <x:v>公司称团队已参与模拟核心前端、混合物理设计和车规DFT，当前岗位覆盖RTL、数字数据流验证、物理设计与DFT；证明研发组织扩张，不证明Vanguard投片、样片、Lockheed战术边缘部署或客户交付</x:v>
+      </x:c>
+      <x:c r="G32" s="80" t="str">
+        <x:v>https://www.mythic.ai/newsroom/mythic-bengaluru-centre-of-excellence</x:v>
+      </x:c>
       <x:c r="H32" s="67"/>
       <x:c r="I32" s="68"/>
       <x:c r="J32" s="2"/>
@@ -8221,8 +8235,8 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="2">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4921207f21dc4a2d"/>
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfc7aa281e3a4397"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfd5e29b4da94075"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93014f2f7a44ce1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>